<commit_message>
Update NPI Dashboard 2026-06-17 09:13
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Prestige N16 Flip AI+</t>
+          <t>Prestige N16 Spark</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Prestige N16 AI+</t>
+          <t>Prestige N16 Flip Spark</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Update NPI Dashboard 2026-06-18 13:35
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -148,10 +148,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -901,13 +901,12 @@
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
-          <t>MLG(魔龍姬)ID，因盤點,排6/15 CR工單重工及測試，6/19入庫</t>
+          <t>MLG(魔龍姬)ID，CR工單已重工完成待入庫</t>
         </is>
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>1)Schedule：因A/B件及rear cover有發黃issue，ID確認重新更換噴漆廠商，MP時間受影響由6/9 delay至6/19
-2)備料: A/B件及rear cover重新備料，6/11首批交料500pcs，至6/30陸續可齊套交料共3.8K，與6月份出貨6.2K有2.4K gap</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -1124,8 +1123,7 @@
       <c r="P8" s="6" t="inlineStr">
         <is>
           <t>1) 認證：SRRC認證中, 影響中國區出貨（可清關出貨，但上架售賣有風險）需在7/8前完成；
-2) Packing: WW版本設計確認中;
-3)Schedule: ID更換噴漆廠商,導致機構件缺料，ATS 由6/26更新為7/1，MP@7/8</t>
+2) Packing: WW版本設計確認中;</t>
         </is>
       </c>
     </row>
@@ -1495,12 +1493,12 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>24VL</t>
+          <t>26VL</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Modern A14 LE J1M</t>
+          <t>Modern A16 LE J1M</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
@@ -1556,15 +1554,14 @@
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
-          <t>MVT測試中，DQA 測試Issue 需微步協助盡快釐清&amp;導入對策，滿足ATS 6/E上線排程</t>
+          <t>MVT測試中，DQA 測試Issue 需微步協助盡快釐清&amp;導入對策,</t>
         </is>
       </c>
       <c r="P14" s="6" t="inlineStr">
         <is>
-          <t>1)物料： adapter：目標6K， 2.8K ETA @ 6/15,其它7/B 陸續進料 B&amp;S物料：6/9 釋放PO給微步，需要微步6/12協助下單備料，目前規劃ATS 6/20 SMT，物料需在6/18前寄送到微步
-2)認證   a)CE：預計6/12認證ready  b)CB：24VL 6/2通知啟動認證，預計6/E ready  C)TUV 認證预计7/E  d)其他地區認證follow In house 流程，有訂單需求後由業務通知申請 e) 24VL/26VL只有TH&amp;SG下單， Total 2072 Pcs：26VL:1.8K TH+80Pcs SG &amp; 24VL: 192Pcs SG  ,SG 無需認證，TH 已通知業務安排申請認證流程（待業務回復）
-3)TYPEC+USB4接口 SI测试Fail，需主板升级，6/8已安排SMT驗證，需微步加快SI驗證，已協調微步6/13到昆山更換PCBA，
-4）MVT Issue 微步Debug 進度緩慢，需微步協調人力加速釐清Issue及導入對策，deadline 6/19</t>
+          <t>1)物料： adapter：目標6K， 已到料2.8K ,其它7/B 陸續進料 B&amp;S物料： 6/18已寄送微步 ，預計6/22到料，
+2)認證 a))TUV 認證预计7/E b)其他地區認證follow In house 流程，有訂單需求後由業務通知申請 c) 24VL/26VL只有TH&amp;SG下單， Total 2072 Pcs：26VL:1.8K TH+80Pcs SG &amp; 24VL: 192Pcs SG ,SG 無需認證，TH 已通知業務安排申請認證流程（待業務回復）
+3）MVT Issue 微步Debug 進度緩慢，需微步協調人力加速釐清Issue及導入對策，目前TTM時間預計從7/8 延後到7/10</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1571,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>26VL</t>
+          <t>24VL</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Modern A16 LE J1M</t>
+          <t>Modern A14 LE J1M</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -1625,25 +1622,24 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026/06/25</t>
+          <t>2026/07/01</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>2026/07/08</t>
+          <t>2026/07/10</t>
         </is>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>MVT測試中，DQA 測試Issue 需微步協助盡快釐清&amp;導入對策,滿足ATS 6/E 規劃</t>
+          <t>MVT測試中，DQA 測試Issue 需微步協助盡快釐清&amp;導入對策，</t>
         </is>
       </c>
       <c r="P15" s="6" t="inlineStr">
         <is>
-          <t>1)物料： adapter：目標6K， 2.8K ETA @ 6/15,其它7/B 陸續進料 B&amp;S物料：6/9 釋放PO給微步，需要微步6/12協助下單備料，目前規劃ATS 6/20 SMT，物料需在6/18前寄送到微步
-2)認證   a)CE：預計6/12認證ready  b)CB：24VL 6/2通知啟動認證，預計6/E ready  C)TUV 認證预计7/E  d)其他地區認證follow In house 流程，有訂單需求後由業務通知申請 e) 24VL/26VL只有TH&amp;SG下單， Total 2072 Pcs：26VL:1.8K TH+80Pcs SG &amp; 24VL: 192Pcs SG  ,SG 無需認證，TH 已通知業務安排申請認證流程（待業務回復）
-3)TYPEC+USB4接口 SI测试Fail，需主板升级，6/8已安排SMT驗證，需微步加快SI驗證，已協調微步6/13到昆山更換PCBA，
-4）MVT Issue 微步Debug 進度緩慢，需微步協調人力加速釐清Issue及導入對策，deadline 6/19</t>
+          <t>1)物料： adapter：目標6K， 已到料2.8K ,其它7/B 陸續進料 B&amp;S物料： 6/18已寄送微步 ，預計6/22到料，
+2)認證 a))TUV 認證预计7/E b)其他地區認證follow In house 流程，有訂單需求後由業務通知申請 c) 24VL/26VL只有TH&amp;SG下單， Total 2072 Pcs：26VL:1.8K TH+80Pcs SG &amp; 24VL: 192Pcs SG ,SG 無需認證，TH 已通知業務安排申請認證流程（待業務回復）
+3）MVT Issue 微步Debug 進度緩慢，需微步協調人力加速釐清Issue及導入對策，目前TTM時間預計從7/8 延後到7/10</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1887,7 @@
       </c>
       <c r="P18" s="6" t="inlineStr">
         <is>
-          <t>1) 台北RD已取得主板,需麻煩各RD加速相關驗證</t>
+          <t>1) 10 gerberout@6/25,需麻煩各RD加速相關驗證</t>
         </is>
       </c>
     </row>
@@ -2544,13 +2540,13 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>2026/06/21</t>
+          <t>2026/06/29</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr"/>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>2026/07/21</t>
+          <t>2026/07/29</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
@@ -2560,7 +2556,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>2026/08/09</t>
+          <t>2026/08/17</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -2570,12 +2566,12 @@
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
-          <t>新料備料中, Weibu plan 6/21 DVT SMT</t>
+          <t>Weibu plan 6/29 DVT SMT, 7/1 ASSY--熱管&amp;D件重新開模, 交期7/1</t>
         </is>
       </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>1)備料for 6/21: a. 熱管6/29交期還在pull in b. D件開模, 交期還在確認中
+          <t>1)Schedule: 考量新料備料時程, 調整試產和ATS時間@8/17 start
 2)認證: 參考Weibu認證Schedule, 有四個國家無法同步於8/E TTM, 持續追蹤中 MX: 11/28 ready；AR:10/3 ready；CO: 9/5 ready；RU: 9/12 ready</t>
         </is>
       </c>
@@ -2621,13 +2617,13 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>2026/06/21</t>
+          <t>2026/06/29</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr"/>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>2026/07/21</t>
+          <t>2026/07/29</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
@@ -2637,7 +2633,7 @@
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>2026/08/09</t>
+          <t>2026/08/17</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr">
@@ -2647,12 +2643,12 @@
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
-          <t>新料備料中, Weibu plan 6/21 DVT SMT</t>
+          <t>Weibu plan 6/29 DVT SMT, 7/1 ASSY --熱管重新開模, 交期6/30</t>
         </is>
       </c>
       <c r="P28" s="6" t="inlineStr">
         <is>
-          <t>1)備料for 6/21: a. 熱管6/29交期還在pull in b. D件開模, 交期還在確認中
+          <t>1)Schedule: 考量新料備料時程, 調整試產和ATS時間@8/17 start
 2)認證: 參考Weibu認證Schedule, 有四個國家無法同步於8/E TTM, 持續追蹤中 MX: 11/28 ready；AR:10/3 ready；CO: 9/5 ready；RU: 9/12 ready</t>
         </is>
       </c>
@@ -2663,151 +2659,143 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>14T3</t>
+          <t>15TK</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Prestige N14 Spark D1M</t>
-        </is>
-      </c>
-      <c r="D29" s="17" t="inlineStr">
-        <is>
-          <t>EVT</t>
+          <t>Cyborg A15 Max C1PWE</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>Design</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>N1 35W</t>
+          <t>HWK 45W</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>倪嬌嬌</t>
+          <t>蔡東宏</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>2025/04/30</t>
+          <t>2026/05/28</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>2025/09/01</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>2026/04/15</t>
-        </is>
-      </c>
+          <t>2026/07/03</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr"/>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>2026/07/20</t>
+          <t>2026/08/06</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/17</t>
         </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
         <is>
-          <t>2026/09/01</t>
+          <t>2026/09/07</t>
         </is>
       </c>
       <c r="N29" s="4" t="inlineStr">
         <is>
-          <t>2026/09/14</t>
+          <t>2026/09/17</t>
         </is>
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
-          <t>EVT DQA更新BSP6.1.2 驗證中,  0C gerber out@6/17</t>
-        </is>
-      </c>
-      <c r="P29" s="6" t="inlineStr">
-        <is>
-          <t>1) 備料： 2.8K panel的驗證 follow leading customer, 交料plan:a. 1st MP lot: 2K 數量, 型號HQ15, 九月份交料(同步Leading customers量產交料時間 具體九月份ETD日期還在追蹤中. b. Others order: 需轉型號至HQxx, 十一月份交料</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
+          <t>AMD預計ww25寄出R9 180/R7 165, RD會先進行重工做開機驗證</t>
+        </is>
+      </c>
+      <c r="P29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30" hidden="1" outlineLevel="1">
+      <c r="A30" s="7" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>15TK</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Cyborg A15 Max C1PWE</t>
-        </is>
-      </c>
-      <c r="D30" s="16" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Cyborg A15 Max C1PWF</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>HWK 45W</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5050</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5060</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
         <is>
           <t>蔡東宏</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="H30" s="9" t="inlineStr">
         <is>
           <t>2026/05/28</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I30" s="9" t="inlineStr">
         <is>
           <t>2026/07/03</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr"/>
-      <c r="K30" s="4" t="inlineStr">
+      <c r="J30" s="9" t="inlineStr"/>
+      <c r="K30" s="9" t="inlineStr">
         <is>
           <t>2026/08/06</t>
         </is>
       </c>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="L30" s="9" t="inlineStr">
         <is>
           <t>2026/08/17</t>
         </is>
       </c>
-      <c r="M30" s="4" t="inlineStr">
+      <c r="M30" s="9" t="inlineStr">
         <is>
           <t>2026/09/07</t>
         </is>
       </c>
-      <c r="N30" s="4" t="inlineStr">
+      <c r="N30" s="9" t="inlineStr">
         <is>
           <t>2026/09/17</t>
         </is>
       </c>
-      <c r="O30" s="6" t="inlineStr">
+      <c r="O30" s="11" t="inlineStr">
         <is>
           <t>AMD預計ww25寄出R9 180/R7 165, RD會先進行重工做開機驗證</t>
         </is>
       </c>
-      <c r="P30" s="6" t="inlineStr"/>
+      <c r="P30" s="11" t="inlineStr"/>
     </row>
     <row r="31" hidden="1" outlineLevel="1">
       <c r="A31" s="7" t="n">
@@ -2820,10 +2808,10 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1PWF</t>
-        </is>
-      </c>
-      <c r="D31" s="18" t="inlineStr">
+          <t>Cyborg A15 Max C1PWG</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -2835,7 +2823,7 @@
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
@@ -2892,10 +2880,10 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1PWG</t>
-        </is>
-      </c>
-      <c r="D32" s="18" t="inlineStr">
+          <t>Cyborg A15 C1PWE</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -2907,7 +2895,7 @@
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
@@ -2922,108 +2910,117 @@
       </c>
       <c r="I32" s="9" t="inlineStr">
         <is>
-          <t>2026/07/03</t>
+          <t>2026/07/17</t>
         </is>
       </c>
       <c r="J32" s="9" t="inlineStr"/>
       <c r="K32" s="9" t="inlineStr">
         <is>
-          <t>2026/08/06</t>
+          <t>2026/08/19</t>
         </is>
       </c>
       <c r="L32" s="9" t="inlineStr">
         <is>
-          <t>2026/08/17</t>
+          <t>2026/08/27</t>
         </is>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>2026/09/07</t>
+          <t>2026/09/19</t>
         </is>
       </c>
       <c r="N32" s="9" t="inlineStr">
         <is>
-          <t>2026/09/17</t>
+          <t>2026/09/29</t>
         </is>
       </c>
       <c r="O32" s="11" t="inlineStr">
         <is>
-          <t>AMD預計ww25寄出R9 180/R7 165, RD會先進行重工做開機驗證</t>
+          <t>AMD預計ww27寄出R7 155/ R5 125, RD會先進行重工做開機驗證</t>
         </is>
       </c>
       <c r="P32" s="11" t="inlineStr"/>
     </row>
-    <row r="33" hidden="1" outlineLevel="1">
-      <c r="A33" s="7" t="n">
+    <row r="33">
+      <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>15TK</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>Cyborg A15 C1PWE</t>
-        </is>
-      </c>
-      <c r="D33" s="18" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E33" s="9" t="inlineStr">
-        <is>
-          <t>HWK 45W</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5050</t>
-        </is>
-      </c>
-      <c r="G33" s="9" t="inlineStr">
-        <is>
-          <t>蔡東宏</t>
-        </is>
-      </c>
-      <c r="H33" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/28</t>
-        </is>
-      </c>
-      <c r="I33" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/17</t>
-        </is>
-      </c>
-      <c r="J33" s="9" t="inlineStr"/>
-      <c r="K33" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/19</t>
-        </is>
-      </c>
-      <c r="L33" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/27</t>
-        </is>
-      </c>
-      <c r="M33" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/19</t>
-        </is>
-      </c>
-      <c r="N33" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/29</t>
-        </is>
-      </c>
-      <c r="O33" s="11" t="inlineStr">
-        <is>
-          <t>AMD預計ww27寄出R7 155/ R5 125, RD會先進行重工做開機驗證</t>
-        </is>
-      </c>
-      <c r="P33" s="11" t="inlineStr"/>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>14T3</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Prestige N14 Spark D1M</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>N1 35W</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>倪嬌嬌</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>2025/04/30</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>2025/09/01</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>2026/04/15</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/20</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/14</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/13</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/26</t>
+        </is>
+      </c>
+      <c r="O33" s="6" t="inlineStr">
+        <is>
+          <t>MVT SMT@7/20--depend on 0C PCB ETA</t>
+        </is>
+      </c>
+      <c r="P33" s="6" t="inlineStr">
+        <is>
+          <t>1) Schedule: NV update BSP時間Factory drop final ETA@10/6, 更新ATS start@10/13
+2)備料： 2.8K panel的驗證 follow leading customer, 交料plan:a. 1st MP lot: 1K 數量, 型號HQ15, 九月份交料(同步Leading customers量產交料時間 具體九月份ETD日期還在追蹤中. b. Others order: 需轉型號至HQxx, 十一月份交料</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -3039,7 +3036,7 @@
           <t>Prestige N16 Spark C1M</t>
         </is>
       </c>
-      <c r="D34" s="17" t="inlineStr">
+      <c r="D34" s="18" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -3177,7 +3174,7 @@
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: NV approved @ 6/11, DVT SMT @ 6/18</t>
+          <t>RPL-HX R + DDR5: DVT SMT @ 6/18 VBIOS先用2653的替用，待1861申請到後請HW重刷測試</t>
         </is>
       </c>
       <c r="P35" s="6" t="inlineStr">
@@ -3257,7 +3254,7 @@
       </c>
       <c r="O36" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: NV approved @ 6/11, DVT SMT @ 6/18</t>
+          <t>RPL-HX R + DDR5: DVT SMT @ 6/18 VBIOS先用2653的替用，待1861申請到後請HW重刷測試</t>
         </is>
       </c>
       <c r="P36" s="11" t="inlineStr">
@@ -3337,7 +3334,7 @@
       </c>
       <c r="O37" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: NV approved @ 6/11, DVT SMT @ 6/18</t>
+          <t>RPL-HX R + DDR5: DVT SMT @ 6/18 VBIOS先用2653的替用，待1861申請到後請HW重刷測試</t>
         </is>
       </c>
       <c r="P37" s="11" t="inlineStr">
@@ -3413,7 +3410,7 @@
       </c>
       <c r="O38" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: 3.0 G/O @ 6/12, 預計DVT SMT @ 6/27</t>
+          <t>RPL-HX R + DDR4: 預計DVT SMT @ 6/29</t>
         </is>
       </c>
       <c r="P38" s="11" t="inlineStr">
@@ -3489,7 +3486,7 @@
       </c>
       <c r="O39" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: 3.0 G/O @ 6/12, 預計DVT SMT @ 6/27</t>
+          <t>RPL-HX R + DDR4: 預計DVT SMT @ 6/29</t>
         </is>
       </c>
       <c r="P39" s="11" t="inlineStr">
@@ -3565,7 +3562,7 @@
       </c>
       <c r="O40" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: 3.0 G/O @ 6/12, 預計DVT SMT @ 6/27</t>
+          <t>RPL-HX R + DDR4: 預計DVT SMT @ 6/29</t>
         </is>
       </c>
       <c r="P40" s="11" t="inlineStr">
@@ -3645,7 +3642,7 @@
       </c>
       <c r="O41" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: NV approved @ 6/11, DVT SMT @ 6/18</t>
+          <t>RPL-HX R + DDR5: DVT SMT @ 6/18 VBIOS先用2653的替用，待1861申請到後請HW重刷測試</t>
         </is>
       </c>
       <c r="P41" s="11" t="inlineStr">
@@ -3721,7 +3718,7 @@
       </c>
       <c r="O42" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: 3.0 G/O @ 6/12, 預計DVT SMT @ 6/27</t>
+          <t>RPL-HX R + DDR4: 預計DVT SMT @ 6/29</t>
         </is>
       </c>
       <c r="P42" s="11" t="inlineStr">
@@ -3801,7 +3798,7 @@
       </c>
       <c r="O43" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: NV approved @ 6/11, DVT SMT @ 6/18</t>
+          <t>RPL-HX R + DDR5: DVT SMT @ 6/18 VBIOS先用2653的替用，待1861申請到後請HW重刷測試</t>
         </is>
       </c>
       <c r="P43" s="11" t="inlineStr">
@@ -3877,7 +3874,7 @@
       </c>
       <c r="O44" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: 3.0 G/O @ 6/12, 預計DVT SMT @ 6/27</t>
+          <t>RPL-HX R + DDR4: 預計DVT SMT @ 6/29</t>
         </is>
       </c>
       <c r="P44" s="11" t="inlineStr">
@@ -3957,7 +3954,7 @@
       </c>
       <c r="O45" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: NV approved @ 6/11, DVT SMT @ 6/18</t>
+          <t>RPL-HX R + DDR5: DVT SMT @ 6/18 VBIOS先用2653的替用，待1861申請到後請HW重刷測試</t>
         </is>
       </c>
       <c r="P45" s="11" t="inlineStr">
@@ -4033,7 +4030,7 @@
       </c>
       <c r="O46" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: 3.0 G/O @ 6/12, 預計DVT SMT @ 6/27</t>
+          <t>RPL-HX R + DDR4: 預計DVT SMT @ 6/29</t>
         </is>
       </c>
       <c r="P46" s="11" t="inlineStr">
@@ -4113,7 +4110,7 @@
       </c>
       <c r="O47" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: NV approved @ 6/11, DVT SMT @ 6/18</t>
+          <t>RPL-HX R + DDR5: DVT SMT @ 6/18 VBIOS先用2653的替用，待1861申請到後請HW重刷測試</t>
         </is>
       </c>
       <c r="P47" s="11" t="inlineStr">
@@ -4189,7 +4186,7 @@
       </c>
       <c r="O48" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: 3.0 G/O @ 6/12, 預計DVT SMT @ 6/27</t>
+          <t>RPL-HX R + DDR4: 預計DVT SMT @ 6/29</t>
         </is>
       </c>
       <c r="P48" s="11" t="inlineStr">
@@ -4212,7 +4209,7 @@
           <t>Crosshair 18 Max HX B2WE</t>
         </is>
       </c>
-      <c r="D49" s="18" t="inlineStr">
+      <c r="D49" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4284,7 +4281,7 @@
           <t>Crosshair 18 Max HX B2WEO</t>
         </is>
       </c>
-      <c r="D50" s="18" t="inlineStr">
+      <c r="D50" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4356,7 +4353,7 @@
           <t>Crosshair 18 Max HX B2WF</t>
         </is>
       </c>
-      <c r="D51" s="18" t="inlineStr">
+      <c r="D51" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4428,7 +4425,7 @@
           <t>Crosshair 18 Max HX B2WFO</t>
         </is>
       </c>
-      <c r="D52" s="18" t="inlineStr">
+      <c r="D52" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4500,7 +4497,7 @@
           <t>Crosshair 18 Max HX B2WG</t>
         </is>
       </c>
-      <c r="D53" s="18" t="inlineStr">
+      <c r="D53" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4572,7 +4569,7 @@
           <t>Crosshair 18 Max HX B2WGO</t>
         </is>
       </c>
-      <c r="D54" s="18" t="inlineStr">
+      <c r="D54" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4644,7 +4641,7 @@
           <t>Crosshair 18 Max HX B2WGX</t>
         </is>
       </c>
-      <c r="D55" s="18" t="inlineStr">
+      <c r="D55" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4716,7 +4713,7 @@
           <t>Crosshair 18 Max HX B2WGXO</t>
         </is>
       </c>
-      <c r="D56" s="18" t="inlineStr">
+      <c r="D56" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4788,7 +4785,7 @@
           <t>Katana 18 HX A2WEK</t>
         </is>
       </c>
-      <c r="D57" s="18" t="inlineStr">
+      <c r="D57" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4860,7 +4857,7 @@
           <t>Katana 18 HX A2WEOK</t>
         </is>
       </c>
-      <c r="D58" s="18" t="inlineStr">
+      <c r="D58" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4936,7 +4933,7 @@
           <t>Katana 18 HX A2WFK</t>
         </is>
       </c>
-      <c r="D59" s="18" t="inlineStr">
+      <c r="D59" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5008,7 +5005,7 @@
           <t>Katana 18 HX A2WFOK</t>
         </is>
       </c>
-      <c r="D60" s="18" t="inlineStr">
+      <c r="D60" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5084,7 +5081,7 @@
           <t>Katana 18 HX A2WGK</t>
         </is>
       </c>
-      <c r="D61" s="18" t="inlineStr">
+      <c r="D61" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5156,7 +5153,7 @@
           <t>Katana 18 HX A2WGOK</t>
         </is>
       </c>
-      <c r="D62" s="18" t="inlineStr">
+      <c r="D62" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5312,7 +5309,7 @@
           <t>Prestige 14 AI+ Flip</t>
         </is>
       </c>
-      <c r="D64" s="18" t="inlineStr">
+      <c r="D64" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5468,7 +5465,7 @@
           <t>Prestige 16 Flip AI+</t>
         </is>
       </c>
-      <c r="D66" s="18" t="inlineStr">
+      <c r="D66" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5624,7 +5621,7 @@
           <t>Stealth 16 AI+ B4WH</t>
         </is>
       </c>
-      <c r="D68" s="18" t="inlineStr">
+      <c r="D68" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5704,7 +5701,7 @@
           <t>Stealth 16 AI+ B4WJ</t>
         </is>
       </c>
-      <c r="D69" s="18" t="inlineStr">
+      <c r="D69" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5865,7 +5862,7 @@
           <t>Stealth 16 AI+ B4WF</t>
         </is>
       </c>
-      <c r="D71" s="18" t="inlineStr">
+      <c r="D71" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5946,7 +5943,7 @@
           <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
         </is>
       </c>
-      <c r="D72" s="18" t="inlineStr">
+      <c r="D72" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6027,7 +6024,7 @@
           <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
         </is>
       </c>
-      <c r="D73" s="18" t="inlineStr">
+      <c r="D73" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6188,7 +6185,7 @@
           <t>Raider 16 Max HX B4WI</t>
         </is>
       </c>
-      <c r="D75" s="18" t="inlineStr">
+      <c r="D75" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6268,7 +6265,7 @@
           <t>Raider 16 Max HX B4WJ</t>
         </is>
       </c>
-      <c r="D76" s="18" t="inlineStr">
+      <c r="D76" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6348,7 +6345,7 @@
           <t>Raider 16  HX B4WH</t>
         </is>
       </c>
-      <c r="D77" s="18" t="inlineStr">
+      <c r="D77" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6428,7 +6425,7 @@
           <t>Raider 16  HX B4WI</t>
         </is>
       </c>
-      <c r="D78" s="18" t="inlineStr">
+      <c r="D78" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6588,7 +6585,7 @@
           <t>Crosshair 16 Max HX E4WFK</t>
         </is>
       </c>
-      <c r="D80" s="18" t="inlineStr">
+      <c r="D80" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6668,7 +6665,7 @@
           <t>Crosshair 16 Max HX E4WGK</t>
         </is>
       </c>
-      <c r="D81" s="18" t="inlineStr">
+      <c r="D81" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6748,7 +6745,7 @@
           <t>Crosshair 16 Max HX E4WGXK</t>
         </is>
       </c>
-      <c r="D82" s="18" t="inlineStr">
+      <c r="D82" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>

</xml_diff>

<commit_message>
Update NPI Dashboard 2026-06-26 16:46
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPI Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -519,7 +519,7 @@
     <outlinePr summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P82"/>
+  <dimension ref="A1:P83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -628,12 +628,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>14V2</t>
+          <t>14T2</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Commercial 14 C13M</t>
+          <t>Prestige 14 Flip AI+ Rhône</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -643,54 +643,54 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>RPL-U 25W</t>
+          <t>PTL-H 30W</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Intel® graphics</t>
+          <t>Intel® Arc™ Graphics</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>杜晨光</t>
+          <t>朱芳芳</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>2026/01/04</t>
+          <t>2026/04/13</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr"/>
       <c r="J2" s="4" t="inlineStr"/>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>2026/02/05</t>
+          <t>2026/05/10</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>2026/03/16</t>
+          <t>2026/05/19</t>
         </is>
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026/05/15</t>
+          <t>2026/06/23</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>2026/05/30</t>
+          <t>2026/06/30</t>
         </is>
       </c>
       <c r="O2" s="6" t="inlineStr">
         <is>
-          <t>因PCB 最快交期落在6/29,加上微步盤點，預計最快7/10 TTM</t>
+          <t>梵谷特仕版 物料持續追踪，6/23 ATS CR，6/E出貨</t>
         </is>
       </c>
       <c r="P2" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1. ALS sensor NG  HDI 進版 6/27重工， 1.A件成品LOGO不良較高，交料瓶頸 請ID&amp;Buyer持續pull in。</t>
         </is>
       </c>
     </row>
@@ -700,12 +700,12 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>14V2</t>
+          <t>14T2</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>Modern 14 H13M</t>
+          <t>Prestige 14 Flip AI+ Starry Night</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
@@ -715,54 +715,54 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>RPL-U 25W</t>
+          <t>PTL-H 30W</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Intel® graphics</t>
+          <t>Intel® Arc™ Graphics</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>杜晨光</t>
+          <t>朱芳芳</t>
         </is>
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>2025/11/14</t>
+          <t>2026/04/13</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr"/>
       <c r="J3" s="9" t="inlineStr"/>
       <c r="K3" s="9" t="inlineStr">
         <is>
-          <t>2026/01/14</t>
+          <t>2026/05/10</t>
         </is>
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t>2026/03/16</t>
+          <t>2026/05/19</t>
         </is>
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>2026/05/15</t>
+          <t>2026/06/23</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
         <is>
-          <t>2026/05/30</t>
+          <t>2026/06/30</t>
         </is>
       </c>
       <c r="O3" s="11" t="inlineStr">
         <is>
-          <t>因PCB 最快交期落在6/29,加上微步盤點，預計最快7/10 TTM</t>
+          <t>梵谷特仕版 物料持續追踪，規劃6/23 ATS CR，6/E出貨</t>
         </is>
       </c>
       <c r="P3" s="11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1. ALS sensor NG  HDI 進版 6/27重工， 2.A件成品LOGO不良較高，交料瓶頸 請ID&amp;Buyer持續pull in。</t>
         </is>
       </c>
     </row>
@@ -772,69 +772,71 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>14T2</t>
+          <t>265L</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Prestige 14 Flip AI+ Rhône</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>ATS</t>
+          <t>Crosshair A16 HX MLG Edition E8WFK</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>PTL-H 30W</t>
+          <t>DRG-HX 55W</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Intel® Arc™ Graphics</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>朱芳芳</t>
+          <t>朱欣怡</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>2026/04/13</t>
+          <t>2026/05/08</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr"/>
       <c r="J4" s="4" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>2026/05/10</t>
+          <t>2026/06/02</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>2026/05/19</t>
+          <t>2026/05/26</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>2026/06/23</t>
+          <t>2026/07/03</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>2026/06/30</t>
+          <t>2026/07/10</t>
         </is>
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
-          <t>梵谷特仕版 物料持續追踪，6/23 ATS CR，6/E出貨</t>
+          <t>MLG(魔龍姬)ID: DQA 測試中</t>
         </is>
       </c>
       <c r="P4" s="6" t="inlineStr">
         <is>
-          <t>1. ALS sensor NG  HDI 進版 6/27重工， 1.A件成品LOGO不良較高，交料瓶頸 請ID&amp;Buyer持續pull in。</t>
+          <t>1) 認證：SRRC認證中, 影響中國區出貨（可清關出貨，但上架售賣有風險）需在7/8前完成；
+2) Packing: WW版本設計確認中;
+3) Schedule: 生管排程, ATS 由7/1更新為7/3. MP @7/10</t>
         </is>
       </c>
     </row>
@@ -844,143 +846,141 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>14T2</t>
+          <t>265L</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Prestige 14 Flip AI+ Starry Night</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>ATS</t>
+          <t>Crosshair A16 HX MLG Edition E8WEK</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>PTL-H 30W</t>
+          <t>DRG-HX 55W</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>Intel® Arc™ Graphics</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>朱芳芳</t>
+          <t>朱欣怡</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>2026/04/13</t>
+          <t>2026/05/08</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr"/>
       <c r="J5" s="9" t="inlineStr"/>
       <c r="K5" s="9" t="inlineStr">
         <is>
-          <t>2026/05/10</t>
+          <t>2026/06/02</t>
         </is>
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>2026/05/19</t>
+          <t>2026/05/26</t>
         </is>
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>2026/06/23</t>
+          <t>2026/07/03</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>2026/06/30</t>
+          <t>2026/07/10</t>
         </is>
       </c>
       <c r="O5" s="11" t="inlineStr">
         <is>
-          <t>梵谷特仕版 物料持續追踪，規劃6/23 ATS CR，6/E出貨</t>
+          <t>MLG(魔龍姬)ID: DQA 測試中</t>
         </is>
       </c>
       <c r="P5" s="11" t="inlineStr">
         <is>
-          <t>1. ALS sensor NG  HDI 進版 6/27重工， 2.A件成品LOGO不良較高，交料瓶頸 請ID&amp;Buyer持續pull in。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" hidden="1" outlineLevel="1">
+      <c r="A6" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>265L</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Crosshair A16 HX MLG Edition E8WFK</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Crosshair A16 HX MLG Edition E8WGK</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>MVT</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>DRG-HX 55W</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5060</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>朱欣怡</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>2026/05/08</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr"/>
+      <c r="J6" s="9" t="inlineStr"/>
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>2026/06/02</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>2026/05/26</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="M6" s="9" t="inlineStr">
         <is>
           <t>2026/07/03</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="N6" s="9" t="inlineStr">
         <is>
           <t>2026/07/10</t>
         </is>
       </c>
-      <c r="O6" s="6" t="inlineStr">
-        <is>
-          <t>MLG(魔龍姬)ID: DQA 測試中</t>
-        </is>
-      </c>
-      <c r="P6" s="6" t="inlineStr">
-        <is>
-          <t>1) 認證：SRRC認證中, 影響中國區出貨（可清關出貨，但上架售賣有風險）需在7/8前完成；
-2) Packing: WW版本設計確認中;
-3) Schedule: 生管排程, ATS 由7/1更新為7/3. MP @7/10</t>
+      <c r="O6" s="11" t="inlineStr">
+        <is>
+          <t>MLG(魔龍姬)ID:  DQA 測試中</t>
+        </is>
+      </c>
+      <c r="P6" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Crosshair A16 HX MLG Edition E8WEK</t>
+          <t>Crosshair A16 HX MLG Edition E8WGXK</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="O7" s="11" t="inlineStr">
         <is>
-          <t>MLG(魔龍姬)ID: DQA 測試中</t>
+          <t>MLG(魔龍姬)ID:  DQA 測試中</t>
         </is>
       </c>
       <c r="P7" s="11" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Crosshair A16 HX MLG Edition E8WGK</t>
+          <t>Crosshair A16 HX E9WEK</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
@@ -1077,12 +1077,12 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>DRG-HX 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -1092,34 +1092,34 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
+          <t>2025/10/22</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr"/>
       <c r="J8" s="9" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>2026/06/02</t>
+          <t>2026/05/18</t>
         </is>
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>2026/05/26</t>
+          <t>2026/06/16</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>2026/07/03</t>
+          <t>2026/07/16</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>2026/07/10</t>
+          <t>2026/07/26</t>
         </is>
       </c>
       <c r="O8" s="11" t="inlineStr">
         <is>
-          <t>MLG(魔龍姬)ID:  DQA 測試中</t>
+          <t>FRG (5/4通知resume）: DQA 測試中</t>
         </is>
       </c>
       <c r="P8" s="11" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Crosshair A16 HX MLG Edition E8WGXK</t>
+          <t>Crosshair A16 HX E9WFK</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
@@ -1149,12 +1149,12 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>DRG-HX 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
@@ -1164,34 +1164,34 @@
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
+          <t>2025/10/22</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr"/>
       <c r="J9" s="9" t="inlineStr"/>
       <c r="K9" s="9" t="inlineStr">
         <is>
-          <t>2026/06/02</t>
+          <t>2026/05/18</t>
         </is>
       </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
-          <t>2026/05/26</t>
+          <t>2026/06/16</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>2026/07/03</t>
+          <t>2026/07/16</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
         <is>
-          <t>2026/07/10</t>
+          <t>2026/07/26</t>
         </is>
       </c>
       <c r="O9" s="11" t="inlineStr">
         <is>
-          <t>MLG(魔龍姬)ID:  DQA 測試中</t>
+          <t>FRG (5/4通知resume）: DQA 測試中</t>
         </is>
       </c>
       <c r="P9" s="11" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Crosshair A16 HX E9WEK</t>
+          <t>Crosshair A16 HX E9WGXK</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
@@ -1221,12 +1221,12 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>FRG-HX 55W</t>
+          <t>FRG-HX3D 55W</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -1272,75 +1272,75 @@
         </is>
       </c>
     </row>
-    <row r="11" hidden="1" outlineLevel="1">
-      <c r="A11" s="7" t="n">
+    <row r="11">
+      <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>265L</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Crosshair A16 HX E9WFK</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>MVT</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>FRG-HX 55W</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5060</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>朱欣怡</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>2025/10/22</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/18</t>
-        </is>
-      </c>
-      <c r="L11" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/16</t>
-        </is>
-      </c>
-      <c r="M11" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/16</t>
-        </is>
-      </c>
-      <c r="N11" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/26</t>
-        </is>
-      </c>
-      <c r="O11" s="11" t="inlineStr">
-        <is>
-          <t>FRG (5/4通知resume）: DQA 測試中</t>
-        </is>
-      </c>
-      <c r="P11" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>14V2</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Commercial 14 C13M</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>ATS</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>RPL-U 25W</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Intel® graphics</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>杜晨光</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>2026/01/04</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>2026/02/05</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>2026/03/16</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/06</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/10</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>因首批安排RPL-U Refresh 優先投產，第二波投產因PCB 最快交期落在6/29,加上微步盤點，預計最快7/10 TTM</t>
+        </is>
+      </c>
+      <c r="P11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1350,69 +1350,69 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>265L</t>
+          <t>14V2</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Crosshair A16 HX E9WGXK</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>MVT</t>
+          <t>Modern 14 H13M</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>ATS</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>RPL-U 25W</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>Intel® graphics</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>朱欣怡</t>
+          <t>杜晨光</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>2025/10/22</t>
+          <t>2025/11/14</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr"/>
       <c r="J12" s="9" t="inlineStr"/>
       <c r="K12" s="9" t="inlineStr">
         <is>
-          <t>2026/05/18</t>
+          <t>2026/01/14</t>
         </is>
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>2026/06/16</t>
+          <t>2026/03/16</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>2026/07/16</t>
+          <t>2026/07/06</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>2026/07/26</t>
+          <t>2026/07/10</t>
         </is>
       </c>
       <c r="O12" s="11" t="inlineStr">
         <is>
-          <t>FRG (5/4通知resume）: DQA 測試中</t>
+          <t>因首批安排RPL-U Refresh 優先投產，第二波投產因PCB 最快交期落在6/29,加上微步盤點，預計最快7/10 TTM</t>
         </is>
       </c>
       <c r="P12" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -2555,12 +2555,12 @@
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
-          <t>HPT sku:RD已重工3台成APU 180且刷16RK的BIOS可開機進OS,需AMD/AMI 儘速release PI code 1200i進行測試</t>
+          <t>HPT sku:RD已重工3台成APU 180,AMI release PI 1200i RC3@6/29,BIOS RD需儘速提供MSI版本BIOSi進行測試</t>
         </is>
       </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但PI code 1200i release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
+          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但AMD PI 1200i NDA release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
 2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS, 若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
         </is>
       </c>
@@ -2632,12 +2632,12 @@
       </c>
       <c r="O28" s="11" t="inlineStr">
         <is>
-          <t>HPT sku:RD已重工3台成APU 180且刷16RK的BIOS可開機進OS,需AMD/AMI 儘速release PI code 1200i進行測試</t>
+          <t>HPT sku:RD已重工3台成APU 180,AMI release PI 1200i RC3@6/29,BIOS RD需儘速提供MSI版本BIOSi進行測試</t>
         </is>
       </c>
       <c r="P28" s="11" t="inlineStr">
         <is>
-          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但PI code 1200i release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
+          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但AMD PI 1200i NDA release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
 2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS, 若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
         </is>
       </c>
@@ -2709,12 +2709,12 @@
       </c>
       <c r="O29" s="11" t="inlineStr">
         <is>
-          <t>HPT sku:RD已重工3台成APU 180且刷16RK的BIOS可開機進OS,需AMD/AMI 儘速release PI code 1200i進行測試</t>
+          <t>HPT sku:RD已重工3台成APU 180,AMI release PI 1200i RC3@6/29,BIOS RD需儘速提供MSI版本BIOSi進行測試</t>
         </is>
       </c>
       <c r="P29" s="11" t="inlineStr">
         <is>
-          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但PI code 1200i release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
+          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但AMD PI 1200i NDA release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
 2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS, 若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
         </is>
       </c>
@@ -2786,12 +2786,12 @@
       </c>
       <c r="O30" s="11" t="inlineStr">
         <is>
-          <t>HPT sku:RD已重工3台成APU 180且刷16RK的BIOS可開機進OS,需AMD/AMI 儘速release PI code 1200i進行測試</t>
+          <t>HPT sku:RD已重工3台成APU 180,AMI release PI 1200i RC3@6/29,BIOS RD需儘速提供MSI版本BIOSi進行測試</t>
         </is>
       </c>
       <c r="P30" s="11" t="inlineStr">
         <is>
-          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但PI code 1200i release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
+          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但AMD PI 1200i NDA release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
 2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS, 若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
         </is>
       </c>
@@ -5541,157 +5541,149 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
+          <t>13Q5</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Prestige 13 AI+ A4M</t>
+        </is>
+      </c>
+      <c r="D67" s="14" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>NVL-H 28W</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Intel® Arc™ Graphics</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>顏春梅</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>2026/06/29</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/18</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/08</t>
+        </is>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/21</t>
+        </is>
+      </c>
+      <c r="L67" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/22</t>
+        </is>
+      </c>
+      <c r="M67" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/22</t>
+        </is>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/31</t>
+        </is>
+      </c>
+      <c r="O67" s="6" t="inlineStr"/>
+      <c r="P67" s="6" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
           <t>2633</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>Stealth 16 AI+ B4WI</t>
         </is>
       </c>
-      <c r="D67" s="14" t="inlineStr">
+      <c r="D68" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E67" s="4" t="inlineStr">
+      <c r="E68" s="4" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F67" s="4" t="inlineStr">
+      <c r="F68" s="4" t="inlineStr">
         <is>
           <t>RTX 5080</t>
         </is>
       </c>
-      <c r="G67" s="4" t="inlineStr">
+      <c r="G68" s="4" t="inlineStr">
         <is>
           <t>朱欣怡</t>
         </is>
       </c>
-      <c r="H67" s="4" t="inlineStr">
+      <c r="H68" s="4" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I67" s="4" t="inlineStr">
+      <c r="I68" s="4" t="inlineStr">
         <is>
           <t>2026/07/22</t>
         </is>
       </c>
-      <c r="J67" s="4" t="inlineStr">
+      <c r="J68" s="4" t="inlineStr">
         <is>
           <t>2026/09/16</t>
         </is>
       </c>
-      <c r="K67" s="4" t="inlineStr">
+      <c r="K68" s="4" t="inlineStr">
         <is>
           <t>2026/11/11</t>
         </is>
       </c>
-      <c r="L67" s="4" t="inlineStr">
+      <c r="L68" s="4" t="inlineStr">
         <is>
           <t>2026/11/30</t>
         </is>
       </c>
-      <c r="M67" s="4" t="inlineStr">
+      <c r="M68" s="4" t="inlineStr">
         <is>
           <t>2026/12/29</t>
         </is>
       </c>
-      <c r="N67" s="4" t="inlineStr">
+      <c r="N68" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="O67" s="6" t="inlineStr">
+      <c r="O68" s="6" t="inlineStr">
         <is>
           <t>0M layout中，预计6/30 gerber out</t>
         </is>
       </c>
-      <c r="P67" s="6" t="inlineStr">
+      <c r="P68" s="6" t="inlineStr">
         <is>
           <t>1) Schedule:NV VBIOS @1/6, gating 8天,預計12/E 拿到WHQL，可能影響到最終TTM 時間</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" hidden="1" outlineLevel="1">
-      <c r="A68" s="7" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" s="8" t="inlineStr">
-        <is>
-          <t>2633</t>
-        </is>
-      </c>
-      <c r="C68" s="9" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WH</t>
-        </is>
-      </c>
-      <c r="D68" s="18" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E68" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 45W</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070Ti</t>
-        </is>
-      </c>
-      <c r="G68" s="9" t="inlineStr">
-        <is>
-          <t>朱欣怡</t>
-        </is>
-      </c>
-      <c r="H68" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/22</t>
-        </is>
-      </c>
-      <c r="I68" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/22</t>
-        </is>
-      </c>
-      <c r="J68" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/16</t>
-        </is>
-      </c>
-      <c r="K68" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/11</t>
-        </is>
-      </c>
-      <c r="L68" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/30</t>
-        </is>
-      </c>
-      <c r="M68" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/29</t>
-        </is>
-      </c>
-      <c r="N68" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="O68" s="11" t="inlineStr">
-        <is>
-          <t>0M layout中，预计6/30 gerber out</t>
-        </is>
-      </c>
-      <c r="P68" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
         </is>
       </c>
     </row>
@@ -5706,231 +5698,230 @@
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
+          <t>Stealth 16 AI+ B4WH</t>
+        </is>
+      </c>
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E69" s="9" t="inlineStr">
+        <is>
+          <t>NVL-H 45W</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070Ti</t>
+        </is>
+      </c>
+      <c r="G69" s="9" t="inlineStr">
+        <is>
+          <t>朱欣怡</t>
+        </is>
+      </c>
+      <c r="H69" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="I69" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/22</t>
+        </is>
+      </c>
+      <c r="J69" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/16</t>
+        </is>
+      </c>
+      <c r="K69" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/11</t>
+        </is>
+      </c>
+      <c r="L69" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/30</t>
+        </is>
+      </c>
+      <c r="M69" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/29</t>
+        </is>
+      </c>
+      <c r="N69" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="O69" s="11" t="inlineStr">
+        <is>
+          <t>0M layout中，预计6/30 gerber out</t>
+        </is>
+      </c>
+      <c r="P69" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" hidden="1" outlineLevel="1">
+      <c r="A70" s="7" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>2633</t>
+        </is>
+      </c>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
           <t>Stealth 16 AI+ B4WJ</t>
         </is>
       </c>
-      <c r="D69" s="18" t="inlineStr">
+      <c r="D70" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E69" s="9" t="inlineStr">
+      <c r="E70" s="9" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F69" s="9" t="inlineStr">
+      <c r="F70" s="9" t="inlineStr">
         <is>
           <t>RTX 5090</t>
         </is>
       </c>
-      <c r="G69" s="9" t="inlineStr">
+      <c r="G70" s="9" t="inlineStr">
         <is>
           <t>朱欣怡</t>
         </is>
       </c>
-      <c r="H69" s="9" t="inlineStr">
+      <c r="H70" s="9" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I69" s="9" t="inlineStr">
+      <c r="I70" s="9" t="inlineStr">
         <is>
           <t>2026/07/22</t>
         </is>
       </c>
-      <c r="J69" s="9" t="inlineStr">
+      <c r="J70" s="9" t="inlineStr">
         <is>
           <t>2026/09/16</t>
         </is>
       </c>
-      <c r="K69" s="9" t="inlineStr">
+      <c r="K70" s="9" t="inlineStr">
         <is>
           <t>2026/11/11</t>
         </is>
       </c>
-      <c r="L69" s="9" t="inlineStr">
+      <c r="L70" s="9" t="inlineStr">
         <is>
           <t>2026/11/30</t>
         </is>
       </c>
-      <c r="M69" s="9" t="inlineStr">
+      <c r="M70" s="9" t="inlineStr">
         <is>
           <t>2026/12/29</t>
         </is>
       </c>
-      <c r="N69" s="9" t="inlineStr">
+      <c r="N70" s="9" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="O69" s="11" t="inlineStr">
+      <c r="O70" s="11" t="inlineStr">
         <is>
           <t>0M layout中，预计6/30 gerber out</t>
         </is>
       </c>
-      <c r="P69" s="11" t="inlineStr">
+      <c r="P70" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>2634</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr">
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>Stealth 16 AI+ B4WE</t>
         </is>
       </c>
-      <c r="D70" s="14" t="inlineStr">
+      <c r="D71" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
+      <c r="E71" s="4" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F70" s="4" t="inlineStr">
+      <c r="F71" s="4" t="inlineStr">
         <is>
           <t>RTX 5050</t>
         </is>
       </c>
-      <c r="G70" s="4" t="inlineStr">
+      <c r="G71" s="4" t="inlineStr">
         <is>
           <t>賴雪鳳</t>
         </is>
       </c>
-      <c r="H70" s="4" t="inlineStr">
+      <c r="H71" s="4" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I70" s="4" t="inlineStr">
+      <c r="I71" s="4" t="inlineStr">
         <is>
           <t>2026/08/07</t>
         </is>
       </c>
-      <c r="J70" s="4" t="inlineStr">
+      <c r="J71" s="4" t="inlineStr">
         <is>
           <t>2026/09/16</t>
         </is>
       </c>
-      <c r="K70" s="4" t="inlineStr">
+      <c r="K71" s="4" t="inlineStr">
         <is>
           <t>2026/11/11</t>
         </is>
       </c>
-      <c r="L70" s="4" t="inlineStr">
+      <c r="L71" s="4" t="inlineStr">
         <is>
           <t>2026/11/27</t>
         </is>
       </c>
-      <c r="M70" s="4" t="inlineStr">
+      <c r="M71" s="4" t="inlineStr">
         <is>
           <t>2026/12/29</t>
         </is>
       </c>
-      <c r="N70" s="4" t="inlineStr">
+      <c r="N71" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="O70" s="6" t="inlineStr">
+      <c r="O71" s="6" t="inlineStr">
         <is>
           <t>0A layout start 6/8-7/17</t>
         </is>
       </c>
-      <c r="P70" s="6" t="inlineStr">
-        <is>
-          <t>1)NV VBIOS 驗證時間6周
-2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" hidden="1" outlineLevel="1">
-      <c r="A71" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="B71" s="8" t="inlineStr">
-        <is>
-          <t>2634</t>
-        </is>
-      </c>
-      <c r="C71" s="9" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WF</t>
-        </is>
-      </c>
-      <c r="D71" s="18" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E71" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 45W</t>
-        </is>
-      </c>
-      <c r="F71" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5060</t>
-        </is>
-      </c>
-      <c r="G71" s="9" t="inlineStr">
-        <is>
-          <t>賴雪鳳</t>
-        </is>
-      </c>
-      <c r="H71" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/22</t>
-        </is>
-      </c>
-      <c r="I71" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/07</t>
-        </is>
-      </c>
-      <c r="J71" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/16</t>
-        </is>
-      </c>
-      <c r="K71" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/11</t>
-        </is>
-      </c>
-      <c r="L71" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/27</t>
-        </is>
-      </c>
-      <c r="M71" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/29</t>
-        </is>
-      </c>
-      <c r="N71" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="O71" s="11" t="inlineStr">
-        <is>
-          <t>0A layout start 6/8-7/17</t>
-        </is>
-      </c>
-      <c r="P71" s="11" t="inlineStr">
+      <c r="P71" s="6" t="inlineStr">
         <is>
           <t>1)NV VBIOS 驗證時間6周
 2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
@@ -5948,7 +5939,7 @@
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
+          <t>Stealth 16 AI+ B4WF</t>
         </is>
       </c>
       <c r="D72" s="18" t="inlineStr">
@@ -5963,7 +5954,7 @@
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G72" s="9" t="inlineStr">
@@ -6029,7 +6020,7 @@
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
+          <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
         </is>
       </c>
       <c r="D73" s="18" t="inlineStr">
@@ -6099,161 +6090,162 @@
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="2" t="n">
+    <row r="74" hidden="1" outlineLevel="1">
+      <c r="A74" s="7" t="n">
         <v>73</v>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>2634</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
+        </is>
+      </c>
+      <c r="D74" s="18" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>NVL-H 45W</t>
+        </is>
+      </c>
+      <c r="F74" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G74" s="9" t="inlineStr">
+        <is>
+          <t>賴雪鳳</t>
+        </is>
+      </c>
+      <c r="H74" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="I74" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/07</t>
+        </is>
+      </c>
+      <c r="J74" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/16</t>
+        </is>
+      </c>
+      <c r="K74" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/11</t>
+        </is>
+      </c>
+      <c r="L74" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/27</t>
+        </is>
+      </c>
+      <c r="M74" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/29</t>
+        </is>
+      </c>
+      <c r="N74" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="O74" s="11" t="inlineStr">
+        <is>
+          <t>0A layout start 6/8-7/17</t>
+        </is>
+      </c>
+      <c r="P74" s="11" t="inlineStr">
+        <is>
+          <t>1)NV VBIOS 驗證時間6周
+2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>2654</t>
         </is>
       </c>
-      <c r="C74" s="4" t="inlineStr">
+      <c r="C75" s="4" t="inlineStr">
         <is>
           <t>Raider 16 Max HX B4WH</t>
         </is>
       </c>
-      <c r="D74" s="14" t="inlineStr">
+      <c r="D75" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E74" s="4" t="inlineStr">
+      <c r="E75" s="4" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F74" s="4" t="inlineStr">
+      <c r="F75" s="4" t="inlineStr">
         <is>
           <t>RTX 5070Ti</t>
         </is>
       </c>
-      <c r="G74" s="4" t="inlineStr">
+      <c r="G75" s="4" t="inlineStr">
         <is>
           <t>吳美芳</t>
         </is>
       </c>
-      <c r="H74" s="4" t="inlineStr">
+      <c r="H75" s="4" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I74" s="4" t="inlineStr">
+      <c r="I75" s="4" t="inlineStr">
         <is>
           <t>2026/07/27</t>
         </is>
       </c>
-      <c r="J74" s="4" t="inlineStr">
+      <c r="J75" s="4" t="inlineStr">
         <is>
           <t>2026/09/29</t>
         </is>
       </c>
-      <c r="K74" s="4" t="inlineStr">
+      <c r="K75" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L74" s="4" t="inlineStr">
+      <c r="L75" s="4" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M74" s="4" t="inlineStr">
+      <c r="M75" s="4" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N74" s="4" t="inlineStr">
+      <c r="N75" s="4" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O74" s="6" t="inlineStr">
+      <c r="O75" s="6" t="inlineStr">
         <is>
           <t>0M layout中，预计6/29 gerber out</t>
         </is>
       </c>
-      <c r="P74" s="6" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" hidden="1" outlineLevel="1">
-      <c r="A75" s="7" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" s="8" t="inlineStr">
-        <is>
-          <t>2654</t>
-        </is>
-      </c>
-      <c r="C75" s="9" t="inlineStr">
-        <is>
-          <t>Raider 16 Max HX B4WI</t>
-        </is>
-      </c>
-      <c r="D75" s="18" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E75" s="9" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F75" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5080</t>
-        </is>
-      </c>
-      <c r="G75" s="9" t="inlineStr">
-        <is>
-          <t>吳美芳</t>
-        </is>
-      </c>
-      <c r="H75" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/19</t>
-        </is>
-      </c>
-      <c r="I75" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/27</t>
-        </is>
-      </c>
-      <c r="J75" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/29</t>
-        </is>
-      </c>
-      <c r="K75" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="L75" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/02</t>
-        </is>
-      </c>
-      <c r="M75" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/08</t>
-        </is>
-      </c>
-      <c r="N75" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/18</t>
-        </is>
-      </c>
-      <c r="O75" s="11" t="inlineStr">
-        <is>
-          <t>0M layout中,预计6/29 gerber out</t>
-        </is>
-      </c>
-      <c r="P75" s="11" t="inlineStr">
+      <c r="P75" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -6270,7 +6262,7 @@
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>Raider 16 Max HX B4WJ</t>
+          <t>Raider 16 Max HX B4WI</t>
         </is>
       </c>
       <c r="D76" s="18" t="inlineStr">
@@ -6285,7 +6277,7 @@
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>RTX 5090</t>
+          <t>RTX 5080</t>
         </is>
       </c>
       <c r="G76" s="9" t="inlineStr">
@@ -6350,7 +6342,7 @@
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>Raider 16  HX B4WH</t>
+          <t>Raider 16 Max HX B4WJ</t>
         </is>
       </c>
       <c r="D77" s="18" t="inlineStr">
@@ -6365,7 +6357,7 @@
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070Ti</t>
+          <t>RTX 5090</t>
         </is>
       </c>
       <c r="G77" s="9" t="inlineStr">
@@ -6410,7 +6402,7 @@
       </c>
       <c r="O77" s="11" t="inlineStr">
         <is>
-          <t>0M layout中，预计6/29 gerber out</t>
+          <t>0M layout中,预计6/29 gerber out</t>
         </is>
       </c>
       <c r="P77" s="11" t="inlineStr">
@@ -6430,230 +6422,230 @@
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
+          <t>Raider 16  HX B4WH</t>
+        </is>
+      </c>
+      <c r="D78" s="18" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E78" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F78" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070Ti</t>
+        </is>
+      </c>
+      <c r="G78" s="9" t="inlineStr">
+        <is>
+          <t>吳美芳</t>
+        </is>
+      </c>
+      <c r="H78" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/19</t>
+        </is>
+      </c>
+      <c r="I78" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/27</t>
+        </is>
+      </c>
+      <c r="J78" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/29</t>
+        </is>
+      </c>
+      <c r="K78" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="L78" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/02</t>
+        </is>
+      </c>
+      <c r="M78" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N78" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O78" s="11" t="inlineStr">
+        <is>
+          <t>0M layout中，预计6/29 gerber out</t>
+        </is>
+      </c>
+      <c r="P78" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" hidden="1" outlineLevel="1">
+      <c r="A79" s="7" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>2654</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
           <t>Raider 16  HX B4WI</t>
         </is>
       </c>
-      <c r="D78" s="18" t="inlineStr">
+      <c r="D79" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E78" s="9" t="inlineStr">
+      <c r="E79" s="9" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F78" s="9" t="inlineStr">
+      <c r="F79" s="9" t="inlineStr">
         <is>
           <t>RTX 5080</t>
         </is>
       </c>
-      <c r="G78" s="9" t="inlineStr">
+      <c r="G79" s="9" t="inlineStr">
         <is>
           <t>吳美芳</t>
         </is>
       </c>
-      <c r="H78" s="9" t="inlineStr">
+      <c r="H79" s="9" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I78" s="9" t="inlineStr">
+      <c r="I79" s="9" t="inlineStr">
         <is>
           <t>2026/07/27</t>
         </is>
       </c>
-      <c r="J78" s="9" t="inlineStr">
+      <c r="J79" s="9" t="inlineStr">
         <is>
           <t>2026/09/29</t>
         </is>
       </c>
-      <c r="K78" s="9" t="inlineStr">
+      <c r="K79" s="9" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L78" s="9" t="inlineStr">
+      <c r="L79" s="9" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M78" s="9" t="inlineStr">
+      <c r="M79" s="9" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N78" s="9" t="inlineStr">
+      <c r="N79" s="9" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O78" s="11" t="inlineStr">
+      <c r="O79" s="11" t="inlineStr">
         <is>
           <t>0M layout中，预计6/29 gerber out</t>
         </is>
       </c>
-      <c r="P78" s="11" t="inlineStr">
+      <c r="P79" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="B79" s="3" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>2655</t>
         </is>
       </c>
-      <c r="C79" s="4" t="inlineStr">
+      <c r="C80" s="4" t="inlineStr">
         <is>
           <t>Crosshair 16 Max HX E4WEK</t>
         </is>
       </c>
-      <c r="D79" s="14" t="inlineStr">
+      <c r="D80" s="14" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E79" s="4" t="inlineStr">
+      <c r="E80" s="4" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F79" s="4" t="inlineStr">
+      <c r="F80" s="4" t="inlineStr">
         <is>
           <t>RTX 5050</t>
         </is>
       </c>
-      <c r="G79" s="4" t="inlineStr">
+      <c r="G80" s="4" t="inlineStr">
         <is>
           <t>鮑佩佩</t>
         </is>
       </c>
-      <c r="H79" s="4" t="inlineStr">
+      <c r="H80" s="4" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I79" s="4" t="inlineStr">
+      <c r="I80" s="4" t="inlineStr">
         <is>
           <t>2026/07/27</t>
         </is>
       </c>
-      <c r="J79" s="4" t="inlineStr">
+      <c r="J80" s="4" t="inlineStr">
         <is>
           <t>2026/09/29</t>
         </is>
       </c>
-      <c r="K79" s="4" t="inlineStr">
+      <c r="K80" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L79" s="4" t="inlineStr">
+      <c r="L80" s="4" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M79" s="4" t="inlineStr">
+      <c r="M80" s="4" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N79" s="4" t="inlineStr">
+      <c r="N80" s="4" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O79" s="6" t="inlineStr">
+      <c r="O80" s="6" t="inlineStr">
         <is>
           <t>0A layout中</t>
         </is>
       </c>
-      <c r="P79" s="6" t="inlineStr">
-        <is>
-          <t>plan 7/3 gerber out，比預期 delay 4d,對後續schedule無影響</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" hidden="1" outlineLevel="1">
-      <c r="A80" s="7" t="n">
-        <v>79</v>
-      </c>
-      <c r="B80" s="8" t="inlineStr">
-        <is>
-          <t>2655</t>
-        </is>
-      </c>
-      <c r="C80" s="9" t="inlineStr">
-        <is>
-          <t>Crosshair 16 Max HX E4WFK</t>
-        </is>
-      </c>
-      <c r="D80" s="18" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E80" s="9" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F80" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5060</t>
-        </is>
-      </c>
-      <c r="G80" s="9" t="inlineStr">
-        <is>
-          <t>鮑佩佩</t>
-        </is>
-      </c>
-      <c r="H80" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/19</t>
-        </is>
-      </c>
-      <c r="I80" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/27</t>
-        </is>
-      </c>
-      <c r="J80" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/29</t>
-        </is>
-      </c>
-      <c r="K80" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="L80" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/02</t>
-        </is>
-      </c>
-      <c r="M80" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/08</t>
-        </is>
-      </c>
-      <c r="N80" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/18</t>
-        </is>
-      </c>
-      <c r="O80" s="11" t="inlineStr">
-        <is>
-          <t>0A layout中</t>
-        </is>
-      </c>
-      <c r="P80" s="11" t="inlineStr">
+      <c r="P80" s="6" t="inlineStr">
         <is>
           <t>plan 7/3 gerber out，比預期 delay 4d,對後續schedule無影響</t>
         </is>
@@ -6670,7 +6662,7 @@
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 16 Max HX E4WGK</t>
+          <t>Crosshair 16 Max HX E4WFK</t>
         </is>
       </c>
       <c r="D81" s="18" t="inlineStr">
@@ -6685,7 +6677,7 @@
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G81" s="9" t="inlineStr">
@@ -6730,7 +6722,7 @@
       </c>
       <c r="O81" s="11" t="inlineStr">
         <is>
-          <t>GN22-X6 8GB SKU,0A layout中</t>
+          <t>0A layout中</t>
         </is>
       </c>
       <c r="P81" s="11" t="inlineStr">
@@ -6750,77 +6742,157 @@
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
+          <t>Crosshair 16 Max HX E4WGK</t>
+        </is>
+      </c>
+      <c r="D82" s="18" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F82" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G82" s="9" t="inlineStr">
+        <is>
+          <t>鮑佩佩</t>
+        </is>
+      </c>
+      <c r="H82" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/19</t>
+        </is>
+      </c>
+      <c r="I82" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/27</t>
+        </is>
+      </c>
+      <c r="J82" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/29</t>
+        </is>
+      </c>
+      <c r="K82" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="L82" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/02</t>
+        </is>
+      </c>
+      <c r="M82" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N82" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O82" s="11" t="inlineStr">
+        <is>
+          <t>GN22-X6 8GB SKU,0A layout中</t>
+        </is>
+      </c>
+      <c r="P82" s="11" t="inlineStr">
+        <is>
+          <t>plan 7/3 gerber out，比預期 delay 4d,對後續schedule無影響</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" hidden="1" outlineLevel="1">
+      <c r="A83" s="7" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>2655</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
           <t>Crosshair 16 Max HX E4WGXK</t>
         </is>
       </c>
-      <c r="D82" s="18" t="inlineStr">
+      <c r="D83" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E82" s="9" t="inlineStr">
+      <c r="E83" s="9" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F82" s="9" t="inlineStr">
+      <c r="F83" s="9" t="inlineStr">
         <is>
           <t>RTX 5070</t>
         </is>
       </c>
-      <c r="G82" s="9" t="inlineStr">
+      <c r="G83" s="9" t="inlineStr">
         <is>
           <t>鮑佩佩</t>
         </is>
       </c>
-      <c r="H82" s="9" t="inlineStr">
+      <c r="H83" s="9" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I82" s="9" t="inlineStr">
+      <c r="I83" s="9" t="inlineStr">
         <is>
           <t>2026/07/27</t>
         </is>
       </c>
-      <c r="J82" s="9" t="inlineStr">
+      <c r="J83" s="9" t="inlineStr">
         <is>
           <t>2026/09/29</t>
         </is>
       </c>
-      <c r="K82" s="9" t="inlineStr">
+      <c r="K83" s="9" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L82" s="9" t="inlineStr">
+      <c r="L83" s="9" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M82" s="9" t="inlineStr">
+      <c r="M83" s="9" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N82" s="9" t="inlineStr">
+      <c r="N83" s="9" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O82" s="11" t="inlineStr">
+      <c r="O83" s="11" t="inlineStr">
         <is>
           <t>GN22-X6 12GB SKU, 0A layout中</t>
         </is>
       </c>
-      <c r="P82" s="11" t="inlineStr">
+      <c r="P83" s="11" t="inlineStr">
         <is>
           <t>plan 7/3 gerber out，比預期 delay 4d,對後續schedule無影響</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P82"/>
+  <autoFilter ref="A1:P83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update NPI Dashboard 2026-06-30 08:15
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPI Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -52,12 +52,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0000B0F0"/>
+      <color rgb="007030A0"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="007030A0"/>
+      <color rgb="0000B0F0"/>
       <sz val="10"/>
     </font>
     <font>
@@ -142,16 +142,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -519,7 +519,7 @@
     <outlinePr summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P83"/>
+  <dimension ref="A1:P81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1582,9 +1582,9 @@
           <t>Cyborg 15 B2VE</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1818,7 +1818,7 @@
           <t>Venture 15 AI+ B3M</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -1894,7 +1894,7 @@
           <t>Katana 15 HX C14WEK</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -1970,7 +1970,7 @@
           <t>Katana 15 HX C14WFK</t>
         </is>
       </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2046,7 +2046,7 @@
           <t>Katana 15 HX C14WGK</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2119,10 +2119,10 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Katana 15 HX C14WGXK</t>
-        </is>
-      </c>
-      <c r="D22" s="16" t="inlineStr">
+          <t>Katana 15 HX C14WEOK</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
@@ -2144,38 +2144,38 @@
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
-          <t>2026/04/20</t>
+          <t>2026/05/15</t>
         </is>
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>2026/06/01</t>
+          <t>2026/06/15</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr"/>
       <c r="K22" s="9" t="inlineStr">
         <is>
-          <t>2026/07/14</t>
+          <t>2026/07/24</t>
         </is>
       </c>
       <c r="L22" s="9" t="inlineStr">
         <is>
-          <t>2026/07/30</t>
+          <t>2026/08/07</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>2026/08/20</t>
+          <t>2026/08/21</t>
         </is>
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>2026/08/30</t>
+          <t>2026/08/31</t>
         </is>
       </c>
       <c r="O22" s="11" t="inlineStr">
         <is>
-          <t>DDR5 sku, DVT測試中,預計7/2 PCB 10 gerberout</t>
+          <t>DDR4 sku, DVT測試中</t>
         </is>
       </c>
       <c r="P22" s="11" t="inlineStr">
@@ -2195,10 +2195,10 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Katana 15 HX C14WEOK</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
+          <t>Katana 15 HX C14WFOK</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
@@ -2271,10 +2271,10 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Katana 15 HX C14WFOK</t>
-        </is>
-      </c>
-      <c r="D24" s="16" t="inlineStr">
+          <t>Katana 15 HX C14WGOK</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
@@ -2336,79 +2336,80 @@
         </is>
       </c>
     </row>
-    <row r="25" hidden="1" outlineLevel="1">
-      <c r="A25" s="7" t="n">
+    <row r="25">
+      <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>15T3</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Katana 15 HX C14WGOK</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>15TK</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Cyborg A15 Max C1PWE</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>RPL-HX refresh 55W</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070</t>
-        </is>
-      </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>HWK 45W</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>RTX 5050</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>蔡東宏</t>
         </is>
       </c>
-      <c r="H25" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/15</t>
-        </is>
-      </c>
-      <c r="I25" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/15</t>
-        </is>
-      </c>
-      <c r="J25" s="9" t="inlineStr"/>
-      <c r="K25" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/24</t>
-        </is>
-      </c>
-      <c r="L25" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/07</t>
-        </is>
-      </c>
-      <c r="M25" s="9" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>2026/05/28</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>2026/06/26</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/17</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/31</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
         <is>
           <t>2026/08/21</t>
         </is>
       </c>
-      <c r="N25" s="9" t="inlineStr">
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>2026/08/31</t>
         </is>
       </c>
-      <c r="O25" s="11" t="inlineStr">
-        <is>
-          <t>DDR4 sku, DVT測試中</t>
-        </is>
-      </c>
-      <c r="P25" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>HPT sku:RD已重工3台成APU 180,AMI release PI 1200i RC3@6/29,BIOS RD需儘速提供MSI版本BIOSi進行測試</t>
+        </is>
+      </c>
+      <c r="P25" s="6" t="inlineStr">
+        <is>
+          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但AMD PI 1200i NDA release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
+2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS, 若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
         </is>
       </c>
     </row>
@@ -2418,27 +2419,27 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>15T3</t>
+          <t>15TK</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Katana 15 HX C14WGXOK</t>
-        </is>
-      </c>
-      <c r="D26" s="16" t="inlineStr">
+          <t>Cyborg A15 Max C1PWF</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>RPL-HX refresh 55W</t>
+          <t>HWK 45W</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
@@ -2448,23 +2449,23 @@
       </c>
       <c r="H26" s="9" t="inlineStr">
         <is>
-          <t>2026/05/15</t>
+          <t>2026/05/28</t>
         </is>
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>2026/06/15</t>
+          <t>2026/06/26</t>
         </is>
       </c>
       <c r="J26" s="9" t="inlineStr"/>
       <c r="K26" s="9" t="inlineStr">
         <is>
-          <t>2026/07/24</t>
+          <t>2026/07/17</t>
         </is>
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>2026/08/07</t>
+          <t>2026/07/31</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
@@ -2479,27 +2480,28 @@
       </c>
       <c r="O26" s="11" t="inlineStr">
         <is>
-          <t>DDR4 sku, DVT測試中</t>
+          <t>HPT sku:RD已重工3台成APU 180,AMI release PI 1200i RC3@6/29,BIOS RD需儘速提供MSI版本BIOSi進行測試</t>
         </is>
       </c>
       <c r="P26" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
+          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但AMD PI 1200i NDA release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
+2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS, 若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" hidden="1" outlineLevel="1">
+      <c r="A27" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>15TK</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Cyborg A15 Max C1PWE</t>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Cyborg A15 Max C1PWG</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
@@ -2507,58 +2509,58 @@
           <t>DVT</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t>HWK 45W</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5050</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t>蔡東宏</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="H27" s="9" t="inlineStr">
         <is>
           <t>2026/05/28</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="I27" s="9" t="inlineStr">
         <is>
           <t>2026/06/26</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr"/>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="J27" s="9" t="inlineStr"/>
+      <c r="K27" s="9" t="inlineStr">
         <is>
           <t>2026/07/17</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr">
+      <c r="L27" s="9" t="inlineStr">
         <is>
           <t>2026/07/31</t>
         </is>
       </c>
-      <c r="M27" s="4" t="inlineStr">
+      <c r="M27" s="9" t="inlineStr">
         <is>
           <t>2026/08/21</t>
         </is>
       </c>
-      <c r="N27" s="4" t="inlineStr">
+      <c r="N27" s="9" t="inlineStr">
         <is>
           <t>2026/08/31</t>
         </is>
       </c>
-      <c r="O27" s="6" t="inlineStr">
+      <c r="O27" s="11" t="inlineStr">
         <is>
           <t>HPT sku:RD已重工3台成APU 180,AMI release PI 1200i RC3@6/29,BIOS RD需儘速提供MSI版本BIOSi進行測試</t>
         </is>
       </c>
-      <c r="P27" s="6" t="inlineStr">
+      <c r="P27" s="11" t="inlineStr">
         <is>
           <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但AMD PI 1200i NDA release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
 2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS, 若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
@@ -2576,10 +2578,10 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1PWF</t>
-        </is>
-      </c>
-      <c r="D28" s="16" t="inlineStr">
+          <t>Cyborg A15 C1PWE</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2591,7 +2593,7 @@
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
@@ -2642,157 +2644,157 @@
         </is>
       </c>
     </row>
-    <row r="29" hidden="1" outlineLevel="1">
-      <c r="A29" s="7" t="n">
+    <row r="29">
+      <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>15TK</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Cyborg A15 Max C1PWG</t>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>24V1</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Modern 14 LE J3M</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>DVT</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>HWK 45W</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070</t>
-        </is>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>蔡東宏</t>
-        </is>
-      </c>
-      <c r="H29" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/28</t>
-        </is>
-      </c>
-      <c r="I29" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/26</t>
-        </is>
-      </c>
-      <c r="J29" s="9" t="inlineStr"/>
-      <c r="K29" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/17</t>
-        </is>
-      </c>
-      <c r="L29" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/31</t>
-        </is>
-      </c>
-      <c r="M29" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/21</t>
-        </is>
-      </c>
-      <c r="N29" s="9" t="inlineStr">
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>WCL 25W</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Intel® graphics</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>倪嬌嬌</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>2026/06/02</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>2026/06/29</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/29</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/06</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/17</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
         <is>
           <t>2026/08/31</t>
         </is>
       </c>
-      <c r="O29" s="11" t="inlineStr">
-        <is>
-          <t>HPT sku:RD已重工3台成APU 180,AMI release PI 1200i RC3@6/29,BIOS RD需儘速提供MSI版本BIOSi進行測試</t>
-        </is>
-      </c>
-      <c r="P29" s="11" t="inlineStr">
-        <is>
-          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但AMD PI 1200i NDA release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
-2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS, 若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" hidden="1" outlineLevel="1">
-      <c r="A30" s="7" t="n">
+      <c r="O29" s="6" t="inlineStr">
+        <is>
+          <t>Weibu plan 6/29 DVT SMT, 7/1 ASSY--熱管&amp;D件重新開模, 交期7/1</t>
+        </is>
+      </c>
+      <c r="P29" s="6" t="inlineStr">
+        <is>
+          <t>1)Schedule: 考量新料備料時程, 調整試產和ATS時間@8/17 start
+2)認證: 參考Weibu認證Schedule, 有四個國家無法同步於8/E TTM, 持續追蹤中 MX: 11/28 ready；AR:10/3 ready；CO: 9/5 ready；RU: 9/12 ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>15TK</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Cyborg A15 C1PWE</t>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>26V1</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Modern 16 LE J3M</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>DVT</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
-        <is>
-          <t>HWK 45W</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5050</t>
-        </is>
-      </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>蔡東宏</t>
-        </is>
-      </c>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/28</t>
-        </is>
-      </c>
-      <c r="I30" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/26</t>
-        </is>
-      </c>
-      <c r="J30" s="9" t="inlineStr"/>
-      <c r="K30" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/17</t>
-        </is>
-      </c>
-      <c r="L30" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/31</t>
-        </is>
-      </c>
-      <c r="M30" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/21</t>
-        </is>
-      </c>
-      <c r="N30" s="9" t="inlineStr">
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>WCL 25W</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Intel® graphics</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>倪嬌嬌</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>2026/06/02</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>2026/06/29</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/29</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/06</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/17</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
         <is>
           <t>2026/08/31</t>
         </is>
       </c>
-      <c r="O30" s="11" t="inlineStr">
-        <is>
-          <t>HPT sku:RD已重工3台成APU 180,AMI release PI 1200i RC3@6/29,BIOS RD需儘速提供MSI版本BIOSi進行測試</t>
-        </is>
-      </c>
-      <c r="P30" s="11" t="inlineStr">
-        <is>
-          <t>1).Schedule:APU 155優先ATS,採購已下單6.5k,以 8 月底 MP為目標,其餘APU sku在9月進行ATS C/R,但AMD PI 1200i NDA release延至6/30與APU 155 PR樣品ETD 延至7/11,已影響 MP 時程,待收到PI code與PR樣品後將依實際測試情況確認是否調整MP時程
-2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS, 若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
+      <c r="O30" s="6" t="inlineStr">
+        <is>
+          <t>Weibu plan 6/29 DVT SMT, 7/1 ASSY --熱管重新開模, 交期6/30</t>
+        </is>
+      </c>
+      <c r="P30" s="6" t="inlineStr">
+        <is>
+          <t>1)Schedule: 考量新料備料時程, 調整試產和ATS時間@8/17 start
+2)認證: 參考Weibu認證Schedule, 有四個國家無法同步於8/E TTM, 持續追蹤中 MX: 11/28 ready；AR:10/3 ready；CO: 9/5 ready；RU: 9/12 ready</t>
         </is>
       </c>
     </row>
@@ -2802,74 +2804,78 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>24V1</t>
+          <t>2623</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Modern 14 LE J3M</t>
-        </is>
-      </c>
-      <c r="D31" s="14" t="inlineStr">
-        <is>
-          <t>Design</t>
+          <t>Prestige N16 Spark C1M</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>EVT</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>WCL 25W</t>
+          <t>N1 45W</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Intel® graphics</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>倪嬌嬌</t>
+          <t>賴雪鳳</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>2026/06/02</t>
+          <t>2025/04/30</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>2026/06/29</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr"/>
+          <t>2025/09/01</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>2026/04/15</t>
+        </is>
+      </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>2026/07/29</t>
+          <t>2026/07/20</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>2026/07/06</t>
+          <t>2026/09/14</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>2026/08/17</t>
+          <t>2026/10/13</t>
         </is>
       </c>
       <c r="N31" s="4" t="inlineStr">
         <is>
-          <t>2026/08/31</t>
+          <t>2026/10/26</t>
         </is>
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
-          <t>Weibu plan 6/29 DVT SMT, 7/1 ASSY--熱管&amp;D件重新開模, 交期7/1</t>
+          <t>1)EVT 更新BSP6.1.2  持續驗證中, 對應NV schedule 更新 MVT延到7/20.
+2) NV 更新BSP 時間 Factory Drop Final ETA 10/6 ,需要1周時間完成 HDI+BIOS 更新ATS strat 10/13</t>
         </is>
       </c>
       <c r="P31" s="6" t="inlineStr">
         <is>
-          <t>1)Schedule: 考量新料備料時程, 調整試產和ATS時間@8/17 start
-2)認證: 參考Weibu認證Schedule, 有四個國家無法同步於8/E TTM, 持續追蹤中 MX: 11/28 ready；AR:10/3 ready；CO: 9/5 ready；RU: 9/12 ready</t>
+          <t>備料: Samsung 2.8K panel 可先出HR14*1K for N1 9月ATS 用, 另外要再驗證HR16 for後續出貨需求</t>
         </is>
       </c>
     </row>
@@ -2879,27 +2885,27 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>26V1</t>
+          <t>14T3</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Modern 16 LE J3M</t>
-        </is>
-      </c>
-      <c r="D32" s="14" t="inlineStr">
-        <is>
-          <t>Design</t>
+          <t>Prestige N14 Spark D1M</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>WCL 25W</t>
+          <t>N1 35W</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Intel® graphics</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -2909,44 +2915,47 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>2026/06/02</t>
+          <t>2025/04/30</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>2026/06/29</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr"/>
+          <t>2025/09/01</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>2026/04/15</t>
+        </is>
+      </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>2026/07/29</t>
+          <t>2026/07/20</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>2026/07/06</t>
+          <t>2026/09/14</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>2026/08/17</t>
+          <t>2026/10/13</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>2026/08/31</t>
+          <t>2026/10/26</t>
         </is>
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
-          <t>Weibu plan 6/29 DVT SMT, 7/1 ASSY --熱管重新開模, 交期6/30</t>
+          <t>MVT SMT@7/20--depend on Material ready date</t>
         </is>
       </c>
       <c r="P32" s="6" t="inlineStr">
         <is>
-          <t>1)Schedule: 考量新料備料時程, 調整試產和ATS時間@8/17 start
-2)認證: 參考Weibu認證Schedule, 有四個國家無法同步於8/E TTM, 持續追蹤中 MX: 11/28 ready；AR:10/3 ready；CO: 9/5 ready；RU: 9/12 ready</t>
+          <t>1)備料：MP focus on 2.8K panel, for MVT@7/M, 待廠商確認中; for MP: a, 1st lot 1K 數量, 型號HQ15, 九月份交料(同步Leading customers量產交料時間 具體九月份ETD日期還在追蹤中. b. Others order: 需轉型號至HQxx, 十一月份交料</t>
         </is>
       </c>
     </row>
@@ -2956,173 +2965,172 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>2623</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Prestige N16 Spark C1M</t>
-        </is>
-      </c>
-      <c r="D33" s="17" t="inlineStr">
-        <is>
-          <t>EVT</t>
+          <t>Katana 18 HX A14WEK</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>N1 45W</t>
+          <t>RPL-HX refresh 55W</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>賴雪鳳</t>
+          <t>顧曉琴</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>2025/04/30</t>
+          <t>2026/05/08</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>2025/09/01</t>
+          <t>2026/06/15</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>2026/04/15</t>
+          <t>2026/08/24</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>2026/07/20</t>
+          <t>2026/10/12</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>2026/09/14</t>
+          <t>2026/11/02</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
         <is>
-          <t>2026/10/13</t>
+          <t>2026/11/21</t>
         </is>
       </c>
       <c r="N33" s="4" t="inlineStr">
         <is>
-          <t>2026/10/26</t>
+          <t>2026/11/30</t>
         </is>
       </c>
       <c r="O33" s="6" t="inlineStr">
         <is>
-          <t>1)EVT 更新BSP6.1.2  持續驗證中, 對應NV schedule 更新 MVT延到7/20.
-2) NV 更新BSP 時間 Factory Drop Final ETA 10/6 ,需要1周時間完成 HDI+BIOS 更新ATS strat 10/13</t>
+          <t>RPL-HX R + DDR5: DVT PCBA快遞3pcs 6/24到,目前已開機,調撥部分6/25到料供RD測試</t>
         </is>
       </c>
       <c r="P33" s="6" t="inlineStr">
         <is>
-          <t>備料: Samsung 2.8K panel 可先出HR14*1K for N1 9月ATS 用, 另外要再驗證HR16 for後續出貨需求</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" hidden="1" outlineLevel="1">
+      <c r="A34" s="7" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>14T3</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Prestige N14 Spark D1M</t>
-        </is>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
-        <is>
-          <t>MVT</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>N1 35W</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>倪嬌嬌</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>2025/04/30</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>2025/09/01</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>2026/04/15</t>
-        </is>
-      </c>
-      <c r="K34" s="4" t="inlineStr">
-        <is>
-          <t>2026/07/20</t>
-        </is>
-      </c>
-      <c r="L34" s="4" t="inlineStr">
-        <is>
-          <t>2026/09/14</t>
-        </is>
-      </c>
-      <c r="M34" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/13</t>
-        </is>
-      </c>
-      <c r="N34" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/26</t>
-        </is>
-      </c>
-      <c r="O34" s="6" t="inlineStr">
-        <is>
-          <t>MVT SMT@7/20--depend on Material ready date</t>
-        </is>
-      </c>
-      <c r="P34" s="6" t="inlineStr">
-        <is>
-          <t>1)備料：MP focus on 2.8K panel, for MVT@7/M, 待廠商確認中; for MP: a, 1st lot 1K 數量, 型號HQ15, 九月份交料(同步Leading customers量產交料時間 具體九月份ETD日期還在追蹤中. b. Others order: 需轉型號至HQxx, 十一月份交料</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>1861</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Katana 18 HX A14WFK</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>RPL-HX refresh 55W</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5060</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>顧曉琴</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/08</t>
+        </is>
+      </c>
+      <c r="I34" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/15</t>
+        </is>
+      </c>
+      <c r="J34" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/24</t>
+        </is>
+      </c>
+      <c r="K34" s="9" t="inlineStr">
+        <is>
+          <t>2026/10/12</t>
+        </is>
+      </c>
+      <c r="L34" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/02</t>
+        </is>
+      </c>
+      <c r="M34" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/21</t>
+        </is>
+      </c>
+      <c r="N34" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/30</t>
+        </is>
+      </c>
+      <c r="O34" s="11" t="inlineStr">
+        <is>
+          <t>RPL-HX R + DDR5: DVT PCBA快遞3pcs 6/24到,目前已開機,調撥部分6/25到料供RD測試</t>
+        </is>
+      </c>
+      <c r="P34" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" hidden="1" outlineLevel="1">
+      <c r="A35" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>1861</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>Katana 18 HX A14WEK</t>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Katana 18 HX A14WGK</t>
         </is>
       </c>
       <c r="D35" s="15" t="inlineStr">
@@ -3130,62 +3138,62 @@
           <t>DVT</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E35" s="9" t="inlineStr">
         <is>
           <t>RPL-HX refresh 55W</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5050</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
         <is>
           <t>顧曉琴</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="H35" s="9" t="inlineStr">
         <is>
           <t>2026/05/08</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="I35" s="9" t="inlineStr">
         <is>
           <t>2026/06/15</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="J35" s="9" t="inlineStr">
         <is>
           <t>2026/08/24</t>
         </is>
       </c>
-      <c r="K35" s="4" t="inlineStr">
+      <c r="K35" s="9" t="inlineStr">
         <is>
           <t>2026/10/12</t>
         </is>
       </c>
-      <c r="L35" s="4" t="inlineStr">
+      <c r="L35" s="9" t="inlineStr">
         <is>
           <t>2026/11/02</t>
         </is>
       </c>
-      <c r="M35" s="4" t="inlineStr">
+      <c r="M35" s="9" t="inlineStr">
         <is>
           <t>2026/11/21</t>
         </is>
       </c>
-      <c r="N35" s="4" t="inlineStr">
+      <c r="N35" s="9" t="inlineStr">
         <is>
           <t>2026/11/30</t>
         </is>
       </c>
-      <c r="O35" s="6" t="inlineStr">
+      <c r="O35" s="11" t="inlineStr">
         <is>
           <t>RPL-HX R + DDR5: DVT PCBA快遞3pcs 6/24到,目前已開機,調撥部分6/25到料供RD測試</t>
         </is>
       </c>
-      <c r="P35" s="6" t="inlineStr">
+      <c r="P35" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -3202,10 +3210,10 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WFK</t>
-        </is>
-      </c>
-      <c r="D36" s="16" t="inlineStr">
+          <t>Katana 18 HX A14WEOK</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3217,7 +3225,7 @@
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
@@ -3227,22 +3235,18 @@
       </c>
       <c r="H36" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
+          <t>2026/05/20</t>
         </is>
       </c>
       <c r="I36" s="9" t="inlineStr">
         <is>
-          <t>2026/06/15</t>
-        </is>
-      </c>
-      <c r="J36" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/24</t>
-        </is>
-      </c>
+          <t>2026/06/27</t>
+        </is>
+      </c>
+      <c r="J36" s="9" t="inlineStr"/>
       <c r="K36" s="9" t="inlineStr">
         <is>
-          <t>2026/10/12</t>
+          <t>2026/10/20</t>
         </is>
       </c>
       <c r="L36" s="9" t="inlineStr">
@@ -3252,22 +3256,22 @@
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>2026/11/21</t>
+          <t>2026/11/23</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>2026/11/30</t>
+          <t>2026/12/02</t>
         </is>
       </c>
       <c r="O36" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT PCBA快遞3pcs 6/24到,目前已開機,調撥部分6/25到料供RD測試</t>
+          <t>RPL-HX R + DDR4: DVT SMT @ 6/30</t>
         </is>
       </c>
       <c r="P36" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -3282,10 +3286,10 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WGK</t>
-        </is>
-      </c>
-      <c r="D37" s="16" t="inlineStr">
+          <t>Katana 18 HX A14WFOK</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3297,7 +3301,7 @@
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
@@ -3307,22 +3311,18 @@
       </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
+          <t>2026/05/20</t>
         </is>
       </c>
       <c r="I37" s="9" t="inlineStr">
         <is>
-          <t>2026/06/15</t>
-        </is>
-      </c>
-      <c r="J37" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/24</t>
-        </is>
-      </c>
+          <t>2026/06/27</t>
+        </is>
+      </c>
+      <c r="J37" s="9" t="inlineStr"/>
       <c r="K37" s="9" t="inlineStr">
         <is>
-          <t>2026/10/12</t>
+          <t>2026/10/20</t>
         </is>
       </c>
       <c r="L37" s="9" t="inlineStr">
@@ -3332,22 +3332,22 @@
       </c>
       <c r="M37" s="9" t="inlineStr">
         <is>
-          <t>2026/11/21</t>
+          <t>2026/11/23</t>
         </is>
       </c>
       <c r="N37" s="9" t="inlineStr">
         <is>
-          <t>2026/11/30</t>
+          <t>2026/12/02</t>
         </is>
       </c>
       <c r="O37" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT PCBA快遞3pcs 6/24到,目前已開機,調撥部分6/25到料供RD測試</t>
+          <t>RPL-HX R + DDR4: DVT SMT @ 6/30</t>
         </is>
       </c>
       <c r="P37" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -3362,10 +3362,10 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WEOK</t>
-        </is>
-      </c>
-      <c r="D38" s="16" t="inlineStr">
+          <t>Katana 18 HX A14WGOK</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
@@ -3438,10 +3438,10 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WFOK</t>
-        </is>
-      </c>
-      <c r="D39" s="16" t="inlineStr">
+          <t>Crosshair 18 Max HX B14WEO</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
@@ -3484,12 +3484,12 @@
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>2026/11/23</t>
+          <t>2026/11/28</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
         <is>
-          <t>2026/12/02</t>
+          <t>2026/12/07</t>
         </is>
       </c>
       <c r="O39" s="11" t="inlineStr">
@@ -3514,10 +3514,10 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WGOK</t>
-        </is>
-      </c>
-      <c r="D40" s="16" t="inlineStr">
+          <t>Crosshair 18 Max HX B14WFO</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3529,7 +3529,7 @@
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
@@ -3560,12 +3560,12 @@
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>2026/11/23</t>
+          <t>2026/11/28</t>
         </is>
       </c>
       <c r="N40" s="9" t="inlineStr">
         <is>
-          <t>2026/12/02</t>
+          <t>2026/12/07</t>
         </is>
       </c>
       <c r="O40" s="11" t="inlineStr">
@@ -3590,10 +3590,10 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B14WEO</t>
-        </is>
-      </c>
-      <c r="D41" s="16" t="inlineStr">
+          <t>Crosshair 18 Max HX B14WGO</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
@@ -3666,10 +3666,10 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B14WFO</t>
-        </is>
-      </c>
-      <c r="D42" s="16" t="inlineStr">
+          <t>Crosshair 18 Max HX B14WGXO</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
@@ -3742,10 +3742,10 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B14WGO</t>
-        </is>
-      </c>
-      <c r="D43" s="16" t="inlineStr">
+          <t>Crosshair 18 Max HX B14WE</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
@@ -3767,15 +3767,19 @@
       </c>
       <c r="H43" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
+          <t>2026/05/08</t>
         </is>
       </c>
       <c r="I43" s="9" t="inlineStr">
         <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
-      <c r="J43" s="9" t="inlineStr"/>
+          <t>2026/06/15</t>
+        </is>
+      </c>
+      <c r="J43" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/24</t>
+        </is>
+      </c>
       <c r="K43" s="9" t="inlineStr">
         <is>
           <t>2026/10/20</t>
@@ -3798,12 +3802,12 @@
       </c>
       <c r="O43" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: DVT SMT @ 6/30</t>
+          <t>RPL-HX R + DDR5: DVT PCBA快遞3pcs 6/24到,目前已開機,調撥部分6/25到料供RD測試</t>
         </is>
       </c>
       <c r="P43" s="11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -3818,10 +3822,10 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B14WGXO</t>
-        </is>
-      </c>
-      <c r="D44" s="16" t="inlineStr">
+          <t>Crosshair 18 Max HX B14WF</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3833,7 +3837,7 @@
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G44" s="9" t="inlineStr">
@@ -3843,15 +3847,19 @@
       </c>
       <c r="H44" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
+          <t>2026/05/08</t>
         </is>
       </c>
       <c r="I44" s="9" t="inlineStr">
         <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
-      <c r="J44" s="9" t="inlineStr"/>
+          <t>2026/06/15</t>
+        </is>
+      </c>
+      <c r="J44" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/24</t>
+        </is>
+      </c>
       <c r="K44" s="9" t="inlineStr">
         <is>
           <t>2026/10/20</t>
@@ -3874,12 +3882,12 @@
       </c>
       <c r="O44" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: DVT SMT @ 6/30</t>
+          <t>RPL-HX R + DDR5: DVT PCBA快遞3pcs 6/24到,目前已開機,調撥部分6/25到料供RD測試</t>
         </is>
       </c>
       <c r="P44" s="11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -3894,10 +3902,10 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B14WE</t>
-        </is>
-      </c>
-      <c r="D45" s="16" t="inlineStr">
+          <t>Crosshair 18 Max HX B14WG</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3909,7 +3917,7 @@
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
@@ -3974,10 +3982,10 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B14WF</t>
-        </is>
-      </c>
-      <c r="D46" s="16" t="inlineStr">
+          <t>Crosshair 18 Max HX B14WGX</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3989,7 +3997,7 @@
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G46" s="9" t="inlineStr">
@@ -4054,22 +4062,22 @@
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B14WG</t>
-        </is>
-      </c>
-      <c r="D47" s="16" t="inlineStr">
-        <is>
-          <t>DVT</t>
+          <t>Crosshair 18 Max HX B2WE</t>
+        </is>
+      </c>
+      <c r="D47" s="18" t="inlineStr">
+        <is>
+          <t>Design</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>RPL-HX refresh 55W</t>
+          <t>RPL-HX Next 55W</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
@@ -4082,44 +4090,36 @@
           <t>2026/05/08</t>
         </is>
       </c>
-      <c r="I47" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/15</t>
-        </is>
-      </c>
-      <c r="J47" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/24</t>
-        </is>
-      </c>
+      <c r="I47" s="9" t="inlineStr"/>
+      <c r="J47" s="9" t="inlineStr"/>
       <c r="K47" s="9" t="inlineStr">
         <is>
-          <t>2026/10/20</t>
+          <t>2026/12/08</t>
         </is>
       </c>
       <c r="L47" s="9" t="inlineStr">
         <is>
-          <t>2026/11/02</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="M47" s="9" t="inlineStr">
         <is>
-          <t>2026/11/28</t>
+          <t>2027/01/19</t>
         </is>
       </c>
       <c r="N47" s="9" t="inlineStr">
         <is>
-          <t>2026/12/07</t>
+          <t>2027/01/30</t>
         </is>
       </c>
       <c r="O47" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT PCBA快遞3pcs 6/24到,目前已開機,調撥部分6/25到料供RD測試</t>
+          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P47" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -4134,22 +4134,22 @@
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B14WGX</t>
-        </is>
-      </c>
-      <c r="D48" s="16" t="inlineStr">
-        <is>
-          <t>DVT</t>
+          <t>Crosshair 18 Max HX B2WEO</t>
+        </is>
+      </c>
+      <c r="D48" s="18" t="inlineStr">
+        <is>
+          <t>Design</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>RPL-HX refresh 55W</t>
+          <t>RPL-HX Next 55W</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
@@ -4159,47 +4159,39 @@
       </c>
       <c r="H48" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I48" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/15</t>
-        </is>
-      </c>
-      <c r="J48" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/24</t>
-        </is>
-      </c>
+          <t>2026/05/20</t>
+        </is>
+      </c>
+      <c r="I48" s="9" t="inlineStr"/>
+      <c r="J48" s="9" t="inlineStr"/>
       <c r="K48" s="9" t="inlineStr">
         <is>
-          <t>2026/10/20</t>
+          <t>2026/12/08</t>
         </is>
       </c>
       <c r="L48" s="9" t="inlineStr">
         <is>
-          <t>2026/11/02</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>2026/11/28</t>
+          <t>2027/01/19</t>
         </is>
       </c>
       <c r="N48" s="9" t="inlineStr">
         <is>
-          <t>2026/12/07</t>
+          <t>2027/01/30</t>
         </is>
       </c>
       <c r="O48" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT PCBA快遞3pcs 6/24到,目前已開機,調撥部分6/25到料供RD測試</t>
+          <t>RPL-HX Next + DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P48" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4206,7 @@
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B2WE</t>
+          <t>Crosshair 18 Max HX B2WF</t>
         </is>
       </c>
       <c r="D49" s="18" t="inlineStr">
@@ -4229,7 +4221,7 @@
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
@@ -4286,7 +4278,7 @@
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B2WEO</t>
+          <t>Crosshair 18 Max HX B2WFO</t>
         </is>
       </c>
       <c r="D50" s="18" t="inlineStr">
@@ -4301,7 +4293,7 @@
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G50" s="9" t="inlineStr">
@@ -4358,7 +4350,7 @@
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B2WF</t>
+          <t>Crosshair 18 Max HX B2WG</t>
         </is>
       </c>
       <c r="D51" s="18" t="inlineStr">
@@ -4373,7 +4365,7 @@
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr">
@@ -4430,7 +4422,7 @@
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B2WFO</t>
+          <t>Crosshair 18 Max HX B2WGO</t>
         </is>
       </c>
       <c r="D52" s="18" t="inlineStr">
@@ -4445,7 +4437,7 @@
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
@@ -4502,7 +4494,7 @@
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B2WG</t>
+          <t>Crosshair 18 Max HX B2WGX</t>
         </is>
       </c>
       <c r="D53" s="18" t="inlineStr">
@@ -4574,7 +4566,7 @@
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B2WGO</t>
+          <t>Crosshair 18 Max HX B2WGXO</t>
         </is>
       </c>
       <c r="D54" s="18" t="inlineStr">
@@ -4646,7 +4638,7 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B2WGX</t>
+          <t>Katana 18 HX A2WEK</t>
         </is>
       </c>
       <c r="D55" s="18" t="inlineStr">
@@ -4661,7 +4653,7 @@
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
@@ -4718,7 +4710,7 @@
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 18 Max HX B2WGXO</t>
+          <t>Katana 18 HX A2WEOK</t>
         </is>
       </c>
       <c r="D56" s="18" t="inlineStr">
@@ -4733,7 +4725,7 @@
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G56" s="9" t="inlineStr">
@@ -4746,7 +4738,11 @@
           <t>2026/05/20</t>
         </is>
       </c>
-      <c r="I56" s="9" t="inlineStr"/>
+      <c r="I56" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/27</t>
+        </is>
+      </c>
       <c r="J56" s="9" t="inlineStr"/>
       <c r="K56" s="9" t="inlineStr">
         <is>
@@ -4770,7 +4766,7 @@
       </c>
       <c r="O56" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next + DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P56" s="11" t="inlineStr">
@@ -4790,7 +4786,7 @@
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WEK</t>
+          <t>Katana 18 HX A2WFK</t>
         </is>
       </c>
       <c r="D57" s="18" t="inlineStr">
@@ -4805,7 +4801,7 @@
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
@@ -4862,7 +4858,7 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WEOK</t>
+          <t>Katana 18 HX A2WFOK</t>
         </is>
       </c>
       <c r="D58" s="18" t="inlineStr">
@@ -4877,7 +4873,7 @@
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
@@ -4938,7 +4934,7 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WFK</t>
+          <t>Katana 18 HX A2WGK</t>
         </is>
       </c>
       <c r="D59" s="18" t="inlineStr">
@@ -4953,7 +4949,7 @@
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
@@ -5010,7 +5006,7 @@
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WFOK</t>
+          <t>Katana 18 HX A2WGOK</t>
         </is>
       </c>
       <c r="D60" s="18" t="inlineStr">
@@ -5025,7 +5021,7 @@
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
@@ -5075,75 +5071,83 @@
         </is>
       </c>
     </row>
-    <row r="61" hidden="1" outlineLevel="1">
-      <c r="A61" s="7" t="n">
+    <row r="61">
+      <c r="A61" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="8" t="inlineStr">
-        <is>
-          <t>1861</t>
-        </is>
-      </c>
-      <c r="C61" s="9" t="inlineStr">
-        <is>
-          <t>Katana 18 HX A2WGK</t>
-        </is>
-      </c>
-      <c r="D61" s="18" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>14T4</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Prestige 14 AI</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E61" s="9" t="inlineStr">
-        <is>
-          <t>RPL-HX Next 55W</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070</t>
-        </is>
-      </c>
-      <c r="G61" s="9" t="inlineStr">
-        <is>
-          <t>顧曉琴</t>
-        </is>
-      </c>
-      <c r="H61" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I61" s="9" t="inlineStr"/>
-      <c r="J61" s="9" t="inlineStr"/>
-      <c r="K61" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/08</t>
-        </is>
-      </c>
-      <c r="L61" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/30</t>
-        </is>
-      </c>
-      <c r="M61" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/19</t>
-        </is>
-      </c>
-      <c r="N61" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/30</t>
-        </is>
-      </c>
-      <c r="O61" s="11" t="inlineStr">
-        <is>
-          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
-        </is>
-      </c>
-      <c r="P61" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>NVL-H 30W</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Intel® Arc™ Graphics</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>朱芳芳</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>2026/05/14</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/22</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/15</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/04</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/20</t>
+        </is>
+      </c>
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/15</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/25</t>
+        </is>
+      </c>
+      <c r="O61" s="6" t="inlineStr">
+        <is>
+          <t>0A gerberout ：6/26,DVT SMT@7/22</t>
+        </is>
+      </c>
+      <c r="P61" s="6" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -5153,12 +5157,12 @@
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>14T4</t>
         </is>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WGOK</t>
+          <t>Prestige 14 AI+ Flip</t>
         </is>
       </c>
       <c r="D62" s="18" t="inlineStr">
@@ -5168,58 +5172,62 @@
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>RPL-HX Next 55W</t>
+          <t>NVL-H 30W</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>Intel® Arc™ Graphics</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>顧曉琴</t>
+          <t>朱芳芳</t>
         </is>
       </c>
       <c r="H62" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
+          <t>2026/05/14</t>
         </is>
       </c>
       <c r="I62" s="9" t="inlineStr">
         <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
-      <c r="J62" s="9" t="inlineStr"/>
+          <t>2026/07/22</t>
+        </is>
+      </c>
+      <c r="J62" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/15</t>
+        </is>
+      </c>
       <c r="K62" s="9" t="inlineStr">
         <is>
-          <t>2026/12/08</t>
+          <t>2026/11/04</t>
         </is>
       </c>
       <c r="L62" s="9" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/11/20</t>
         </is>
       </c>
       <c r="M62" s="9" t="inlineStr">
         <is>
-          <t>2027/01/19</t>
+          <t>2026/12/15</t>
         </is>
       </c>
       <c r="N62" s="9" t="inlineStr">
         <is>
-          <t>2027/01/30</t>
+          <t>2026/12/25</t>
         </is>
       </c>
       <c r="O62" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>0A gerberout ：6/26,DVT SMT@7/22</t>
         </is>
       </c>
       <c r="P62" s="11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -5229,15 +5237,15 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>14T4</t>
+          <t>2624</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Prestige 14 AI</t>
-        </is>
-      </c>
-      <c r="D63" s="14" t="inlineStr">
+          <t>Prestige 16 AI+</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5262,11 +5270,7 @@
           <t>2026/05/14</t>
         </is>
       </c>
-      <c r="I63" s="4" t="inlineStr">
-        <is>
-          <t>2026/07/22</t>
-        </is>
-      </c>
+      <c r="I63" s="4" t="inlineStr"/>
       <c r="J63" s="4" t="inlineStr">
         <is>
           <t>2026/09/15</t>
@@ -5309,12 +5313,12 @@
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>14T4</t>
+          <t>2624</t>
         </is>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Prestige 14 AI+ Flip</t>
+          <t>Prestige 16 Flip AI+</t>
         </is>
       </c>
       <c r="D64" s="18" t="inlineStr">
@@ -5342,11 +5346,7 @@
           <t>2026/05/14</t>
         </is>
       </c>
-      <c r="I64" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/22</t>
-        </is>
-      </c>
+      <c r="I64" s="9" t="inlineStr"/>
       <c r="J64" s="9" t="inlineStr">
         <is>
           <t>2026/09/15</t>
@@ -5389,22 +5389,22 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>2624</t>
+          <t>13Q5</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Prestige 16 AI+</t>
-        </is>
-      </c>
-      <c r="D65" s="14" t="inlineStr">
+          <t>Prestige 13 AI+ A4M</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>NVL-H 30W</t>
+          <t>NVL-H 28W</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -5414,356 +5414,365 @@
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>朱芳芳</t>
+          <t>顏春梅</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>2026/05/14</t>
-        </is>
-      </c>
-      <c r="I65" s="4" t="inlineStr"/>
+          <t>2026/06/29</t>
+        </is>
+      </c>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/18</t>
+        </is>
+      </c>
       <c r="J65" s="4" t="inlineStr">
         <is>
-          <t>2026/09/15</t>
+          <t>2026/10/08</t>
         </is>
       </c>
       <c r="K65" s="4" t="inlineStr">
         <is>
-          <t>2026/11/04</t>
+          <t>2026/11/21</t>
         </is>
       </c>
       <c r="L65" s="4" t="inlineStr">
         <is>
-          <t>2026/11/20</t>
+          <t>2026/11/22</t>
         </is>
       </c>
       <c r="M65" s="4" t="inlineStr">
         <is>
-          <t>2026/12/15</t>
+          <t>2026/12/22</t>
         </is>
       </c>
       <c r="N65" s="4" t="inlineStr">
         <is>
-          <t>2026/12/25</t>
-        </is>
-      </c>
-      <c r="O65" s="6" t="inlineStr">
-        <is>
-          <t>0A gerberout ：6/26,DVT SMT@7/22</t>
-        </is>
-      </c>
-      <c r="P65" s="6" t="inlineStr">
+          <t>2026/12/31</t>
+        </is>
+      </c>
+      <c r="O65" s="6" t="inlineStr"/>
+      <c r="P65" s="6" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>2633</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WI</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>NVL-H 45W</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>RTX 5080</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>朱欣怡</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/22</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/16</t>
+        </is>
+      </c>
+      <c r="K66" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/11</t>
+        </is>
+      </c>
+      <c r="L66" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/30</t>
+        </is>
+      </c>
+      <c r="M66" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/29</t>
+        </is>
+      </c>
+      <c r="N66" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="O66" s="6" t="inlineStr">
+        <is>
+          <t>0M layout中，预计6/30 gerber out</t>
+        </is>
+      </c>
+      <c r="P66" s="6" t="inlineStr">
+        <is>
+          <t>1) Schedule:NV VBIOS @1/6, gating 8天,預計12/E 拿到WHQL，可能影響到最終TTM 時間</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" hidden="1" outlineLevel="1">
+      <c r="A67" s="7" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>2633</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WH</t>
+        </is>
+      </c>
+      <c r="D67" s="18" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E67" s="9" t="inlineStr">
+        <is>
+          <t>NVL-H 45W</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070Ti</t>
+        </is>
+      </c>
+      <c r="G67" s="9" t="inlineStr">
+        <is>
+          <t>朱欣怡</t>
+        </is>
+      </c>
+      <c r="H67" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="I67" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/22</t>
+        </is>
+      </c>
+      <c r="J67" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/16</t>
+        </is>
+      </c>
+      <c r="K67" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/11</t>
+        </is>
+      </c>
+      <c r="L67" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/30</t>
+        </is>
+      </c>
+      <c r="M67" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/29</t>
+        </is>
+      </c>
+      <c r="N67" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="O67" s="11" t="inlineStr">
+        <is>
+          <t>0M layout中，预计6/30 gerber out</t>
+        </is>
+      </c>
+      <c r="P67" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="66" hidden="1" outlineLevel="1">
-      <c r="A66" s="7" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" s="8" t="inlineStr">
-        <is>
-          <t>2624</t>
-        </is>
-      </c>
-      <c r="C66" s="9" t="inlineStr">
-        <is>
-          <t>Prestige 16 Flip AI+</t>
-        </is>
-      </c>
-      <c r="D66" s="18" t="inlineStr">
+    <row r="68" hidden="1" outlineLevel="1">
+      <c r="A68" s="7" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>2633</t>
+        </is>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WJ</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E66" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 30W</t>
-        </is>
-      </c>
-      <c r="F66" s="9" t="inlineStr">
-        <is>
-          <t>Intel® Arc™ Graphics</t>
-        </is>
-      </c>
-      <c r="G66" s="9" t="inlineStr">
-        <is>
-          <t>朱芳芳</t>
-        </is>
-      </c>
-      <c r="H66" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/14</t>
-        </is>
-      </c>
-      <c r="I66" s="9" t="inlineStr"/>
-      <c r="J66" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/15</t>
-        </is>
-      </c>
-      <c r="K66" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/04</t>
-        </is>
-      </c>
-      <c r="L66" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/20</t>
-        </is>
-      </c>
-      <c r="M66" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/15</t>
-        </is>
-      </c>
-      <c r="N66" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/25</t>
-        </is>
-      </c>
-      <c r="O66" s="11" t="inlineStr">
-        <is>
-          <t>0A gerberout ：6/26,DVT SMT@7/22</t>
-        </is>
-      </c>
-      <c r="P66" s="11" t="inlineStr">
+      <c r="E68" s="9" t="inlineStr">
+        <is>
+          <t>NVL-H 45W</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5090</t>
+        </is>
+      </c>
+      <c r="G68" s="9" t="inlineStr">
+        <is>
+          <t>朱欣怡</t>
+        </is>
+      </c>
+      <c r="H68" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="I68" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/22</t>
+        </is>
+      </c>
+      <c r="J68" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/16</t>
+        </is>
+      </c>
+      <c r="K68" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/11</t>
+        </is>
+      </c>
+      <c r="L68" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/30</t>
+        </is>
+      </c>
+      <c r="M68" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/29</t>
+        </is>
+      </c>
+      <c r="N68" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="O68" s="11" t="inlineStr">
+        <is>
+          <t>0M layout中，预计6/30 gerber out</t>
+        </is>
+      </c>
+      <c r="P68" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>13Q5</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>Prestige 13 AI+ A4M</t>
-        </is>
-      </c>
-      <c r="D67" s="14" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>2634</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WE</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>NVL-H 28W</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>Intel® Arc™ Graphics</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>顏春梅</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>2026/06/29</t>
-        </is>
-      </c>
-      <c r="I67" s="4" t="inlineStr">
-        <is>
-          <t>2026/08/18</t>
-        </is>
-      </c>
-      <c r="J67" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/08</t>
-        </is>
-      </c>
-      <c r="K67" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/21</t>
-        </is>
-      </c>
-      <c r="L67" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/22</t>
-        </is>
-      </c>
-      <c r="M67" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/22</t>
-        </is>
-      </c>
-      <c r="N67" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/31</t>
-        </is>
-      </c>
-      <c r="O67" s="6" t="inlineStr"/>
-      <c r="P67" s="6" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>2633</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WI</t>
-        </is>
-      </c>
-      <c r="D68" s="14" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="E69" s="4" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F68" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5080</t>
-        </is>
-      </c>
-      <c r="G68" s="4" t="inlineStr">
-        <is>
-          <t>朱欣怡</t>
-        </is>
-      </c>
-      <c r="H68" s="4" t="inlineStr">
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>RTX 5050</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>賴雪鳳</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I68" s="4" t="inlineStr">
-        <is>
-          <t>2026/07/22</t>
-        </is>
-      </c>
-      <c r="J68" s="4" t="inlineStr">
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/07</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
         <is>
           <t>2026/09/16</t>
         </is>
       </c>
-      <c r="K68" s="4" t="inlineStr">
+      <c r="K69" s="4" t="inlineStr">
         <is>
           <t>2026/11/11</t>
         </is>
       </c>
-      <c r="L68" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/30</t>
-        </is>
-      </c>
-      <c r="M68" s="4" t="inlineStr">
+      <c r="L69" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/27</t>
+        </is>
+      </c>
+      <c r="M69" s="4" t="inlineStr">
         <is>
           <t>2026/12/29</t>
         </is>
       </c>
-      <c r="N68" s="4" t="inlineStr">
+      <c r="N69" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="O68" s="6" t="inlineStr">
-        <is>
-          <t>0M layout中，预计6/30 gerber out</t>
-        </is>
-      </c>
-      <c r="P68" s="6" t="inlineStr">
-        <is>
-          <t>1) Schedule:NV VBIOS @1/6, gating 8天,預計12/E 拿到WHQL，可能影響到最終TTM 時間</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" hidden="1" outlineLevel="1">
-      <c r="A69" s="7" t="n">
-        <v>68</v>
-      </c>
-      <c r="B69" s="8" t="inlineStr">
-        <is>
-          <t>2633</t>
-        </is>
-      </c>
-      <c r="C69" s="9" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WH</t>
-        </is>
-      </c>
-      <c r="D69" s="18" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E69" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 45W</t>
-        </is>
-      </c>
-      <c r="F69" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070Ti</t>
-        </is>
-      </c>
-      <c r="G69" s="9" t="inlineStr">
-        <is>
-          <t>朱欣怡</t>
-        </is>
-      </c>
-      <c r="H69" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/22</t>
-        </is>
-      </c>
-      <c r="I69" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/22</t>
-        </is>
-      </c>
-      <c r="J69" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/16</t>
-        </is>
-      </c>
-      <c r="K69" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/11</t>
-        </is>
-      </c>
-      <c r="L69" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/30</t>
-        </is>
-      </c>
-      <c r="M69" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/29</t>
-        </is>
-      </c>
-      <c r="N69" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="O69" s="11" t="inlineStr">
-        <is>
-          <t>0M layout中，预计6/30 gerber out</t>
-        </is>
-      </c>
-      <c r="P69" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="O69" s="6" t="inlineStr">
+        <is>
+          <t>0A layout start 6/8-7/17</t>
+        </is>
+      </c>
+      <c r="P69" s="6" t="inlineStr">
+        <is>
+          <t>1)NV VBIOS 驗證時間6周
+2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
         </is>
       </c>
     </row>
@@ -5773,12 +5782,12 @@
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>2633</t>
+          <t>2634</t>
         </is>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WJ</t>
+          <t>Stealth 16 AI+ B4WF</t>
         </is>
       </c>
       <c r="D70" s="18" t="inlineStr">
@@ -5793,12 +5802,12 @@
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>RTX 5090</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>朱欣怡</t>
+          <t>賴雪鳳</t>
         </is>
       </c>
       <c r="H70" s="9" t="inlineStr">
@@ -5808,7 +5817,7 @@
       </c>
       <c r="I70" s="9" t="inlineStr">
         <is>
-          <t>2026/07/22</t>
+          <t>2026/08/07</t>
         </is>
       </c>
       <c r="J70" s="9" t="inlineStr">
@@ -5823,7 +5832,7 @@
       </c>
       <c r="L70" s="9" t="inlineStr">
         <is>
-          <t>2026/11/30</t>
+          <t>2026/11/27</t>
         </is>
       </c>
       <c r="M70" s="9" t="inlineStr">
@@ -5838,90 +5847,91 @@
       </c>
       <c r="O70" s="11" t="inlineStr">
         <is>
-          <t>0M layout中，预计6/30 gerber out</t>
+          <t>0A layout start 6/8-7/17</t>
         </is>
       </c>
       <c r="P70" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="n">
+          <t>1)NV VBIOS 驗證時間6周
+2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" hidden="1" outlineLevel="1">
+      <c r="A71" s="7" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="3" t="inlineStr">
+      <c r="B71" s="8" t="inlineStr">
         <is>
           <t>2634</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WE</t>
-        </is>
-      </c>
-      <c r="D71" s="14" t="inlineStr">
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E71" s="4" t="inlineStr">
+      <c r="E71" s="9" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F71" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5050</t>
-        </is>
-      </c>
-      <c r="G71" s="4" t="inlineStr">
+      <c r="F71" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G71" s="9" t="inlineStr">
         <is>
           <t>賴雪鳳</t>
         </is>
       </c>
-      <c r="H71" s="4" t="inlineStr">
+      <c r="H71" s="9" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I71" s="4" t="inlineStr">
+      <c r="I71" s="9" t="inlineStr">
         <is>
           <t>2026/08/07</t>
         </is>
       </c>
-      <c r="J71" s="4" t="inlineStr">
+      <c r="J71" s="9" t="inlineStr">
         <is>
           <t>2026/09/16</t>
         </is>
       </c>
-      <c r="K71" s="4" t="inlineStr">
+      <c r="K71" s="9" t="inlineStr">
         <is>
           <t>2026/11/11</t>
         </is>
       </c>
-      <c r="L71" s="4" t="inlineStr">
+      <c r="L71" s="9" t="inlineStr">
         <is>
           <t>2026/11/27</t>
         </is>
       </c>
-      <c r="M71" s="4" t="inlineStr">
+      <c r="M71" s="9" t="inlineStr">
         <is>
           <t>2026/12/29</t>
         </is>
       </c>
-      <c r="N71" s="4" t="inlineStr">
+      <c r="N71" s="9" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="O71" s="6" t="inlineStr">
+      <c r="O71" s="11" t="inlineStr">
         <is>
           <t>0A layout start 6/8-7/17</t>
         </is>
       </c>
-      <c r="P71" s="6" t="inlineStr">
+      <c r="P71" s="11" t="inlineStr">
         <is>
           <t>1)NV VBIOS 驗證時間6周
 2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
@@ -5939,7 +5949,7 @@
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WF</t>
+          <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
         </is>
       </c>
       <c r="D72" s="18" t="inlineStr">
@@ -5954,7 +5964,7 @@
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G72" s="9" t="inlineStr">
@@ -6009,84 +6019,83 @@
         </is>
       </c>
     </row>
-    <row r="73" hidden="1" outlineLevel="1">
-      <c r="A73" s="7" t="n">
+    <row r="73">
+      <c r="A73" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="B73" s="8" t="inlineStr">
-        <is>
-          <t>2634</t>
-        </is>
-      </c>
-      <c r="C73" s="9" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
-        </is>
-      </c>
-      <c r="D73" s="18" t="inlineStr">
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>2654</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Raider 16 Max HX B4WH</t>
+        </is>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E73" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 45W</t>
-        </is>
-      </c>
-      <c r="F73" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070</t>
-        </is>
-      </c>
-      <c r="G73" s="9" t="inlineStr">
-        <is>
-          <t>賴雪鳳</t>
-        </is>
-      </c>
-      <c r="H73" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/22</t>
-        </is>
-      </c>
-      <c r="I73" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/07</t>
-        </is>
-      </c>
-      <c r="J73" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/16</t>
-        </is>
-      </c>
-      <c r="K73" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/11</t>
-        </is>
-      </c>
-      <c r="L73" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/27</t>
-        </is>
-      </c>
-      <c r="M73" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/29</t>
-        </is>
-      </c>
-      <c r="N73" s="9" t="inlineStr">
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>RTX 5070Ti</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>吳美芳</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>2026/05/19</t>
+        </is>
+      </c>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/27</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/29</t>
+        </is>
+      </c>
+      <c r="K73" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="O73" s="11" t="inlineStr">
-        <is>
-          <t>0A layout start 6/8-7/17</t>
-        </is>
-      </c>
-      <c r="P73" s="11" t="inlineStr">
-        <is>
-          <t>1)NV VBIOS 驗證時間6周
-2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
+      <c r="L73" s="4" t="inlineStr">
+        <is>
+          <t>2027/02/02</t>
+        </is>
+      </c>
+      <c r="M73" s="4" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N73" s="4" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O73" s="6" t="inlineStr">
+        <is>
+          <t>0M layout中，预计6/29 gerber out</t>
+        </is>
+      </c>
+      <c r="P73" s="6" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -6096,12 +6105,12 @@
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>2634</t>
+          <t>2654</t>
         </is>
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
+          <t>Raider 16 Max HX B4WI</t>
         </is>
       </c>
       <c r="D74" s="18" t="inlineStr">
@@ -6111,141 +6120,140 @@
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>NVL-H 45W</t>
+          <t>NVL-HX 55W</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5080</t>
         </is>
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>賴雪鳳</t>
+          <t>吳美芳</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
         <is>
-          <t>2026/05/22</t>
+          <t>2026/05/19</t>
         </is>
       </c>
       <c r="I74" s="9" t="inlineStr">
         <is>
-          <t>2026/08/07</t>
+          <t>2026/07/27</t>
         </is>
       </c>
       <c r="J74" s="9" t="inlineStr">
         <is>
-          <t>2026/09/16</t>
+          <t>2026/09/29</t>
         </is>
       </c>
       <c r="K74" s="9" t="inlineStr">
         <is>
-          <t>2026/11/11</t>
+          <t>2027/01/11</t>
         </is>
       </c>
       <c r="L74" s="9" t="inlineStr">
         <is>
-          <t>2026/11/27</t>
+          <t>2027/02/02</t>
         </is>
       </c>
       <c r="M74" s="9" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2027/03/08</t>
         </is>
       </c>
       <c r="N74" s="9" t="inlineStr">
         <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O74" s="11" t="inlineStr">
+        <is>
+          <t>0M layout中,预计6/29 gerber out</t>
+        </is>
+      </c>
+      <c r="P74" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" hidden="1" outlineLevel="1">
+      <c r="A75" s="7" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>2654</t>
+        </is>
+      </c>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>Raider 16 Max HX B4WJ</t>
+        </is>
+      </c>
+      <c r="D75" s="18" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5090</t>
+        </is>
+      </c>
+      <c r="G75" s="9" t="inlineStr">
+        <is>
+          <t>吳美芳</t>
+        </is>
+      </c>
+      <c r="H75" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/19</t>
+        </is>
+      </c>
+      <c r="I75" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/27</t>
+        </is>
+      </c>
+      <c r="J75" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/29</t>
+        </is>
+      </c>
+      <c r="K75" s="9" t="inlineStr">
+        <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="O74" s="11" t="inlineStr">
-        <is>
-          <t>0A layout start 6/8-7/17</t>
-        </is>
-      </c>
-      <c r="P74" s="11" t="inlineStr">
-        <is>
-          <t>1)NV VBIOS 驗證時間6周
-2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>2654</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>Raider 16 Max HX B4WH</t>
-        </is>
-      </c>
-      <c r="D75" s="14" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5070Ti</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>吳美芳</t>
-        </is>
-      </c>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>2026/05/19</t>
-        </is>
-      </c>
-      <c r="I75" s="4" t="inlineStr">
-        <is>
-          <t>2026/07/27</t>
-        </is>
-      </c>
-      <c r="J75" s="4" t="inlineStr">
-        <is>
-          <t>2026/09/29</t>
-        </is>
-      </c>
-      <c r="K75" s="4" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="L75" s="4" t="inlineStr">
+      <c r="L75" s="9" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M75" s="4" t="inlineStr">
+      <c r="M75" s="9" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N75" s="4" t="inlineStr">
+      <c r="N75" s="9" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O75" s="6" t="inlineStr">
-        <is>
-          <t>0M layout中，预计6/29 gerber out</t>
-        </is>
-      </c>
-      <c r="P75" s="6" t="inlineStr">
+      <c r="O75" s="11" t="inlineStr">
+        <is>
+          <t>0M layout中,预计6/29 gerber out</t>
+        </is>
+      </c>
+      <c r="P75" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -6262,7 +6270,7 @@
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>Raider 16 Max HX B4WI</t>
+          <t>Raider 16  HX B4WH</t>
         </is>
       </c>
       <c r="D76" s="18" t="inlineStr">
@@ -6277,7 +6285,7 @@
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>RTX 5080</t>
+          <t>RTX 5070Ti</t>
         </is>
       </c>
       <c r="G76" s="9" t="inlineStr">
@@ -6322,7 +6330,7 @@
       </c>
       <c r="O76" s="11" t="inlineStr">
         <is>
-          <t>0M layout中,预计6/29 gerber out</t>
+          <t>0M layout中，预计6/29 gerber out</t>
         </is>
       </c>
       <c r="P76" s="11" t="inlineStr">
@@ -6342,7 +6350,7 @@
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>Raider 16 Max HX B4WJ</t>
+          <t>Raider 16  HX B4WI</t>
         </is>
       </c>
       <c r="D77" s="18" t="inlineStr">
@@ -6357,7 +6365,7 @@
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>RTX 5090</t>
+          <t>RTX 5080</t>
         </is>
       </c>
       <c r="G77" s="9" t="inlineStr">
@@ -6402,7 +6410,7 @@
       </c>
       <c r="O77" s="11" t="inlineStr">
         <is>
-          <t>0M layout中,预计6/29 gerber out</t>
+          <t>0M layout中，预计6/29 gerber out</t>
         </is>
       </c>
       <c r="P77" s="11" t="inlineStr">
@@ -6411,83 +6419,83 @@
         </is>
       </c>
     </row>
-    <row r="78" hidden="1" outlineLevel="1">
-      <c r="A78" s="7" t="n">
+    <row r="78">
+      <c r="A78" s="2" t="n">
         <v>77</v>
       </c>
-      <c r="B78" s="8" t="inlineStr">
-        <is>
-          <t>2654</t>
-        </is>
-      </c>
-      <c r="C78" s="9" t="inlineStr">
-        <is>
-          <t>Raider 16  HX B4WH</t>
-        </is>
-      </c>
-      <c r="D78" s="18" t="inlineStr">
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>2655</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Crosshair 16 Max HX E4WEK</t>
+        </is>
+      </c>
+      <c r="D78" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E78" s="9" t="inlineStr">
+      <c r="E78" s="4" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F78" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070Ti</t>
-        </is>
-      </c>
-      <c r="G78" s="9" t="inlineStr">
-        <is>
-          <t>吳美芳</t>
-        </is>
-      </c>
-      <c r="H78" s="9" t="inlineStr">
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>RTX 5050</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>鮑佩佩</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I78" s="9" t="inlineStr">
+      <c r="I78" s="4" t="inlineStr">
         <is>
           <t>2026/07/27</t>
         </is>
       </c>
-      <c r="J78" s="9" t="inlineStr">
+      <c r="J78" s="4" t="inlineStr">
         <is>
           <t>2026/09/29</t>
         </is>
       </c>
-      <c r="K78" s="9" t="inlineStr">
+      <c r="K78" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L78" s="9" t="inlineStr">
+      <c r="L78" s="4" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M78" s="9" t="inlineStr">
+      <c r="M78" s="4" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N78" s="9" t="inlineStr">
+      <c r="N78" s="4" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O78" s="11" t="inlineStr">
-        <is>
-          <t>0M layout中，预计6/29 gerber out</t>
-        </is>
-      </c>
-      <c r="P78" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="O78" s="6" t="inlineStr">
+        <is>
+          <t>0A layout中</t>
+        </is>
+      </c>
+      <c r="P78" s="6" t="inlineStr">
+        <is>
+          <t>plan 7/3 gerber out，比預期 delay 4d,對後續schedule無影響</t>
         </is>
       </c>
     </row>
@@ -6497,12 +6505,12 @@
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>2654</t>
+          <t>2655</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>Raider 16  HX B4WI</t>
+          <t>Crosshair 16 Max HX E4WFK</t>
         </is>
       </c>
       <c r="D79" s="18" t="inlineStr">
@@ -6517,12 +6525,12 @@
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>RTX 5080</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>吳美芳</t>
+          <t>鮑佩佩</t>
         </is>
       </c>
       <c r="H79" s="9" t="inlineStr">
@@ -6562,90 +6570,90 @@
       </c>
       <c r="O79" s="11" t="inlineStr">
         <is>
-          <t>0M layout中，预计6/29 gerber out</t>
+          <t>0A layout中</t>
         </is>
       </c>
       <c r="P79" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="n">
+          <t>plan 7/3 gerber out，比預期 delay 4d,對後續schedule無影響</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" hidden="1" outlineLevel="1">
+      <c r="A80" s="7" t="n">
         <v>79</v>
       </c>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="B80" s="8" t="inlineStr">
         <is>
           <t>2655</t>
         </is>
       </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>Crosshair 16 Max HX E4WEK</t>
-        </is>
-      </c>
-      <c r="D80" s="14" t="inlineStr">
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>Crosshair 16 Max HX E4WGK</t>
+        </is>
+      </c>
+      <c r="D80" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="E80" s="4" t="inlineStr">
+      <c r="E80" s="9" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F80" s="4" t="inlineStr">
-        <is>
-          <t>RTX 5050</t>
-        </is>
-      </c>
-      <c r="G80" s="4" t="inlineStr">
+      <c r="F80" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G80" s="9" t="inlineStr">
         <is>
           <t>鮑佩佩</t>
         </is>
       </c>
-      <c r="H80" s="4" t="inlineStr">
+      <c r="H80" s="9" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I80" s="4" t="inlineStr">
+      <c r="I80" s="9" t="inlineStr">
         <is>
           <t>2026/07/27</t>
         </is>
       </c>
-      <c r="J80" s="4" t="inlineStr">
+      <c r="J80" s="9" t="inlineStr">
         <is>
           <t>2026/09/29</t>
         </is>
       </c>
-      <c r="K80" s="4" t="inlineStr">
+      <c r="K80" s="9" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L80" s="4" t="inlineStr">
+      <c r="L80" s="9" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M80" s="4" t="inlineStr">
+      <c r="M80" s="9" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N80" s="4" t="inlineStr">
+      <c r="N80" s="9" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O80" s="6" t="inlineStr">
-        <is>
-          <t>0A layout中</t>
-        </is>
-      </c>
-      <c r="P80" s="6" t="inlineStr">
+      <c r="O80" s="11" t="inlineStr">
+        <is>
+          <t>GN22-X6 8GB SKU,0A layout中</t>
+        </is>
+      </c>
+      <c r="P80" s="11" t="inlineStr">
         <is>
           <t>plan 7/3 gerber out，比預期 delay 4d,對後續schedule無影響</t>
         </is>
@@ -6662,7 +6670,7 @@
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 16 Max HX E4WFK</t>
+          <t>Crosshair 16 Max HX E4WGXK</t>
         </is>
       </c>
       <c r="D81" s="18" t="inlineStr">
@@ -6677,7 +6685,7 @@
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G81" s="9" t="inlineStr">
@@ -6722,7 +6730,7 @@
       </c>
       <c r="O81" s="11" t="inlineStr">
         <is>
-          <t>0A layout中</t>
+          <t>GN22-X6 12GB SKU, 0A layout中</t>
         </is>
       </c>
       <c r="P81" s="11" t="inlineStr">
@@ -6731,168 +6739,8 @@
         </is>
       </c>
     </row>
-    <row r="82" hidden="1" outlineLevel="1">
-      <c r="A82" s="7" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" s="8" t="inlineStr">
-        <is>
-          <t>2655</t>
-        </is>
-      </c>
-      <c r="C82" s="9" t="inlineStr">
-        <is>
-          <t>Crosshair 16 Max HX E4WGK</t>
-        </is>
-      </c>
-      <c r="D82" s="18" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E82" s="9" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F82" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070</t>
-        </is>
-      </c>
-      <c r="G82" s="9" t="inlineStr">
-        <is>
-          <t>鮑佩佩</t>
-        </is>
-      </c>
-      <c r="H82" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/19</t>
-        </is>
-      </c>
-      <c r="I82" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/27</t>
-        </is>
-      </c>
-      <c r="J82" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/29</t>
-        </is>
-      </c>
-      <c r="K82" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="L82" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/02</t>
-        </is>
-      </c>
-      <c r="M82" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/08</t>
-        </is>
-      </c>
-      <c r="N82" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/18</t>
-        </is>
-      </c>
-      <c r="O82" s="11" t="inlineStr">
-        <is>
-          <t>GN22-X6 8GB SKU,0A layout中</t>
-        </is>
-      </c>
-      <c r="P82" s="11" t="inlineStr">
-        <is>
-          <t>plan 7/3 gerber out，比預期 delay 4d,對後續schedule無影響</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" hidden="1" outlineLevel="1">
-      <c r="A83" s="7" t="n">
-        <v>82</v>
-      </c>
-      <c r="B83" s="8" t="inlineStr">
-        <is>
-          <t>2655</t>
-        </is>
-      </c>
-      <c r="C83" s="9" t="inlineStr">
-        <is>
-          <t>Crosshair 16 Max HX E4WGXK</t>
-        </is>
-      </c>
-      <c r="D83" s="18" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E83" s="9" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F83" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070</t>
-        </is>
-      </c>
-      <c r="G83" s="9" t="inlineStr">
-        <is>
-          <t>鮑佩佩</t>
-        </is>
-      </c>
-      <c r="H83" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/19</t>
-        </is>
-      </c>
-      <c r="I83" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/27</t>
-        </is>
-      </c>
-      <c r="J83" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/29</t>
-        </is>
-      </c>
-      <c r="K83" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="L83" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/02</t>
-        </is>
-      </c>
-      <c r="M83" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/08</t>
-        </is>
-      </c>
-      <c r="N83" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/18</t>
-        </is>
-      </c>
-      <c r="O83" s="11" t="inlineStr">
-        <is>
-          <t>GN22-X6 12GB SKU, 0A layout中</t>
-        </is>
-      </c>
-      <c r="P83" s="11" t="inlineStr">
-        <is>
-          <t>plan 7/3 gerber out，比預期 delay 4d,對後續schedule無影響</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:P83"/>
+  <autoFilter ref="A1:P81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update NPI Dashboard 2026-07-06 09:00
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -52,12 +52,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0000B0F0"/>
+      <color rgb="007030A0"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="007030A0"/>
+      <color rgb="0000B0F0"/>
       <sz val="10"/>
     </font>
     <font>
@@ -139,19 +139,19 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1509,9 +1509,9 @@
           <t>Cyborg 15 B2VEK</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -1743,7 +1743,7 @@
           <t>Venture 15 AI+ B3M</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -1819,7 +1819,7 @@
           <t>Katana 15 HX C14WEK</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -1895,7 +1895,7 @@
           <t>Katana 15 HX C14WFK</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -1971,7 +1971,7 @@
           <t>Katana 15 HX C14WGK</t>
         </is>
       </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2047,7 +2047,7 @@
           <t>Katana 15 HX C14WEOK</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2123,7 +2123,7 @@
           <t>Katana 15 HX C14WFOK</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2199,7 +2199,7 @@
           <t>Katana 15 HX C14WGOK</t>
         </is>
       </c>
-      <c r="D23" s="16" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2275,7 +2275,7 @@
           <t>Modern 14 LE J3M</t>
         </is>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="D24" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -2352,7 +2352,7 @@
           <t>Modern 16 LE J3M</t>
         </is>
       </c>
-      <c r="D25" s="17" t="inlineStr">
+      <c r="D25" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -2429,7 +2429,7 @@
           <t>Cyborg A15 Max C1PWE</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2482,7 +2482,7 @@
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
-          <t>HPT sku: 目前測試有AMD Graphics驅動無法安裝/TP沒功能/LAN 設備丢失等問題, 麻煩RD盡快釐清</t>
+          <t>HPT sku: 目前AMD Graphics驅動無法安裝/TP沒功能, 請RD儘速釐清</t>
         </is>
       </c>
       <c r="P26" s="6" t="inlineStr">
@@ -2507,7 +2507,7 @@
           <t>Cyborg A15 Max C1PWF</t>
         </is>
       </c>
-      <c r="D27" s="16" t="inlineStr">
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2560,7 +2560,7 @@
       </c>
       <c r="O27" s="11" t="inlineStr">
         <is>
-          <t>HPT sku: 目前測試有AMD Graphics驅動無法安裝/TP沒功能/LAN 設備丢失等問題, 麻煩RD盡快釐清</t>
+          <t>HPT sku: 目前AMD Graphics驅動無法安裝/TP沒功能, 請RD儘速釐清</t>
         </is>
       </c>
       <c r="P27" s="11" t="inlineStr">
@@ -2585,7 +2585,7 @@
           <t>Cyborg A15 Max C1PWG</t>
         </is>
       </c>
-      <c r="D28" s="16" t="inlineStr">
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2638,7 +2638,7 @@
       </c>
       <c r="O28" s="11" t="inlineStr">
         <is>
-          <t>HPT sku: 目前測試有AMD Graphics驅動無法安裝/TP沒功能/LAN 設備丢失等問題, 麻煩RD盡快釐清</t>
+          <t>HPT sku: 目前AMD Graphics驅動無法安裝/TP沒功能, 請RD儘速釐清</t>
         </is>
       </c>
       <c r="P28" s="11" t="inlineStr">
@@ -2663,7 +2663,7 @@
           <t>Cyborg A15 C1PWE</t>
         </is>
       </c>
-      <c r="D29" s="16" t="inlineStr">
+      <c r="D29" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="O29" s="11" t="inlineStr">
         <is>
-          <t>HPT sku: 目前測試有AMD Graphics驅動無法安裝/TP沒功能/LAN 設備丢失等問題, 麻煩RD盡快釐清</t>
+          <t>HPT sku: 目前AMD Graphics驅動無法安裝/TP沒功能, 請RD儘速釐清</t>
         </is>
       </c>
       <c r="P29" s="11" t="inlineStr">
@@ -2823,7 +2823,7 @@
           <t>Prestige N16 C1M</t>
         </is>
       </c>
-      <c r="D31" s="18" t="inlineStr">
+      <c r="D31" s="17" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -2904,7 +2904,7 @@
           <t>Katana 18 HX A14WEK</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2984,7 +2984,7 @@
           <t>Katana 18 HX A14WFK</t>
         </is>
       </c>
-      <c r="D33" s="16" t="inlineStr">
+      <c r="D33" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3064,7 +3064,7 @@
           <t>Katana 18 HX A14WGK</t>
         </is>
       </c>
-      <c r="D34" s="16" t="inlineStr">
+      <c r="D34" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3144,7 +3144,7 @@
           <t>Katana 18 HX A14WEOK</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr">
+      <c r="D35" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3220,7 +3220,7 @@
           <t>Katana 18 HX A14WFOK</t>
         </is>
       </c>
-      <c r="D36" s="16" t="inlineStr">
+      <c r="D36" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3296,7 +3296,7 @@
           <t>Katana 18 HX A14WGOK</t>
         </is>
       </c>
-      <c r="D37" s="16" t="inlineStr">
+      <c r="D37" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3372,7 +3372,7 @@
           <t>Crosshair 18 Max HX B14WEO</t>
         </is>
       </c>
-      <c r="D38" s="16" t="inlineStr">
+      <c r="D38" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3448,7 +3448,7 @@
           <t>Crosshair 18 Max HX B14WFO</t>
         </is>
       </c>
-      <c r="D39" s="16" t="inlineStr">
+      <c r="D39" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3524,7 +3524,7 @@
           <t>Crosshair 18 Max HX B14WGO</t>
         </is>
       </c>
-      <c r="D40" s="16" t="inlineStr">
+      <c r="D40" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3600,7 +3600,7 @@
           <t>Crosshair 18 Max HX B14WGXO</t>
         </is>
       </c>
-      <c r="D41" s="16" t="inlineStr">
+      <c r="D41" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3676,7 +3676,7 @@
           <t>Crosshair 18 Max HX B14WE</t>
         </is>
       </c>
-      <c r="D42" s="16" t="inlineStr">
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3756,7 +3756,7 @@
           <t>Crosshair 18 Max HX B14WF</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3836,7 +3836,7 @@
           <t>Crosshair 18 Max HX B14WG</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
+      <c r="D44" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3916,7 +3916,7 @@
           <t>Crosshair 18 Max HX B14WGX</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
+      <c r="D45" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3996,7 +3996,7 @@
           <t>Crosshair 18 Max HX B2WE</t>
         </is>
       </c>
-      <c r="D46" s="14" t="inlineStr">
+      <c r="D46" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4068,7 +4068,7 @@
           <t>Crosshair 18 Max HX B2WEO</t>
         </is>
       </c>
-      <c r="D47" s="14" t="inlineStr">
+      <c r="D47" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4140,7 +4140,7 @@
           <t>Crosshair 18 Max HX B2WF</t>
         </is>
       </c>
-      <c r="D48" s="14" t="inlineStr">
+      <c r="D48" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4212,7 +4212,7 @@
           <t>Crosshair 18 Max HX B2WFO</t>
         </is>
       </c>
-      <c r="D49" s="14" t="inlineStr">
+      <c r="D49" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4284,7 +4284,7 @@
           <t>Crosshair 18 Max HX B2WG</t>
         </is>
       </c>
-      <c r="D50" s="14" t="inlineStr">
+      <c r="D50" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4356,7 +4356,7 @@
           <t>Crosshair 18 Max HX B2WGO</t>
         </is>
       </c>
-      <c r="D51" s="14" t="inlineStr">
+      <c r="D51" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4428,7 +4428,7 @@
           <t>Crosshair 18 Max HX B2WGX</t>
         </is>
       </c>
-      <c r="D52" s="14" t="inlineStr">
+      <c r="D52" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4500,7 +4500,7 @@
           <t>Crosshair 18 Max HX B2WGXO</t>
         </is>
       </c>
-      <c r="D53" s="14" t="inlineStr">
+      <c r="D53" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4572,7 +4572,7 @@
           <t>Katana 18 HX A2WEK</t>
         </is>
       </c>
-      <c r="D54" s="14" t="inlineStr">
+      <c r="D54" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4644,7 +4644,7 @@
           <t>Katana 18 HX A2WEOK</t>
         </is>
       </c>
-      <c r="D55" s="14" t="inlineStr">
+      <c r="D55" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4720,7 +4720,7 @@
           <t>Katana 18 HX A2WFK</t>
         </is>
       </c>
-      <c r="D56" s="14" t="inlineStr">
+      <c r="D56" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4792,7 +4792,7 @@
           <t>Katana 18 HX A2WFOK</t>
         </is>
       </c>
-      <c r="D57" s="14" t="inlineStr">
+      <c r="D57" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4868,7 +4868,7 @@
           <t>Katana 18 HX A2WGK</t>
         </is>
       </c>
-      <c r="D58" s="14" t="inlineStr">
+      <c r="D58" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4940,7 +4940,7 @@
           <t>Katana 18 HX A2WGOK</t>
         </is>
       </c>
-      <c r="D59" s="14" t="inlineStr">
+      <c r="D59" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5016,7 +5016,7 @@
           <t>Prestige 14 AI</t>
         </is>
       </c>
-      <c r="D60" s="15" t="inlineStr">
+      <c r="D60" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -5096,7 +5096,7 @@
           <t>Prestige 14 AI+ Flip</t>
         </is>
       </c>
-      <c r="D61" s="16" t="inlineStr">
+      <c r="D61" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -5176,7 +5176,7 @@
           <t>Prestige 16 AI+</t>
         </is>
       </c>
-      <c r="D62" s="15" t="inlineStr">
+      <c r="D62" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -5252,9 +5252,9 @@
           <t>Prestige 16 Flip AI+</t>
         </is>
       </c>
-      <c r="D63" s="14" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
@@ -5305,7 +5305,7 @@
       </c>
       <c r="O63" s="11" t="inlineStr">
         <is>
-          <t>0A gerberout ：6/26,DVT SMT@7/22</t>
+          <t>DVT SMT@7/22</t>
         </is>
       </c>
       <c r="P63" s="11" t="inlineStr">
@@ -5328,7 +5328,7 @@
           <t>Prestige 13 AI+ A4M</t>
         </is>
       </c>
-      <c r="D64" s="17" t="inlineStr">
+      <c r="D64" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5408,7 +5408,7 @@
           <t>Stealth 16 AI+ B4WI</t>
         </is>
       </c>
-      <c r="D65" s="17" t="inlineStr">
+      <c r="D65" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5488,7 +5488,7 @@
           <t>Stealth 16 AI+ B4WH</t>
         </is>
       </c>
-      <c r="D66" s="14" t="inlineStr">
+      <c r="D66" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5568,7 +5568,7 @@
           <t>Stealth 16 AI+ B4WJ</t>
         </is>
       </c>
-      <c r="D67" s="14" t="inlineStr">
+      <c r="D67" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5648,7 +5648,7 @@
           <t>Stealth 16 AI+ B4WE</t>
         </is>
       </c>
-      <c r="D68" s="17" t="inlineStr">
+      <c r="D68" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5729,7 +5729,7 @@
           <t>Stealth 16 AI+ B4WF</t>
         </is>
       </c>
-      <c r="D69" s="14" t="inlineStr">
+      <c r="D69" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5810,7 +5810,7 @@
           <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
         </is>
       </c>
-      <c r="D70" s="14" t="inlineStr">
+      <c r="D70" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5891,7 +5891,7 @@
           <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
         </is>
       </c>
-      <c r="D71" s="14" t="inlineStr">
+      <c r="D71" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5972,7 +5972,7 @@
           <t>Raider 16 Max HX B4WH</t>
         </is>
       </c>
-      <c r="D72" s="15" t="inlineStr">
+      <c r="D72" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -6052,7 +6052,7 @@
           <t>Raider 16 Max HX B4WI</t>
         </is>
       </c>
-      <c r="D73" s="16" t="inlineStr">
+      <c r="D73" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -6132,7 +6132,7 @@
           <t>Raider 16 Max HX B4WJ</t>
         </is>
       </c>
-      <c r="D74" s="16" t="inlineStr">
+      <c r="D74" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -6212,7 +6212,7 @@
           <t>Raider 16  HX B4WH</t>
         </is>
       </c>
-      <c r="D75" s="16" t="inlineStr">
+      <c r="D75" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -6292,7 +6292,7 @@
           <t>Raider 16  HX B4WI</t>
         </is>
       </c>
-      <c r="D76" s="16" t="inlineStr">
+      <c r="D76" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -6372,9 +6372,9 @@
           <t>Crosshair 16 Max HX E4WEK</t>
         </is>
       </c>
-      <c r="D77" s="17" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D77" s="14" t="inlineStr">
+        <is>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
@@ -6452,9 +6452,9 @@
           <t>Crosshair 16 Max HX E4WFK</t>
         </is>
       </c>
-      <c r="D78" s="14" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D78" s="15" t="inlineStr">
+        <is>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
@@ -6532,9 +6532,9 @@
           <t>Crosshair 16 Max HX E4WGK</t>
         </is>
       </c>
-      <c r="D79" s="14" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D79" s="15" t="inlineStr">
+        <is>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
@@ -6612,9 +6612,9 @@
           <t>Crosshair 16 Max HX E4WGXK</t>
         </is>
       </c>
-      <c r="D80" s="14" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D80" s="15" t="inlineStr">
+        <is>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Update NPI Dashboard 2026-07-09 14:08
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPI Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -57,12 +57,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0000B0F0"/>
+      <color rgb="00ED7D31"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00ED7D31"/>
+      <color rgb="0000B0F0"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -148,10 +148,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -519,7 +519,7 @@
     <outlinePr summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P80"/>
+  <dimension ref="A1:P86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>RMB 100 35W</t>
+          <t>RMB 100 25W</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1333,17 +1333,18 @@
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>2026/07/10</t>
+          <t>2026/07/13</t>
         </is>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
-          <t>ATS 預計7/1 ASSY，客驗安排7/4 ，7/10 機台入庫</t>
+          <t>因D件缺料，ASSY 由7/1 推遲到7/5，機台入庫時間預計從7/10延後到7/13</t>
         </is>
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>1)	MVT Issue，Free DOS下，secure boor enable,不能從U盤啟動&amp;UCSI功能未導入 需微步協調人力加速，確保在7/8前導入對策，</t>
+          <t>1).Schedule delay 3天
+2).ATS  Issue 進版EC·QA客驗機台最快7/10提供·需QA協助Support三天驗完同步需要微步確保在7/10一早提供客驗機台</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1369,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>RMB 100 35W</t>
+          <t>RMB 100 28W</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -1409,17 +1410,17 @@
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>2026/07/13</t>
+          <t>2026/07/15</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
-          <t>因26VL 機構物料7/3 ready，預計7/4 ATS ASSY ，7/13 機台入庫</t>
+          <t>ATS Issue需進版EC，預計7/9 提供DQA客驗機台，</t>
         </is>
       </c>
       <c r="P12" s="6" t="inlineStr">
         <is>
-          <t>1)	MVT Issue，Free DOS下，secure boor enable,不能從U盤啟動&amp;UCSI功能未導入 需微步協調人力加速，確保在7/8前導入對策，</t>
+          <t>SChedule delay 2d：電池來料電池FW錯誤(規格要求1C·來料0.5C)需退料返工處理·機台入庫時間預計從7/13延後到7/15</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1487,7 @@
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
-          <t>（清白光鍵盤庫存）測試HDI預計7/3完成DQA開始驗證,測試預計２周時間</t>
+          <t>（清白光鍵盤庫存）DQA測試中,預計7/20完成</t>
         </is>
       </c>
       <c r="P13" s="6" t="inlineStr">
@@ -1554,7 +1555,7 @@
       </c>
       <c r="O14" s="11" t="inlineStr">
         <is>
-          <t>（清日文4區RGB鍵盤庫存）預計7/6 試組機台, DQA預計測試2周時間</t>
+          <t>（清日文4區RGB鍵盤庫存）DQA測試中,預計7/21完成</t>
         </is>
       </c>
       <c r="P14" s="11" t="inlineStr">
@@ -1796,12 +1797,12 @@
       </c>
       <c r="O17" s="6" t="inlineStr">
         <is>
-          <t>MVT備料中</t>
+          <t>MVT1 正式組裝@7/13</t>
         </is>
       </c>
       <c r="P17" s="6" t="inlineStr">
         <is>
-          <t>1) 組裝正式上線時間延後2天, MP時間暫不影響</t>
+          <t>1) w/FP的Touchpad 試產物料,需要採購協助Pull in</t>
         </is>
       </c>
     </row>
@@ -2275,9 +2276,9 @@
           <t>Modern 14 LE J3M</t>
         </is>
       </c>
-      <c r="D24" s="16" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -2302,7 +2303,7 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>2026/06/29</t>
+          <t>2026/07/07</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr"/>
@@ -2318,7 +2319,7 @@
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>2026/08/17</t>
+          <t>2026/08/18</t>
         </is>
       </c>
       <c r="N24" s="4" t="inlineStr">
@@ -2328,13 +2329,12 @@
       </c>
       <c r="O24" s="6" t="inlineStr">
         <is>
-          <t>Weibu update 7/6 ASSY--受新料交期和盤點影響</t>
+          <t>Weibu 7/7 ASSY, 7/10安排機器出貨for MSIK &amp; MSIT</t>
         </is>
       </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>1)Schedule: 考量新料備料時程, 調整試產和ATS時間@8/17 start
-2)認證: 參考Weibu認證Schedule, 有四個國家無法同步於8/E TTM, 持續追蹤中 MX: 11/28 ready；AR:10/3 ready；CO: 9/5 ready；RU: 9/12 ready</t>
+          <t>1)認證: 參考Weibu認證Schedule, a. 美洲US FCC 9/8 b.歐洲CE NB &amp;澳洲RCM 8/28 ready, 認證時間有風險, 已經highlight給微步team作認證評估</t>
         </is>
       </c>
     </row>
@@ -2352,9 +2352,9 @@
           <t>Modern 16 LE J3M</t>
         </is>
       </c>
-      <c r="D25" s="16" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>2026/06/29</t>
+          <t>2026/07/07</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr"/>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>2026/08/17</t>
+          <t>2026/08/18</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
@@ -2405,13 +2405,12 @@
       </c>
       <c r="O25" s="6" t="inlineStr">
         <is>
-          <t>Weibu update 7/6 ASSY--受新料交期和盤點影響</t>
+          <t>Weibu 7/7ASSY, 7/11安排機器出貨for MSIK&amp;MSIT</t>
         </is>
       </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>1)Schedule: 考量新料備料時程, 調整試產和ATS時間@8/17 start
-2)認證: 參考Weibu認證Schedule, 有四個國家無法同步於8/E TTM, 持續追蹤中 MX: 11/28 ready；AR:10/3 ready；CO: 9/5 ready；RU: 9/12 ready</t>
+          <t>1)認證: 參考Weibu認證Schedule, a. 美洲US FCC 9/8 b.歐洲CE NB &amp;澳洲RCM 8/28 ready, 認證時間有風險, 已經highlight給微步team作認證評估</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2777,7 @@
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>2026/07/20</t>
+          <t>2026/08/03</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
@@ -2798,12 +2797,12 @@
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
-          <t>MVT SMT@7/20--depend on Material ready date作調整</t>
+          <t>MVT SMT@8/3--depend on Material ready date作調整</t>
         </is>
       </c>
       <c r="P30" s="6" t="inlineStr">
         <is>
-          <t>1) Schedule: 因color plan變更, MVT機構件備料ready日期還待ID&amp;ME確認中, 待評估完成更新MVT ASSY date
+          <t>1) Schedule: MVT機構件備料ready日期預計8/7完成備料
 2）Color plan change: a. 顏色變更至炭黑色 b. D件改噴漆製程
 3)備料：量產交料HQ23, 十一月份交料(MSI wish 10/B交料, 待Samsung確認回復）</t>
         </is>
@@ -2823,7 +2822,7 @@
           <t>Prestige N16 C1M</t>
         </is>
       </c>
-      <c r="D31" s="17" t="inlineStr">
+      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -2860,7 +2859,7 @@
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>2026/07/20</t>
+          <t>2026/08/03</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
@@ -2880,8 +2879,7 @@
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
-          <t>1)EVT 更新BSP6.2.1  持續驗證中, 對應NV schedule 更新 MVT延到7/20.
-2) NV 更新BSP 時間 Factory Drop Final ETA 10/6 ,需要1周時間完成 HDI+BIOS 更新ATS strat 10/13</t>
+          <t>1)EVT 更新BSP6.2.1  持續驗證中, 因ID 顏色修改+機構修模 MVT 預計延後2周到8/3</t>
         </is>
       </c>
       <c r="P31" s="6" t="inlineStr">
@@ -2961,7 +2959,7 @@
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中</t>
+          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖</t>
         </is>
       </c>
       <c r="P32" s="6" t="inlineStr">
@@ -3041,7 +3039,7 @@
       </c>
       <c r="O33" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中</t>
+          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖</t>
         </is>
       </c>
       <c r="P33" s="11" t="inlineStr">
@@ -3121,7 +3119,7 @@
       </c>
       <c r="O34" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中</t>
+          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖</t>
         </is>
       </c>
       <c r="P34" s="11" t="inlineStr">
@@ -3197,7 +3195,7 @@
       </c>
       <c r="O35" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: DVT PCBA 7/2 調撥，預計7/6 RD領取測試</t>
+          <t>RPL-HX R + DDR4: DVT 7/6 RD領取測試</t>
         </is>
       </c>
       <c r="P35" s="11" t="inlineStr">
@@ -3273,7 +3271,7 @@
       </c>
       <c r="O36" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: DVT PCBA 7/2 調撥，預計7/6 RD領取測試</t>
+          <t>RPL-HX R + DDR4: DVT 7/6 RD領取測試</t>
         </is>
       </c>
       <c r="P36" s="11" t="inlineStr">
@@ -3349,7 +3347,7 @@
       </c>
       <c r="O37" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: DVT PCBA 7/2 調撥，預計7/6 RD領取測試</t>
+          <t>RPL-HX R + DDR4: DVT 7/6 RD領取測試</t>
         </is>
       </c>
       <c r="P37" s="11" t="inlineStr">
@@ -3425,7 +3423,7 @@
       </c>
       <c r="O38" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: DVT PCBA 7/2 調撥，預計7/6 RD領取測試</t>
+          <t>RPL-HX R + DDR4: DVT 7/6 RD領取測試</t>
         </is>
       </c>
       <c r="P38" s="11" t="inlineStr">
@@ -3501,7 +3499,7 @@
       </c>
       <c r="O39" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: DVT PCBA 7/2 調撥，預計7/6 RD領取測試</t>
+          <t>RPL-HX R + DDR4: DVT 7/6 RD領取測試</t>
         </is>
       </c>
       <c r="P39" s="11" t="inlineStr">
@@ -3577,7 +3575,7 @@
       </c>
       <c r="O40" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: DVT PCBA 7/2 調撥，預計7/6 RD領取測試</t>
+          <t>RPL-HX R + DDR4: DVT 7/6 RD領取測試</t>
         </is>
       </c>
       <c r="P40" s="11" t="inlineStr">
@@ -3653,7 +3651,7 @@
       </c>
       <c r="O41" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: DVT PCBA 7/2 調撥，預計7/6 RD領取測試</t>
+          <t>RPL-HX R + DDR4: DVT 7/6 RD領取測試</t>
         </is>
       </c>
       <c r="P41" s="11" t="inlineStr">
@@ -3733,7 +3731,7 @@
       </c>
       <c r="O42" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中</t>
+          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖</t>
         </is>
       </c>
       <c r="P42" s="11" t="inlineStr">
@@ -3813,7 +3811,7 @@
       </c>
       <c r="O43" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中</t>
+          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖</t>
         </is>
       </c>
       <c r="P43" s="11" t="inlineStr">
@@ -3893,7 +3891,7 @@
       </c>
       <c r="O44" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中</t>
+          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖</t>
         </is>
       </c>
       <c r="P44" s="11" t="inlineStr">
@@ -3973,7 +3971,7 @@
       </c>
       <c r="O45" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中</t>
+          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖</t>
         </is>
       </c>
       <c r="P45" s="11" t="inlineStr">
@@ -3996,7 +3994,7 @@
           <t>Crosshair 18 Max HX B2WE</t>
         </is>
       </c>
-      <c r="D46" s="18" t="inlineStr">
+      <c r="D46" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4068,7 +4066,7 @@
           <t>Crosshair 18 Max HX B2WEO</t>
         </is>
       </c>
-      <c r="D47" s="18" t="inlineStr">
+      <c r="D47" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4140,7 +4138,7 @@
           <t>Crosshair 18 Max HX B2WF</t>
         </is>
       </c>
-      <c r="D48" s="18" t="inlineStr">
+      <c r="D48" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4212,7 +4210,7 @@
           <t>Crosshair 18 Max HX B2WFO</t>
         </is>
       </c>
-      <c r="D49" s="18" t="inlineStr">
+      <c r="D49" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4284,7 +4282,7 @@
           <t>Crosshair 18 Max HX B2WG</t>
         </is>
       </c>
-      <c r="D50" s="18" t="inlineStr">
+      <c r="D50" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4356,7 +4354,7 @@
           <t>Crosshair 18 Max HX B2WGO</t>
         </is>
       </c>
-      <c r="D51" s="18" t="inlineStr">
+      <c r="D51" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4428,7 +4426,7 @@
           <t>Crosshair 18 Max HX B2WGX</t>
         </is>
       </c>
-      <c r="D52" s="18" t="inlineStr">
+      <c r="D52" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4500,7 +4498,7 @@
           <t>Crosshair 18 Max HX B2WGXO</t>
         </is>
       </c>
-      <c r="D53" s="18" t="inlineStr">
+      <c r="D53" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4572,7 +4570,7 @@
           <t>Katana 18 HX A2WEK</t>
         </is>
       </c>
-      <c r="D54" s="18" t="inlineStr">
+      <c r="D54" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4644,7 +4642,7 @@
           <t>Katana 18 HX A2WEOK</t>
         </is>
       </c>
-      <c r="D55" s="18" t="inlineStr">
+      <c r="D55" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4720,7 +4718,7 @@
           <t>Katana 18 HX A2WFK</t>
         </is>
       </c>
-      <c r="D56" s="18" t="inlineStr">
+      <c r="D56" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4792,7 +4790,7 @@
           <t>Katana 18 HX A2WFOK</t>
         </is>
       </c>
-      <c r="D57" s="18" t="inlineStr">
+      <c r="D57" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4868,7 +4866,7 @@
           <t>Katana 18 HX A2WGK</t>
         </is>
       </c>
-      <c r="D58" s="18" t="inlineStr">
+      <c r="D58" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4940,7 +4938,7 @@
           <t>Katana 18 HX A2WGOK</t>
         </is>
       </c>
-      <c r="D59" s="18" t="inlineStr">
+      <c r="D59" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5328,7 +5326,7 @@
           <t>Prestige 13 AI+ A4M</t>
         </is>
       </c>
-      <c r="D64" s="16" t="inlineStr">
+      <c r="D64" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5408,7 +5406,7 @@
           <t>Stealth 16 AI+ B4WI</t>
         </is>
       </c>
-      <c r="D65" s="16" t="inlineStr">
+      <c r="D65" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5488,7 +5486,7 @@
           <t>Stealth 16 AI+ B4WH</t>
         </is>
       </c>
-      <c r="D66" s="18" t="inlineStr">
+      <c r="D66" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5568,7 +5566,7 @@
           <t>Stealth 16 AI+ B4WJ</t>
         </is>
       </c>
-      <c r="D67" s="18" t="inlineStr">
+      <c r="D67" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5648,7 +5646,7 @@
           <t>Stealth 16 AI+ B4WE</t>
         </is>
       </c>
-      <c r="D68" s="16" t="inlineStr">
+      <c r="D68" s="18" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5665,7 +5663,7 @@
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>賴雪鳳</t>
+          <t>朱欣怡</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
@@ -5729,7 +5727,7 @@
           <t>Stealth 16 AI+ B4WF</t>
         </is>
       </c>
-      <c r="D69" s="18" t="inlineStr">
+      <c r="D69" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5746,7 +5744,7 @@
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>賴雪鳳</t>
+          <t>朱欣怡</t>
         </is>
       </c>
       <c r="H69" s="9" t="inlineStr">
@@ -5810,7 +5808,7 @@
           <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
         </is>
       </c>
-      <c r="D70" s="18" t="inlineStr">
+      <c r="D70" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5827,7 +5825,7 @@
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>賴雪鳳</t>
+          <t>朱欣怡</t>
         </is>
       </c>
       <c r="H70" s="9" t="inlineStr">
@@ -5891,7 +5889,7 @@
           <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
         </is>
       </c>
-      <c r="D71" s="18" t="inlineStr">
+      <c r="D71" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5908,7 +5906,7 @@
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>賴雪鳳</t>
+          <t>朱欣怡</t>
         </is>
       </c>
       <c r="H71" s="9" t="inlineStr">
@@ -6364,17 +6362,17 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>2655</t>
+          <t>1851</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Crosshair 16 Max HX E4WEK</t>
-        </is>
-      </c>
-      <c r="D77" s="14" t="inlineStr">
-        <is>
-          <t>DVT</t>
+          <t>Titan 18 HX B4WH</t>
+        </is>
+      </c>
+      <c r="D77" s="18" t="inlineStr">
+        <is>
+          <t>Design</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
@@ -6384,37 +6382,37 @@
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070Ti</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>鮑佩佩</t>
+          <t>高宇奇</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>2026/05/19</t>
+          <t>2026/06/29</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>2026/07/27</t>
+          <t>2026/08/14</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
-          <t>2026/09/29</t>
+          <t>2026/10/23</t>
         </is>
       </c>
       <c r="K77" s="4" t="inlineStr">
         <is>
-          <t>2027/01/11</t>
+          <t>2027/01/08</t>
         </is>
       </c>
       <c r="L77" s="4" t="inlineStr">
         <is>
-          <t>2027/02/02</t>
+          <t>2027/02/01</t>
         </is>
       </c>
       <c r="M77" s="4" t="inlineStr">
@@ -6429,14 +6427,10 @@
       </c>
       <c r="O77" s="6" t="inlineStr">
         <is>
-          <t>0A 7/3 gerber out</t>
-        </is>
-      </c>
-      <c r="P77" s="6" t="inlineStr">
-        <is>
-          <t>na</t>
-        </is>
-      </c>
+          <t>0M layout進行中,預計7/27 0M gerber out.</t>
+        </is>
+      </c>
+      <c r="P77" s="6" t="inlineStr"/>
     </row>
     <row r="78" hidden="1" outlineLevel="1">
       <c r="A78" s="7" t="n">
@@ -6444,17 +6438,17 @@
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>2655</t>
+          <t>1851</t>
         </is>
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 16 Max HX E4WFK</t>
-        </is>
-      </c>
-      <c r="D78" s="15" t="inlineStr">
-        <is>
-          <t>DVT</t>
+          <t>Titan 18 HX B4WI</t>
+        </is>
+      </c>
+      <c r="D78" s="17" t="inlineStr">
+        <is>
+          <t>Design</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
@@ -6464,37 +6458,37 @@
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5080</t>
         </is>
       </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>鮑佩佩</t>
+          <t>高宇奇</t>
         </is>
       </c>
       <c r="H78" s="9" t="inlineStr">
         <is>
-          <t>2026/05/19</t>
+          <t>2026/06/29</t>
         </is>
       </c>
       <c r="I78" s="9" t="inlineStr">
         <is>
-          <t>2026/07/27</t>
+          <t>2026/08/14</t>
         </is>
       </c>
       <c r="J78" s="9" t="inlineStr">
         <is>
-          <t>2026/09/29</t>
+          <t>2026/10/23</t>
         </is>
       </c>
       <c r="K78" s="9" t="inlineStr">
         <is>
-          <t>2027/01/11</t>
+          <t>2027/01/08</t>
         </is>
       </c>
       <c r="L78" s="9" t="inlineStr">
         <is>
-          <t>2027/02/02</t>
+          <t>2027/02/01</t>
         </is>
       </c>
       <c r="M78" s="9" t="inlineStr">
@@ -6509,14 +6503,10 @@
       </c>
       <c r="O78" s="11" t="inlineStr">
         <is>
-          <t>0A 7/3 gerber out</t>
-        </is>
-      </c>
-      <c r="P78" s="11" t="inlineStr">
-        <is>
-          <t>na</t>
-        </is>
-      </c>
+          <t>0M layout進行中,預計7/27 0M gerber out.</t>
+        </is>
+      </c>
+      <c r="P78" s="11" t="inlineStr"/>
     </row>
     <row r="79" hidden="1" outlineLevel="1">
       <c r="A79" s="7" t="n">
@@ -6524,17 +6514,17 @@
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>2655</t>
+          <t>1851</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 16 Max HX E4WGK</t>
-        </is>
-      </c>
-      <c r="D79" s="15" t="inlineStr">
-        <is>
-          <t>DVT</t>
+          <t>Titan 18 HX B4WJ</t>
+        </is>
+      </c>
+      <c r="D79" s="17" t="inlineStr">
+        <is>
+          <t>Design</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
@@ -6544,37 +6534,37 @@
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5090</t>
         </is>
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>鮑佩佩</t>
+          <t>高宇奇</t>
         </is>
       </c>
       <c r="H79" s="9" t="inlineStr">
         <is>
-          <t>2026/05/19</t>
+          <t>2026/06/29</t>
         </is>
       </c>
       <c r="I79" s="9" t="inlineStr">
         <is>
-          <t>2026/07/27</t>
+          <t>2026/08/14</t>
         </is>
       </c>
       <c r="J79" s="9" t="inlineStr">
         <is>
-          <t>2026/09/29</t>
+          <t>2026/10/23</t>
         </is>
       </c>
       <c r="K79" s="9" t="inlineStr">
         <is>
-          <t>2027/01/11</t>
+          <t>2027/01/08</t>
         </is>
       </c>
       <c r="L79" s="9" t="inlineStr">
         <is>
-          <t>2027/02/02</t>
+          <t>2027/02/01</t>
         </is>
       </c>
       <c r="M79" s="9" t="inlineStr">
@@ -6589,14 +6579,10 @@
       </c>
       <c r="O79" s="11" t="inlineStr">
         <is>
-          <t>GN22-X6 8GB SKU,0A 7/3 gerber out</t>
-        </is>
-      </c>
-      <c r="P79" s="11" t="inlineStr">
-        <is>
-          <t>na</t>
-        </is>
-      </c>
+          <t>0M layout進行中,預計7/27 0M gerber out.</t>
+        </is>
+      </c>
+      <c r="P79" s="11" t="inlineStr"/>
     </row>
     <row r="80" hidden="1" outlineLevel="1">
       <c r="A80" s="7" t="n">
@@ -6604,82 +6590,550 @@
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
+          <t>1851</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>Raider 18 Max HX B4WH</t>
+        </is>
+      </c>
+      <c r="D80" s="17" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 65W</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070Ti</t>
+        </is>
+      </c>
+      <c r="G80" s="9" t="inlineStr">
+        <is>
+          <t>高宇奇</t>
+        </is>
+      </c>
+      <c r="H80" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/29</t>
+        </is>
+      </c>
+      <c r="I80" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/14</t>
+        </is>
+      </c>
+      <c r="J80" s="9" t="inlineStr">
+        <is>
+          <t>2026/10/23</t>
+        </is>
+      </c>
+      <c r="K80" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/08</t>
+        </is>
+      </c>
+      <c r="L80" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/01</t>
+        </is>
+      </c>
+      <c r="M80" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N80" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O80" s="11" t="inlineStr">
+        <is>
+          <t>0M layout進行中,預計7/27 0M gerber out.</t>
+        </is>
+      </c>
+      <c r="P80" s="11" t="inlineStr"/>
+    </row>
+    <row r="81" hidden="1" outlineLevel="1">
+      <c r="A81" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>1851</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>Raider 18 Max HX B4WI</t>
+        </is>
+      </c>
+      <c r="D81" s="17" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 65W</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5080</t>
+        </is>
+      </c>
+      <c r="G81" s="9" t="inlineStr">
+        <is>
+          <t>高宇奇</t>
+        </is>
+      </c>
+      <c r="H81" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/29</t>
+        </is>
+      </c>
+      <c r="I81" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/14</t>
+        </is>
+      </c>
+      <c r="J81" s="9" t="inlineStr">
+        <is>
+          <t>2026/10/23</t>
+        </is>
+      </c>
+      <c r="K81" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/08</t>
+        </is>
+      </c>
+      <c r="L81" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/01</t>
+        </is>
+      </c>
+      <c r="M81" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N81" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O81" s="11" t="inlineStr">
+        <is>
+          <t>0M layout進行中,預計7/27 0M gerber out.</t>
+        </is>
+      </c>
+      <c r="P81" s="11" t="inlineStr"/>
+    </row>
+    <row r="82" hidden="1" outlineLevel="1">
+      <c r="A82" s="7" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>1851</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>Raider 18 Max HX B4WJ</t>
+        </is>
+      </c>
+      <c r="D82" s="17" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 65W</t>
+        </is>
+      </c>
+      <c r="F82" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5090</t>
+        </is>
+      </c>
+      <c r="G82" s="9" t="inlineStr">
+        <is>
+          <t>高宇奇</t>
+        </is>
+      </c>
+      <c r="H82" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/29</t>
+        </is>
+      </c>
+      <c r="I82" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/14</t>
+        </is>
+      </c>
+      <c r="J82" s="9" t="inlineStr">
+        <is>
+          <t>2026/10/23</t>
+        </is>
+      </c>
+      <c r="K82" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/08</t>
+        </is>
+      </c>
+      <c r="L82" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/01</t>
+        </is>
+      </c>
+      <c r="M82" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N82" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O82" s="11" t="inlineStr">
+        <is>
+          <t>0M layout進行中,預計7/27 0M gerber out.</t>
+        </is>
+      </c>
+      <c r="P82" s="11" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
           <t>2655</t>
         </is>
       </c>
-      <c r="C80" s="9" t="inlineStr">
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Crosshair 16 Max HX E4WEK</t>
+        </is>
+      </c>
+      <c r="D83" s="14" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>RTX 5050</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>鮑佩佩</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>2026/05/19</t>
+        </is>
+      </c>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>2026/07/27</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/29</t>
+        </is>
+      </c>
+      <c r="K83" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="L83" s="4" t="inlineStr">
+        <is>
+          <t>2027/02/02</t>
+        </is>
+      </c>
+      <c r="M83" s="4" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N83" s="4" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O83" s="6" t="inlineStr">
+        <is>
+          <t>0A 7/3 gerber out.plan 7/27 DVT SMT1</t>
+        </is>
+      </c>
+      <c r="P83" s="6" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" hidden="1" outlineLevel="1">
+      <c r="A84" s="7" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>2655</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="inlineStr">
+        <is>
+          <t>Crosshair 16 Max HX E4WFK</t>
+        </is>
+      </c>
+      <c r="D84" s="15" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E84" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F84" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5060</t>
+        </is>
+      </c>
+      <c r="G84" s="9" t="inlineStr">
+        <is>
+          <t>鮑佩佩</t>
+        </is>
+      </c>
+      <c r="H84" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/19</t>
+        </is>
+      </c>
+      <c r="I84" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/27</t>
+        </is>
+      </c>
+      <c r="J84" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/29</t>
+        </is>
+      </c>
+      <c r="K84" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="L84" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/02</t>
+        </is>
+      </c>
+      <c r="M84" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N84" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O84" s="11" t="inlineStr">
+        <is>
+          <t>0A 7/3 gerber out.plan 7/27 DVT SMT1</t>
+        </is>
+      </c>
+      <c r="P84" s="11" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" hidden="1" outlineLevel="1">
+      <c r="A85" s="7" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>2655</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>Crosshair 16 Max HX E4WGK</t>
+        </is>
+      </c>
+      <c r="D85" s="15" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F85" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G85" s="9" t="inlineStr">
+        <is>
+          <t>鮑佩佩</t>
+        </is>
+      </c>
+      <c r="H85" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/19</t>
+        </is>
+      </c>
+      <c r="I85" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/27</t>
+        </is>
+      </c>
+      <c r="J85" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/29</t>
+        </is>
+      </c>
+      <c r="K85" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="L85" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/02</t>
+        </is>
+      </c>
+      <c r="M85" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N85" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O85" s="11" t="inlineStr">
+        <is>
+          <t>0A 7/3 gerber out.plan 7/27 DVT SMT1</t>
+        </is>
+      </c>
+      <c r="P85" s="11" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" hidden="1" outlineLevel="1">
+      <c r="A86" s="7" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>2655</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="inlineStr">
         <is>
           <t>Crosshair 16 Max HX E4WGXK</t>
         </is>
       </c>
-      <c r="D80" s="15" t="inlineStr">
+      <c r="D86" s="15" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E80" s="9" t="inlineStr">
+      <c r="E86" s="9" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F80" s="9" t="inlineStr">
+      <c r="F86" s="9" t="inlineStr">
         <is>
           <t>RTX 5070</t>
         </is>
       </c>
-      <c r="G80" s="9" t="inlineStr">
+      <c r="G86" s="9" t="inlineStr">
         <is>
           <t>鮑佩佩</t>
         </is>
       </c>
-      <c r="H80" s="9" t="inlineStr">
+      <c r="H86" s="9" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I80" s="9" t="inlineStr">
+      <c r="I86" s="9" t="inlineStr">
         <is>
           <t>2026/07/27</t>
         </is>
       </c>
-      <c r="J80" s="9" t="inlineStr">
+      <c r="J86" s="9" t="inlineStr">
         <is>
           <t>2026/09/29</t>
         </is>
       </c>
-      <c r="K80" s="9" t="inlineStr">
+      <c r="K86" s="9" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L80" s="9" t="inlineStr">
+      <c r="L86" s="9" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M80" s="9" t="inlineStr">
+      <c r="M86" s="9" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N80" s="9" t="inlineStr">
+      <c r="N86" s="9" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O80" s="11" t="inlineStr">
-        <is>
-          <t>GN22-X6 12GB SKU,0A 7/3 gerber out</t>
-        </is>
-      </c>
-      <c r="P80" s="11" t="inlineStr">
+      <c r="O86" s="11" t="inlineStr">
+        <is>
+          <t>0A 7/3 gerber out.plan 7/27 DVT SMT1</t>
+        </is>
+      </c>
+      <c r="P86" s="11" t="inlineStr">
         <is>
           <t>na</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P80"/>
+  <autoFilter ref="A1:P86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update NPI Dashboard 2026-07-13 08:25
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -682,12 +682,12 @@
       </c>
       <c r="O2" s="6" t="inlineStr">
         <is>
-          <t>因首批安排RPL-U Refresh 優先投產，第二波投產因PCB 最快交期落在6/29,加上微步盤點，預計最快7/10 TTM</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="P2" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>因首批安排RPL-U Refresh 優先投產，第二波投產因PCB 最快交期落在6/29,加上微步盤點，機台7/9 入庫</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Crosshair A16 HX E9WEK</t>
+          <t>Crosshair A16 HX E9WGXK</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -865,12 +865,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>FRG-HX 55W</t>
+          <t>FRG-HX3D 55W</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1）暫無業務報價，BTO 未開</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Crosshair A16 HX E9WFK</t>
+          <t>Crosshair A16 HX E9WEK</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Crosshair A16 HX E9WGXK</t>
+          <t>Crosshair A16 HX E9WFK</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -1009,12 +1009,12 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>FRG-HX3D 55W</t>
+          <t>FRG-HX 55W</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -2438,9 +2438,9 @@
       </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>1) Schedule: MVT機構件備料ready日期預計8/7完成備料
-2）Color plan change: a. 顏色變更至炭黑色 b. D件改噴漆製程
-3)備料：量產交料HQ23, 十一月份交料(MSI wish 10/B交料, 待Samsung確認回復）</t>
+          <t>1) Schedule: MVT D件備料ready日期待採購/ME確認中
+2）Color plan: 維持開案版本
+3)備料：量產交料HQ23, 十月份交料, 待Samsung確認具體日期</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NPI Dashboard 2026-07-30 15:15
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -93,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -135,6 +135,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -670,12 +673,12 @@
       </c>
       <c r="O2" s="6" t="inlineStr">
         <is>
-          <t>（清日文4區RGB鍵盤庫存）DQA測試中,預計7/21完成</t>
+          <t>（清日文4區RGB鍵盤庫存)</t>
         </is>
       </c>
       <c r="P2" s="6" t="inlineStr">
         <is>
-          <t>1)DQA驗證有Audio問題, WHQL驅動預計7/24提供,需要Preload和DQA等單位加班驗證,滿足業務7/30出貨需求</t>
+          <t>1)方向鍵上的快捷鍵無功能, EC和BIOS需要進版, 請DQA協助快掃測試</t>
         </is>
       </c>
     </row>
@@ -742,12 +745,12 @@
       </c>
       <c r="O3" s="11" t="inlineStr">
         <is>
-          <t>（清白光鍵盤庫存）DQA測試中,預計7/20完成</t>
+          <t>（清白光鍵盤庫存）ATS C/R驗證中</t>
         </is>
       </c>
       <c r="P3" s="11" t="inlineStr">
         <is>
-          <t>1)DQA驗證有Audio問題, WHQL驅動預計7/24提供,需要Preload和DQA等單位加班驗證</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -814,9 +817,7 @@
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
-          <t>DQA test中,
-1) ME: 搖擺測試pass
-2）Function：待新版MSI Center AP release( 包入MKT name支援AI Noise Cancellation Pro), 安排HDI製作</t>
+          <t>DQA MP HDI測試進行中, 暫無量產工單產生</t>
         </is>
       </c>
       <c r="P4" s="6" t="inlineStr">
@@ -878,19 +879,17 @@
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/07</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>2026/08/07</t>
+          <t>2026/08/12</t>
         </is>
       </c>
       <c r="O5" s="11" t="inlineStr">
         <is>
-          <t>DQA test中,
-1) ME: 搖擺測試pass
-2）Function：最新版MSI Center AP聯網會支援noise Cancellation Pro, 待安排HDI製作</t>
+          <t>ATS C/R工單： 9S7-15Q373-1258* 50 pcs 預排8/7 ASSY</t>
         </is>
       </c>
       <c r="P5" s="11" t="inlineStr">
@@ -962,9 +961,7 @@
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
-          <t>DQA test中,
-1) ME: 搖擺測試pass
-2）Function：待新版MSI Center AP release( 包入MKT name支援AI Noise Cancellation Pro), 安排HDI製作</t>
+          <t>DQA MP HDI測試進行中, 暫無量產工單產生</t>
         </is>
       </c>
       <c r="P6" s="6" t="inlineStr">
@@ -1026,19 +1023,17 @@
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/07</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>2026/08/07</t>
+          <t>2026/08/12</t>
         </is>
       </c>
       <c r="O7" s="11" t="inlineStr">
         <is>
-          <t>DQA test中,
-1) ME: 搖擺測試pass
-2）Function：待新版MSI Center AP release( 包入MKT name支援AI Noise Cancellation Pro), 安排HDI製作</t>
+          <t>ATS C/R工單： 9S7-17U344-449 * 50 pcs 預排8/7 ASSY</t>
         </is>
       </c>
       <c r="P7" s="11" t="inlineStr">
@@ -1100,19 +1095,17 @@
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/08</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>2026/08/07</t>
+          <t>2026/08/12</t>
         </is>
       </c>
       <c r="O8" s="11" t="inlineStr">
         <is>
-          <t>DQA test中,
-1) ME: 搖擺測試pass
-2）Function：待新版MSI Center AP release( 包入MKT name支援AI Noise Cancellation Pro), 安排HDI製作</t>
+          <t>9S7-17U344-441 * 300pcs ASSY @ 8/8</t>
         </is>
       </c>
       <c r="P8" s="11" t="inlineStr">
@@ -1135,9 +1128,9 @@
           <t>Venture 15 AI+ B3M</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -1188,12 +1181,13 @@
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
-          <t>MVT2 組裝@7/27</t>
+          <t>MVT2驗證中</t>
         </is>
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>1) ATS與MP的物料簽樣與備料,需要RD與採購和物管協助</t>
+          <t>1) ATS與MP的物料簽樣與備料,需要RD與採購和物管協助
+2)A件交期依森田薄膜進料時間,15T2 ATS組裝在8/20, MP在8/30, 會比原時程晚2天,會導致15T2無法meet 8/27 MP的目標,需要RD/採購協助pull in</t>
         </is>
       </c>
     </row>
@@ -1269,8 +1263,7 @@
       </c>
       <c r="P10" s="6" t="inlineStr">
         <is>
-          <t>(
-1) ATS與MP的物料簽樣與備料,需要RD與採購和物管協助</t>
+          <t>1).Materiel: #A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/E MP的目標,麻煩RD/採購pull in森田薄膜進料時間. #因7/28需量產備料四區鍵盤,如果還有鍵盤相關問題,請儘速提出</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1339,7 @@
       </c>
       <c r="P11" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1).Materiel: #A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/E MP的目標,麻煩RD/採購pull in森田薄膜進料時間. #因7/28需量產備料四區鍵盤,如果還有鍵盤相關問題,請儘速提出</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1415,7 @@
       </c>
       <c r="P12" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1).Materiel: #A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/E MP的目標,麻煩RD/採購pull in森田薄膜進料時間. #因7/28需量產備料四區鍵盤,如果還有鍵盤相關問題,請儘速提出</t>
         </is>
       </c>
     </row>
@@ -1493,12 +1486,13 @@
       </c>
       <c r="O13" s="11" t="inlineStr">
         <is>
-          <t>DDR4 sku, 7/24 MVT SMT, 預計7/27試組, 7/29組裝</t>
+          <t>DDR4 sku,MVT組裝中,預計8/4拿到機器開始測試,8/7 PCB risk buy</t>
         </is>
       </c>
       <c r="P13" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1) ATS與MP的物料簽樣與備料,需要RD與採購和物管協助
+2)A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/30 MP的目標,需要RD/採購協助助pull in</t>
         </is>
       </c>
     </row>
@@ -1569,12 +1563,13 @@
       </c>
       <c r="O14" s="11" t="inlineStr">
         <is>
-          <t>DDR4 sku, 7/24 MVT SMT, 預計7/27試組, 7/29組裝</t>
+          <t>DDR4 sku,MVT組裝中,預計8/4拿到機器開始測試,8/7 PCB risk buy</t>
         </is>
       </c>
       <c r="P14" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1) ATS與MP的物料簽樣與備料,需要RD與採購和物管協助
+2)A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/30 MP的目標,需要RD/採購協助助pull in</t>
         </is>
       </c>
     </row>
@@ -1645,12 +1640,12 @@
       </c>
       <c r="O15" s="11" t="inlineStr">
         <is>
-          <t>DDR4 sku, 7/24 MVT SMT, 預計7/27試組, 7/29組裝</t>
+          <t>DDR4 sku,MVT組裝中,預計8/4拿到機器開始測試,8/7 PCB risk buy</t>
         </is>
       </c>
       <c r="P15" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1).Materiel: #A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/E MP的目標,麻煩RD/採購pull in森田薄膜進料時間.</t>
         </is>
       </c>
     </row>
@@ -1729,6 +1724,89 @@
         </is>
       </c>
       <c r="P16" s="6" t="inlineStr">
+        <is>
+          <t>1)Battery life: 2.8K panel+day0 rev.B+balance mode測試，Web browersing測試達716min，接近過關。NV更新會導入部分省電作法於Rev. C，待更新SW後驗證。
+2)NV Abnormal shut down 的solution，經DQA於BSP Day0 rev.B驗證後，未發生除error code "0x7E"外的ABS現象，後續會持續觀察。
+3) Day0 rev.C BIOS 7/29 release，測試image預計7/30 release，工廠/DQA將同時切換測試。
+4)工廠用MP樣品測試，反應主要問題，需RD一起分析 1.Long run自動測試 S3/S4/S5/ Reboot/ FSU進系統在login 画面持续转圈宕機，黑屏無顯 ,宕機 2. LCD 花屏（panel 有黑線) 3. camera 開啟錄像后 camera APP 卡住</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" hidden="1" outlineLevel="1">
+      <c r="A17" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>2621</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Prestige N16 Flip AI+ C1XMT</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>N1x 80W</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>林晉弘</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>2024/11/25</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>2025/01/20</t>
+        </is>
+      </c>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>2025/06/25</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="inlineStr">
+        <is>
+          <t>2026/03/12</t>
+        </is>
+      </c>
+      <c r="L17" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/30</t>
+        </is>
+      </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/17</t>
+        </is>
+      </c>
+      <c r="N17" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/31</t>
+        </is>
+      </c>
+      <c r="O17" s="11" t="inlineStr">
+        <is>
+          <t>MVT測試中</t>
+        </is>
+      </c>
+      <c r="P17" s="11" t="inlineStr">
         <is>
           <t>1)Battery life: 以2.8K panel+day0 rev.A環境用balance mode測試，Modern standby可達標準，Web browersing尚差0.2Hr，將於BSP Day0 rev.B再進行驗證。
 2)NV Abnormal shut down 的solution，確認需於BSP Day0 rev.B驗證，預計7/23 image完成後，DQA/工廠會同時切換驗證確認。
@@ -1737,89 +1815,6 @@
         </is>
       </c>
     </row>
-    <row r="17" hidden="1" outlineLevel="1">
-      <c r="A17" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>2621</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Prestige N16 Flip AI+ C1XMT</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>MVT</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>N1x 80W</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>林晉弘</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>2024/11/25</t>
-        </is>
-      </c>
-      <c r="I17" s="9" t="inlineStr">
-        <is>
-          <t>2025/01/20</t>
-        </is>
-      </c>
-      <c r="J17" s="9" t="inlineStr">
-        <is>
-          <t>2025/06/25</t>
-        </is>
-      </c>
-      <c r="K17" s="9" t="inlineStr">
-        <is>
-          <t>2026/03/12</t>
-        </is>
-      </c>
-      <c r="L17" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/30</t>
-        </is>
-      </c>
-      <c r="M17" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/17</t>
-        </is>
-      </c>
-      <c r="N17" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/31</t>
-        </is>
-      </c>
-      <c r="O17" s="11" t="inlineStr">
-        <is>
-          <t>MVT測試中</t>
-        </is>
-      </c>
-      <c r="P17" s="11" t="inlineStr">
-        <is>
-          <t>1)Battery life: 以2.8K panel+day0 rev.A環境用balance mode測試，Modern standby可達標準，Web browersing尚差0.2Hr，將於BSP Day0 rev.B再進行驗證。
-2)NV Abnormal shut down 的solution，確認需於BSP Day0 rev.B驗證，預計7/23 image完成後，DQA/工廠會同時切換驗證確認。
-3)NV更新可for出貨的 GPU driver提前於8/3美國時間release，後須計畫以此版本進行測試並出貨，不影響現行Schedule，ATS仍定於8/17開始
-4)for NV/MSFT 113pcs樣品，已於7/17 SMT，7/22 ASS'Y，並通知業務轉單，預計下周可出貨</t>
-        </is>
-      </c>
-    </row>
     <row r="18">
       <c r="A18" s="2" t="n">
         <v>17</v>
@@ -1834,9 +1829,9 @@
           <t>Modern 14 LE J3M</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1887,13 +1882,14 @@
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
-          <t>MSIK: DQA test中; Weibu: plan MVT 7/29 SMT, 確認料況中</t>
+          <t>Weibu: MVT 7/30 ASSY中</t>
         </is>
       </c>
       <c r="P18" s="6" t="inlineStr">
         <is>
           <t>1)認證：8/E ready可出貨地區:  DE/UK/TR/BNX/NEU/SEE/FR/ES/PL/CZ/CIS/IT/JP/AU
-2）認證 8/E無法同步ready地區:  9/8 ready: LA/CA/ AR/CL  9/18 ready: UA 10/2 ready: CO/RU 12/18 ready: MX</t>
+2）認證 8/E無法同步ready地區:  9/8 ready: LA/CA/ AR/CL  9/18 ready: UA 10/2 ready: CO/RU 12/18 ready: MX
+2）備料: 日文鍵芯開放時程待追蹤</t>
         </is>
       </c>
     </row>
@@ -1911,9 +1907,9 @@
           <t>Modern 16 LE J3M</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1964,7 +1960,7 @@
       </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
-          <t>MSIK: DQA test中; Weibu: plan MVT 7/29 SMT, 確認料況中</t>
+          <t>Weibu: 7/30 MVT ASSY</t>
         </is>
       </c>
       <c r="P19" s="6" t="inlineStr">
@@ -2333,7 +2329,7 @@
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/13</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
@@ -2353,13 +2349,13 @@
       </c>
       <c r="O24" s="6" t="inlineStr">
         <is>
-          <t>MVT SMT@8/3--depend on Material ready date作調整</t>
+          <t>MVT SMT@8/13--depend on PS chip &amp; Software時間作調整</t>
         </is>
       </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>1) Schedule: a.MVT D件備料ready日期@7/29 b. CPU交期還未放行, 先預估8/B交期
-3)備料：量產交料HQ23, 最新交期回復在12月份（follow leading customer）交料, 還在持續追蹤中</t>
+          <t>1) Schedule:  本週CPU交期還未放行, 綜合PS software時間, 先預抓8/13 MVT start.
+2)備料：量產交料2.8k HQ23, 最新MP*1K交期回復在12/M（follow leading customer）交料, 與ATS start Gap 2個月, 採購協助push廠商交期中</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2410,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/13</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
@@ -2434,8 +2430,7 @@
       </c>
       <c r="O25" s="6" t="inlineStr">
         <is>
-          <t>1)EVT 更新BSP6.2.1  持續驗證中,ID定案 顏色keep 淺灰+ D side 咬花
-3) N1 SoC 出貨延遲 MVT 預計延到8/3 SMT, 8/4 Pre-Assy ,8/6 Assy</t>
+          <t>N1 SoC 出貨延遲 MVT 預計延到8/13 SMT</t>
         </is>
       </c>
       <c r="P25" s="6" t="inlineStr">
@@ -2458,9 +2453,9 @@
           <t>Katana 18 HX A14WEK</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>EVT</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -2490,7 +2485,7 @@
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>2026/08/24</t>
+          <t>2026/08/12</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
@@ -2515,7 +2510,7 @@
       </c>
       <c r="O26" s="6" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
+          <t>RPL-HX R + DDR5: 7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
         </is>
       </c>
       <c r="P26" s="6" t="inlineStr">
@@ -2538,9 +2533,9 @@
           <t>Katana 18 HX A14WFK</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>EVT</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
@@ -2570,7 +2565,7 @@
       </c>
       <c r="J27" s="9" t="inlineStr">
         <is>
-          <t>2026/08/24</t>
+          <t>2026/08/12</t>
         </is>
       </c>
       <c r="K27" s="9" t="inlineStr">
@@ -2595,7 +2590,7 @@
       </c>
       <c r="O27" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
+          <t>RPL-HX R + DDR5: 7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
         </is>
       </c>
       <c r="P27" s="11" t="inlineStr">
@@ -2618,9 +2613,9 @@
           <t>Katana 18 HX A14WGK</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>EVT</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -2650,7 +2645,7 @@
       </c>
       <c r="J28" s="9" t="inlineStr">
         <is>
-          <t>2026/08/24</t>
+          <t>2026/08/12</t>
         </is>
       </c>
       <c r="K28" s="9" t="inlineStr">
@@ -2675,7 +2670,7 @@
       </c>
       <c r="O28" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
+          <t>RPL-HX R + DDR5: 7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
         </is>
       </c>
       <c r="P28" s="11" t="inlineStr">
@@ -3230,9 +3225,9 @@
           <t>Crosshair 18 Max HX B14WE</t>
         </is>
       </c>
-      <c r="D36" s="13" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>EVT</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
@@ -3262,7 +3257,7 @@
       </c>
       <c r="J36" s="9" t="inlineStr">
         <is>
-          <t>2026/08/24</t>
+          <t>2026/08/12</t>
         </is>
       </c>
       <c r="K36" s="9" t="inlineStr">
@@ -3287,7 +3282,7 @@
       </c>
       <c r="O36" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
+          <t>RPL-HX R + DDR5: 7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
         </is>
       </c>
       <c r="P36" s="11" t="inlineStr">
@@ -3310,9 +3305,9 @@
           <t>Crosshair 18 Max HX B14WF</t>
         </is>
       </c>
-      <c r="D37" s="13" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>EVT</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
@@ -3342,7 +3337,7 @@
       </c>
       <c r="J37" s="9" t="inlineStr">
         <is>
-          <t>2026/08/24</t>
+          <t>2026/08/12</t>
         </is>
       </c>
       <c r="K37" s="9" t="inlineStr">
@@ -3367,7 +3362,7 @@
       </c>
       <c r="O37" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
+          <t>RPL-HX R + DDR5: 7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
         </is>
       </c>
       <c r="P37" s="11" t="inlineStr">
@@ -3390,9 +3385,9 @@
           <t>Crosshair 18 Max HX B14WG</t>
         </is>
       </c>
-      <c r="D38" s="13" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>EVT</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3422,7 +3417,7 @@
       </c>
       <c r="J38" s="9" t="inlineStr">
         <is>
-          <t>2026/08/24</t>
+          <t>2026/08/12</t>
         </is>
       </c>
       <c r="K38" s="9" t="inlineStr">
@@ -3447,7 +3442,7 @@
       </c>
       <c r="O38" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
+          <t>RPL-HX R + DDR5: 7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
         </is>
       </c>
       <c r="P38" s="11" t="inlineStr">
@@ -3470,9 +3465,9 @@
           <t>Crosshair 18 Max HX B14WGX</t>
         </is>
       </c>
-      <c r="D39" s="13" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>EVT</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
@@ -3502,7 +3497,7 @@
       </c>
       <c r="J39" s="9" t="inlineStr">
         <is>
-          <t>2026/08/24</t>
+          <t>2026/08/12</t>
         </is>
       </c>
       <c r="K39" s="9" t="inlineStr">
@@ -3527,7 +3522,7 @@
       </c>
       <c r="O39" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: DVT 測試中,預計7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
+          <t>RPL-HX R + DDR5: 7/28 0B出圖, SMT1 @ 8/12 SMT2 @ 8/24 for ASSY</t>
         </is>
       </c>
       <c r="P39" s="11" t="inlineStr">
@@ -3550,7 +3545,7 @@
           <t>Crosshair 18 Max HX B2WE</t>
         </is>
       </c>
-      <c r="D40" s="15" t="inlineStr">
+      <c r="D40" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3622,7 +3617,7 @@
           <t>Crosshair 18 Max HX B2WEO</t>
         </is>
       </c>
-      <c r="D41" s="15" t="inlineStr">
+      <c r="D41" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3694,7 +3689,7 @@
           <t>Crosshair 18 Max HX B2WF</t>
         </is>
       </c>
-      <c r="D42" s="15" t="inlineStr">
+      <c r="D42" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3766,7 +3761,7 @@
           <t>Crosshair 18 Max HX B2WFO</t>
         </is>
       </c>
-      <c r="D43" s="15" t="inlineStr">
+      <c r="D43" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3838,7 +3833,7 @@
           <t>Crosshair 18 Max HX B2WG</t>
         </is>
       </c>
-      <c r="D44" s="15" t="inlineStr">
+      <c r="D44" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3910,7 +3905,7 @@
           <t>Crosshair 18 Max HX B2WGO</t>
         </is>
       </c>
-      <c r="D45" s="15" t="inlineStr">
+      <c r="D45" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3982,7 +3977,7 @@
           <t>Crosshair 18 Max HX B2WGX</t>
         </is>
       </c>
-      <c r="D46" s="15" t="inlineStr">
+      <c r="D46" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4054,7 +4049,7 @@
           <t>Crosshair 18 Max HX B2WGXO</t>
         </is>
       </c>
-      <c r="D47" s="15" t="inlineStr">
+      <c r="D47" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4126,7 +4121,7 @@
           <t>Katana 18 HX A2WEK</t>
         </is>
       </c>
-      <c r="D48" s="15" t="inlineStr">
+      <c r="D48" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4198,7 +4193,7 @@
           <t>Katana 18 HX A2WEOK</t>
         </is>
       </c>
-      <c r="D49" s="15" t="inlineStr">
+      <c r="D49" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4274,7 +4269,7 @@
           <t>Katana 18 HX A2WFK</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4346,7 +4341,7 @@
           <t>Katana 18 HX A2WFOK</t>
         </is>
       </c>
-      <c r="D51" s="15" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4422,7 +4417,7 @@
           <t>Katana 18 HX A2WGK</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
+      <c r="D52" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4494,7 +4489,7 @@
           <t>Katana 18 HX A2WGOK</t>
         </is>
       </c>
-      <c r="D53" s="15" t="inlineStr">
+      <c r="D53" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4627,7 +4622,7 @@
       </c>
       <c r="O54" s="6" t="inlineStr">
         <is>
-          <t>DVT SMT@7/27</t>
+          <t>DVT 開機OK， RD test :8/4~8/31</t>
         </is>
       </c>
       <c r="P54" s="6" t="inlineStr">
@@ -4707,7 +4702,7 @@
       </c>
       <c r="O55" s="11" t="inlineStr">
         <is>
-          <t>DVT SMT@7/27</t>
+          <t>DVT 開機OK， RD test :8/4~8/31</t>
         </is>
       </c>
       <c r="P55" s="11" t="inlineStr">
@@ -4783,7 +4778,7 @@
       </c>
       <c r="O56" s="6" t="inlineStr">
         <is>
-          <t>DVT SMT@7/27</t>
+          <t>DVT 開機OK， RD test :8/4~8/31</t>
         </is>
       </c>
       <c r="P56" s="6" t="inlineStr">
@@ -4859,7 +4854,7 @@
       </c>
       <c r="O57" s="11" t="inlineStr">
         <is>
-          <t>DVT SMT@7/27</t>
+          <t>DVT 開機OK， RD test :8/4~8/31</t>
         </is>
       </c>
       <c r="P57" s="11" t="inlineStr">
@@ -4882,7 +4877,7 @@
           <t>Prestige 13 AI+ A4M</t>
         </is>
       </c>
-      <c r="D58" s="16" t="inlineStr">
+      <c r="D58" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4944,7 +4939,7 @@
       </c>
       <c r="P58" s="6" t="inlineStr">
         <is>
-          <t>Audio Codec由原來的Reltek更換為TI，線路設計，placement變更</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -5019,7 +5014,7 @@
       </c>
       <c r="O59" s="6" t="inlineStr">
         <is>
-          <t>產線排程 DVT SMT@7/23</t>
+          <t>DVT SMT@7/23, RD 開機中</t>
         </is>
       </c>
       <c r="P59" s="6" t="inlineStr">
@@ -5100,7 +5095,7 @@
       </c>
       <c r="O60" s="11" t="inlineStr">
         <is>
-          <t>產線排程 DVT SMT@7/23</t>
+          <t>DVT SMT@7/23, RD 開機中</t>
         </is>
       </c>
       <c r="P60" s="11" t="inlineStr">
@@ -5180,7 +5175,7 @@
       </c>
       <c r="O61" s="11" t="inlineStr">
         <is>
-          <t>產線排程 DVT SMT@7/23</t>
+          <t>DVT SMT@7/23, RD 開機中</t>
         </is>
       </c>
       <c r="P61" s="11" t="inlineStr">
@@ -5203,7 +5198,7 @@
           <t>Stealth 16 AI+ B4WE</t>
         </is>
       </c>
-      <c r="D62" s="16" t="inlineStr">
+      <c r="D62" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5230,7 +5225,7 @@
       </c>
       <c r="I62" s="4" t="inlineStr">
         <is>
-          <t>2026/07/30</t>
+          <t>2026/07/31</t>
         </is>
       </c>
       <c r="J62" s="4" t="inlineStr">
@@ -5260,7 +5255,7 @@
       </c>
       <c r="O62" s="6" t="inlineStr">
         <is>
-          <t>0A 7/15 gerber out</t>
+          <t>0A 7/31 SMT</t>
         </is>
       </c>
       <c r="P62" s="6" t="inlineStr">
@@ -5284,7 +5279,7 @@
           <t>Stealth 16 AI+ B4WF</t>
         </is>
       </c>
-      <c r="D63" s="15" t="inlineStr">
+      <c r="D63" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5311,7 +5306,7 @@
       </c>
       <c r="I63" s="9" t="inlineStr">
         <is>
-          <t>2026/07/30</t>
+          <t>2026/07/31</t>
         </is>
       </c>
       <c r="J63" s="9" t="inlineStr">
@@ -5341,7 +5336,7 @@
       </c>
       <c r="O63" s="11" t="inlineStr">
         <is>
-          <t>0A 7/15 gerber out</t>
+          <t>0A 7/31 SMT</t>
         </is>
       </c>
       <c r="P63" s="11" t="inlineStr">
@@ -5365,7 +5360,7 @@
           <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
         </is>
       </c>
-      <c r="D64" s="15" t="inlineStr">
+      <c r="D64" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5392,7 +5387,7 @@
       </c>
       <c r="I64" s="9" t="inlineStr">
         <is>
-          <t>2026/07/30</t>
+          <t>2026/07/31</t>
         </is>
       </c>
       <c r="J64" s="9" t="inlineStr">
@@ -5422,7 +5417,7 @@
       </c>
       <c r="O64" s="11" t="inlineStr">
         <is>
-          <t>0A 7/15 gerber out</t>
+          <t>0A 7/31 SMT</t>
         </is>
       </c>
       <c r="P64" s="11" t="inlineStr">
@@ -5446,7 +5441,7 @@
           <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
         </is>
       </c>
-      <c r="D65" s="15" t="inlineStr">
+      <c r="D65" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5473,7 +5468,7 @@
       </c>
       <c r="I65" s="9" t="inlineStr">
         <is>
-          <t>2026/07/30</t>
+          <t>2026/07/31</t>
         </is>
       </c>
       <c r="J65" s="9" t="inlineStr">
@@ -5503,7 +5498,7 @@
       </c>
       <c r="O65" s="11" t="inlineStr">
         <is>
-          <t>0A 7/15 gerber out</t>
+          <t>0A 7/31 SMT</t>
         </is>
       </c>
       <c r="P65" s="11" t="inlineStr">
@@ -5527,7 +5522,7 @@
           <t>Raider 16 HX B14WI</t>
         </is>
       </c>
-      <c r="D66" s="16" t="inlineStr">
+      <c r="D66" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5604,10 +5599,10 @@
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Raider 16 HX B14WH</t>
-        </is>
-      </c>
-      <c r="D67" s="15" t="inlineStr">
+          <t>Raider 16 HX B14WJ</t>
+        </is>
+      </c>
+      <c r="D67" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5619,7 +5614,7 @@
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070Ti</t>
+          <t>RTX 5090</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
@@ -5664,10 +5659,14 @@
       </c>
       <c r="O67" s="11" t="inlineStr">
         <is>
-          <t>leverage Raider 16 HX B14WJ</t>
-        </is>
-      </c>
-      <c r="P67" s="11" t="inlineStr"/>
+          <t>7/24 Kick off，預計0M gerberout 8/28</t>
+        </is>
+      </c>
+      <c r="P67" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="68" hidden="1" outlineLevel="1">
       <c r="A68" s="7" t="n">
@@ -5680,10 +5679,10 @@
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>Raider 16 HX B14WJ</t>
-        </is>
-      </c>
-      <c r="D68" s="15" t="inlineStr">
+          <t>Raider 16 HX B14WH</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5695,7 +5694,7 @@
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>RTX 5090</t>
+          <t>RTX 5070Ti</t>
         </is>
       </c>
       <c r="G68" s="9" t="inlineStr">
@@ -5740,7 +5739,7 @@
       </c>
       <c r="O68" s="11" t="inlineStr">
         <is>
-          <t>7/24 Kick off，預計0A gerberout 8/28</t>
+          <t>leverage Raider 16 HX B14WJ</t>
         </is>
       </c>
       <c r="P68" s="11" t="inlineStr"/>
@@ -5786,7 +5785,7 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/05</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -5816,7 +5815,7 @@
       </c>
       <c r="O69" s="6" t="inlineStr">
         <is>
-          <t>预计8/3 DVT打板</t>
+          <t>预计8/5 DVT打板</t>
         </is>
       </c>
       <c r="P69" s="6" t="inlineStr">
@@ -5866,7 +5865,7 @@
       </c>
       <c r="I70" s="9" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/05</t>
         </is>
       </c>
       <c r="J70" s="9" t="inlineStr">
@@ -5896,7 +5895,7 @@
       </c>
       <c r="O70" s="11" t="inlineStr">
         <is>
-          <t>预计8/3 DVT打板</t>
+          <t>预计8/5 DVT打板</t>
         </is>
       </c>
       <c r="P70" s="11" t="inlineStr">
@@ -5946,7 +5945,7 @@
       </c>
       <c r="I71" s="9" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/05</t>
         </is>
       </c>
       <c r="J71" s="9" t="inlineStr">
@@ -5976,7 +5975,7 @@
       </c>
       <c r="O71" s="11" t="inlineStr">
         <is>
-          <t>预计8/3 DVT打板</t>
+          <t>预计8/5 DVT打板</t>
         </is>
       </c>
       <c r="P71" s="11" t="inlineStr">
@@ -6026,7 +6025,7 @@
       </c>
       <c r="I72" s="4" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/06</t>
         </is>
       </c>
       <c r="J72" s="4" t="inlineStr">
@@ -6056,12 +6055,12 @@
       </c>
       <c r="O72" s="6" t="inlineStr">
         <is>
-          <t>8/3 DVT SMT(H&amp;HX同步打板驗證)</t>
+          <t>8/6  DVT SMT</t>
         </is>
       </c>
       <c r="P72" s="6" t="inlineStr">
         <is>
-          <t>Spec變更:由crosshair max正式改Raider系列,對應thermal 手工樣品需重新打樣, RD 確認預計8/17收到樣品開始測試，比原計劃delay1周，雖不影響TTM，但期望RD 持續push廠商，keep原schedule不變,否則可能會影響到後續規劃的特仕版送樣時間,持續tracking</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -6106,7 +6105,7 @@
       </c>
       <c r="I73" s="9" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/06</t>
         </is>
       </c>
       <c r="J73" s="9" t="inlineStr">
@@ -6136,12 +6135,12 @@
       </c>
       <c r="O73" s="11" t="inlineStr">
         <is>
-          <t>8/3 DVT SMT(H&amp;HX同步打板驗證)</t>
+          <t>8/6  DVT SMT</t>
         </is>
       </c>
       <c r="P73" s="11" t="inlineStr">
         <is>
-          <t>Spec變更:由crosshair max正式改Raider系列,對應thermal 手工樣品需重新打樣, RD 確認預計8/17收到樣品開始測試，比原計劃delay1周，雖不影響TTM，但期望RD 持續push廠商，keep原schedule不變,否則可能會影響到後續規劃的特仕版送樣時間,持續tracking</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -6186,7 +6185,7 @@
       </c>
       <c r="I74" s="9" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/06</t>
         </is>
       </c>
       <c r="J74" s="9" t="inlineStr">
@@ -6216,12 +6215,12 @@
       </c>
       <c r="O74" s="11" t="inlineStr">
         <is>
-          <t>8/3 DVT SMT(H&amp;HX同步打板驗證)</t>
+          <t>8/6  DVT SMT</t>
         </is>
       </c>
       <c r="P74" s="11" t="inlineStr">
         <is>
-          <t>Spec變更:由crosshair max正式改Raider系列,對應thermal 手工樣品需重新打樣, RD 確認預計8/17收到樣品開始測試，比原計劃delay1周，雖不影響TTM，但期望RD 持續push廠商，keep原schedule不變,否則可能會影響到後續規劃的特仕版送樣時間,持續tracking</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -6266,7 +6265,7 @@
       </c>
       <c r="I75" s="9" t="inlineStr">
         <is>
-          <t>2026/08/03</t>
+          <t>2026/08/06</t>
         </is>
       </c>
       <c r="J75" s="9" t="inlineStr">
@@ -6296,12 +6295,12 @@
       </c>
       <c r="O75" s="11" t="inlineStr">
         <is>
-          <t>8/3 DVT SMT(H&amp;HX同步打板驗證)</t>
+          <t>8/6  DVT SMT</t>
         </is>
       </c>
       <c r="P75" s="11" t="inlineStr">
         <is>
-          <t>Spec變更:由crosshair max正式改Raider系列,對應thermal 手工樣品需重新打樣, RD 確認預計8/17收到樣品開始測試，比原計劃delay1周，雖不影響TTM，但期望RD 持續push廠商，keep原schedule不變,否則可能會影響到後續規劃的特仕版送樣時間,持續tracking</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -6319,7 +6318,7 @@
           <t>Titan 18 HX B4WH</t>
         </is>
       </c>
-      <c r="D76" s="16" t="inlineStr">
+      <c r="D76" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6381,7 +6380,8 @@
       </c>
       <c r="P76" s="6" t="inlineStr">
         <is>
-          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study.</t>
+          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.
+2) Seamless Haptic TP待Liteon提供final線路圖/2D3D/Spec for Lockdown確認.</t>
         </is>
       </c>
     </row>
@@ -6399,7 +6399,7 @@
           <t>Titan 18 HX B4WI</t>
         </is>
       </c>
-      <c r="D77" s="15" t="inlineStr">
+      <c r="D77" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6461,7 +6461,8 @@
       </c>
       <c r="P77" s="11" t="inlineStr">
         <is>
-          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study.</t>
+          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.
+2) Seamless Haptic TP待Liteon提供final線路圖/2D3D/Spec for Lockdown確認.</t>
         </is>
       </c>
     </row>
@@ -6479,7 +6480,7 @@
           <t>Titan 18 HX B4WJ</t>
         </is>
       </c>
-      <c r="D78" s="15" t="inlineStr">
+      <c r="D78" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6541,7 +6542,8 @@
       </c>
       <c r="P78" s="11" t="inlineStr">
         <is>
-          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study.</t>
+          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.
+2) Seamless Haptic TP待Liteon提供final線路圖/2D3D/Spec for Lockdown確認.</t>
         </is>
       </c>
     </row>
@@ -6559,7 +6561,7 @@
           <t>Raider 18 Max HX B4WH</t>
         </is>
       </c>
-      <c r="D79" s="15" t="inlineStr">
+      <c r="D79" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6621,7 +6623,7 @@
       </c>
       <c r="P79" s="11" t="inlineStr">
         <is>
-          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study.</t>
+          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.</t>
         </is>
       </c>
     </row>
@@ -6639,7 +6641,7 @@
           <t>Raider 18 Max HX B4WI</t>
         </is>
       </c>
-      <c r="D80" s="15" t="inlineStr">
+      <c r="D80" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6701,7 +6703,7 @@
       </c>
       <c r="P80" s="11" t="inlineStr">
         <is>
-          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study.</t>
+          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.</t>
         </is>
       </c>
     </row>
@@ -6719,7 +6721,7 @@
           <t>Raider 18 Max HX B4WJ</t>
         </is>
       </c>
-      <c r="D81" s="15" t="inlineStr">
+      <c r="D81" s="16" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6781,7 +6783,7 @@
       </c>
       <c r="P81" s="11" t="inlineStr">
         <is>
-          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study.</t>
+          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NPI Dashboard 2026-07-31 13:36
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -1258,12 +1258,13 @@
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
-          <t>DDR5 sku, MVT測試中, 7/24調撥,預計7/30 PCB risk buy</t>
+          <t>DDR5 sku, MVT2 組裝中</t>
         </is>
       </c>
       <c r="P10" s="6" t="inlineStr">
         <is>
-          <t>1).Materiel: #A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/E MP的目標,麻煩RD/採購pull in森田薄膜進料時間. #因7/28需量產備料四區鍵盤,如果還有鍵盤相關問題,請儘速提出</t>
+          <t>1) ATS與MP的物料簽樣與備料,需要RD與採購和物管協助
+2)A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/30 MP的目標,需要RD/採購協助助pull in</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1335,13 @@
       </c>
       <c r="O11" s="11" t="inlineStr">
         <is>
-          <t>DDR5 sku, MVT測試中, 7/24調撥,預計7/30 PCB risk buy</t>
+          <t>DDR5 sku, MVT2組裝中</t>
         </is>
       </c>
       <c r="P11" s="11" t="inlineStr">
         <is>
-          <t>1).Materiel: #A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/E MP的目標,麻煩RD/採購pull in森田薄膜進料時間. #因7/28需量產備料四區鍵盤,如果還有鍵盤相關問題,請儘速提出</t>
+          <t>1) ATS與MP的物料簽樣與備料,需要RD與採購和物管協助
+2)A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/30 MP的目標,需要RD/採購協助助pull in</t>
         </is>
       </c>
     </row>
@@ -1410,12 +1412,13 @@
       </c>
       <c r="O12" s="11" t="inlineStr">
         <is>
-          <t>DDR5 sku, MVT測試中, 7/24調撥,預計7/30 PCB risk buy</t>
+          <t>DDR5 sku, MVT2組裝中</t>
         </is>
       </c>
       <c r="P12" s="11" t="inlineStr">
         <is>
-          <t>1).Materiel: #A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/E MP的目標,麻煩RD/採購pull in森田薄膜進料時間. #因7/28需量產備料四區鍵盤,如果還有鍵盤相關問題,請儘速提出</t>
+          <t>1) ATS與MP的物料簽樣與備料,需要RD與採購和物管協助
+2)A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/30 MP的目標,需要RD/採購協助助pull in</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1648,8 @@
       </c>
       <c r="P15" s="11" t="inlineStr">
         <is>
-          <t>1).Materiel: #A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/E MP的目標,麻煩RD/採購pull in森田薄膜進料時間.</t>
+          <t>1) ATS與MP的物料簽樣與備料,需要RD與採購和物管協助
+2)A件交期依森田薄膜進料時間,預計15T3組裝在8/25,MP在9/3,會比原時程晚4天,會導致15T3無法meet原8/30 MP的目標,需要RD/採購協助助pull in</t>
         </is>
       </c>
     </row>
@@ -1808,10 +1812,10 @@
       </c>
       <c r="P17" s="11" t="inlineStr">
         <is>
-          <t>1)Battery life: 以2.8K panel+day0 rev.A環境用balance mode測試，Modern standby可達標準，Web browersing尚差0.2Hr，將於BSP Day0 rev.B再進行驗證。
-2)NV Abnormal shut down 的solution，確認需於BSP Day0 rev.B驗證，預計7/23 image完成後，DQA/工廠會同時切換驗證確認。
-3)NV更新可for出貨的 GPU driver提前於8/3美國時間release，後須計畫以此版本進行測試並出貨，不影響現行Schedule，ATS仍定於8/17開始
-4)for NV/MSFT 113pcs樣品，已於7/17 SMT，7/22 ASS'Y，並通知業務轉單，預計下周可出貨</t>
+          <t>1)Battery life: 2.8K panel+day0 rev.B+balance mode測試，Web browersing測試達716min，接近過關。NV更新會導入部分省電作法於Rev. C，待更新SW後驗證。
+2)NV Abnormal shut down 的solution，經DQA於BSP Day0 rev.B驗證後，未發生除error code "0x7E"外的ABS現象，後續會持續觀察。
+3) Day0 rev.C BIOS 7/29 release，測試image預計7/30 release，工廠/DQA將同時切換測試。
+4)工廠用MP樣品測試，反應主要問題，需RD一起分析 1.Long run自動測試 S3/S4/S5/ Reboot/ FSU進系統在login 画面持续转圈宕機，黑屏無顯 ,宕機 2. LCD 花屏（panel 有黑線) 3. camera 開啟錄像后 camera APP 卡住</t>
         </is>
       </c>
     </row>
@@ -5019,8 +5023,9 @@
       </c>
       <c r="P59" s="6" t="inlineStr">
         <is>
-          <t>1) B07-669945C-T07，FW 燒錄不上，待治具更新軟體;
-2) Schedule:NV VBIOS @1/6, gating 8天,預計12/E 拿到WHQL，可能影響到最終TTM 時間</t>
+          <t>1)目前0M PCBA未開機,0N geberout@8/25;
+2) B07-669945C-T07，FW 燒錄不上，待治具更新軟體;
+3) Schedule:NV VBIOS @1/6, gating 8天,預計12/E 拿到WHQL，可能影響到最終TTM 時間</t>
         </is>
       </c>
     </row>
@@ -5519,7 +5524,7 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Raider 16 HX B14WI</t>
+          <t>Raider 16 HX B14WH</t>
         </is>
       </c>
       <c r="D66" s="17" t="inlineStr">
@@ -5534,7 +5539,7 @@
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>RTX 5080</t>
+          <t>RTX 5070Ti</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -5579,7 +5584,7 @@
       </c>
       <c r="O66" s="6" t="inlineStr">
         <is>
-          <t>leverage Raider 16 HX B14WJ</t>
+          <t>7/24 Kick off，預計0M gerberout 8/28</t>
         </is>
       </c>
       <c r="P66" s="6" t="inlineStr">
@@ -5599,7 +5604,7 @@
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Raider 16 HX B14WJ</t>
+          <t>Raider 16 HX B14WI</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -5614,7 +5619,7 @@
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>RTX 5090</t>
+          <t>RTX 5080</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
@@ -5679,7 +5684,7 @@
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>Raider 16 HX B14WH</t>
+          <t>Raider 16 HX B14WJ</t>
         </is>
       </c>
       <c r="D68" s="16" t="inlineStr">
@@ -5694,7 +5699,7 @@
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070Ti</t>
+          <t>RTX 5090</t>
         </is>
       </c>
       <c r="G68" s="9" t="inlineStr">
@@ -5739,10 +5744,14 @@
       </c>
       <c r="O68" s="11" t="inlineStr">
         <is>
-          <t>leverage Raider 16 HX B14WJ</t>
-        </is>
-      </c>
-      <c r="P68" s="11" t="inlineStr"/>
+          <t>7/24 Kick off，預計0M gerberout 8/28</t>
+        </is>
+      </c>
+      <c r="P68" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -6060,7 +6069,7 @@
       </c>
       <c r="P72" s="6" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>由raider改回crosshair，待確認 final SPEC&amp;ID color plan，對schedule 影響TBD</t>
         </is>
       </c>
     </row>
@@ -6140,7 +6149,7 @@
       </c>
       <c r="P73" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>由raider改回crosshair，待確認 final SPEC&amp;ID color plan，對schedule 影響TBD</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6229,7 @@
       </c>
       <c r="P74" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>由raider改回crosshair，待確認 final SPEC&amp;ID color plan，對schedule 影響TBD</t>
         </is>
       </c>
     </row>
@@ -6300,7 +6309,7 @@
       </c>
       <c r="P75" s="11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>由raider改回crosshair，待確認 final SPEC&amp;ID color plan，對schedule 影響TBD</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NPI Dashboard 2026-08-03 08:35
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -47,12 +47,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="007030A0"/>
+      <color rgb="00ED7D31"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00ED7D31"/>
+      <color rgb="007030A0"/>
       <sz val="10"/>
     </font>
     <font>
@@ -134,13 +134,13 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1985,12 +1985,12 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1PWE</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>DVT</t>
+          <t>Cyborg A15 Max C1PWF</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -2021,33 +2021,35 @@
       <c r="J20" s="4" t="inlineStr"/>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>2026/08/04</t>
+          <t>2026/08/07</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/08/21</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>2026/09/09</t>
+          <t>2026/09/12</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>2026/09/19</t>
+          <t>2026/09/22</t>
         </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
-          <t>HPT sku:預計8/3 MVT SMT,目前HPT1搭配RC4版本的BIOS測試MODS still fail,請BIOS RD持續與AMD co-work釐清問題</t>
+          <t>HPT sku:預計8/7 MVT SMT,請BIOS RD儘速提供PI 1200i NDA版本的MSI BIOS</t>
         </is>
       </c>
       <c r="P20" s="6" t="inlineStr">
         <is>
-          <t>1).Schedule:AMD原預計7/22 release PI 1200I NDA,再次延期,待 AMD提供進一步時程後,將更新 MP Schedule.
-2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
+          <t>"
+1).Schedule:AMD PI 1200i NDA release@7/28 USA time(original 6/19,delay 39天)與工廠將MVT排程延至8/7 (original 8/4,delay 3天),因要和量產工單一起生產,因應上述時程變更,MP預計延至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
+22),後續將依實際測試結果滾動式調整專案時程。
+2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響"</t>
         </is>
       </c>
     </row>
@@ -2062,12 +2064,12 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1PWF</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>DVT</t>
+          <t>Cyborg A15 Max C1PWG</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -2077,7 +2079,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
@@ -2098,33 +2100,35 @@
       <c r="J21" s="9" t="inlineStr"/>
       <c r="K21" s="9" t="inlineStr">
         <is>
-          <t>2026/08/04</t>
+          <t>2026/08/07</t>
         </is>
       </c>
       <c r="L21" s="9" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/08/21</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
         <is>
-          <t>2026/09/09</t>
+          <t>2026/09/12</t>
         </is>
       </c>
       <c r="N21" s="9" t="inlineStr">
         <is>
-          <t>2026/09/19</t>
+          <t>2026/09/22</t>
         </is>
       </c>
       <c r="O21" s="11" t="inlineStr">
         <is>
-          <t>HPT sku:預計8/3 MVT SMT,目前HPT1搭配RC4版本的BIOS測試MODS still fail,請BIOS RD持續與AMD co-work釐清問題</t>
+          <t>HPT sku:預計8/7 MVT SMT,請BIOS RD儘速提供PI 1200i NDA版本的MSI BIOS</t>
         </is>
       </c>
       <c r="P21" s="11" t="inlineStr">
         <is>
-          <t>1).Schedule:AMD原預計7/22 release PI 1200I NDA,再次延期,待 AMD提供進一步時程後,將更新 MP Schedule.
-2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
+          <t>"
+1).Schedule:AMD PI 1200i NDA release@7/28 USA time(original 6/19,delay 39天)與工廠將MVT排程延至8/7 (original 8/4,delay 3天),因要和量產工單一起生產,因應上述時程變更,MP預計延至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
+22),後續將依實際測試結果滾動式調整專案時程。
+2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響"</t>
         </is>
       </c>
     </row>
@@ -2139,12 +2143,12 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1PWG</t>
-        </is>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>DVT</t>
+          <t>Cyborg A15 Max C1PWE</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -2154,7 +2158,7 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
@@ -2175,32 +2179,33 @@
       <c r="J22" s="9" t="inlineStr"/>
       <c r="K22" s="9" t="inlineStr">
         <is>
-          <t>2026/08/04</t>
+          <t>2026/08/07</t>
         </is>
       </c>
       <c r="L22" s="9" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/08/21</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>2026/09/09</t>
+          <t>2026/09/12</t>
         </is>
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>2026/09/19</t>
+          <t>2026/09/22</t>
         </is>
       </c>
       <c r="O22" s="11" t="inlineStr">
         <is>
-          <t>HPT sku:預計8/3 MVT SMT,目前HPT1搭配RC4版本的BIOS測試MODS still fail,請BIOS RD持續與AMD co-work釐清問題</t>
+          <t>HPT sku:預計8/7 MVT SMT,請BIOS RD儘速提供PI 1200i NDA版本的MSI BIOS</t>
         </is>
       </c>
       <c r="P22" s="11" t="inlineStr">
         <is>
-          <t>1).Schedule:AMD原預計7/22 release PI 1200I NDA,再次延期,待 AMD提供進一步時程後,將更新 MP Schedule.
+          <t>1).Schedule:AMD PI 1200i NDA release@7/28 USA time(original 6/19,delay 39天)與工廠將MVT排程延至8/7 (original 8/4,delay 3天),因要和量產工單一起生產,因應上述時程變更,MP預計延至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
+22),後續將依實際測試結果滾動式調整專案時程。
 2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
         </is>
       </c>
@@ -2219,9 +2224,9 @@
           <t>Cyborg A15 C1PWE</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>DVT</t>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>MVT</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -2252,32 +2257,33 @@
       <c r="J23" s="9" t="inlineStr"/>
       <c r="K23" s="9" t="inlineStr">
         <is>
-          <t>2026/08/04</t>
+          <t>2026/08/07</t>
         </is>
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/08/21</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>2026/09/09</t>
+          <t>2026/09/12</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>2026/09/19</t>
+          <t>2026/09/22</t>
         </is>
       </c>
       <c r="O23" s="11" t="inlineStr">
         <is>
-          <t>HPT sku:預計8/3 MVT SMT,目前HPT1搭配RC4版本的BIOS測試MODS still fail,請BIOS RD持續與AMD co-work釐清問題</t>
+          <t>HPT sku:預計8/7 MVT SMT,請BIOS RD儘速提供PI 1200i NDA版本的MSI BIOS</t>
         </is>
       </c>
       <c r="P23" s="11" t="inlineStr">
         <is>
-          <t>1).Schedule:AMD原預計7/22 release PI 1200I NDA,再次延期,待 AMD提供進一步時程後,將更新 MP Schedule.
+          <t>1).Schedule:AMD PI 1200i NDA release@7/28 USA time(original 6/19,delay 39天)與工廠將MVT排程延至8/7 (original 8/4,delay 3天),因要和量產工單一起生產,因應上述時程變更,MP預計延至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
+22),後續將依實際測試結果滾動式調整專案時程。
 2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
         </is>
       </c>
@@ -2377,7 +2383,7 @@
           <t>Prestige N16 AI+ C1M</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -2457,7 +2463,7 @@
           <t>Katana 18 HX A14WEK</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -2537,7 +2543,7 @@
           <t>Katana 18 HX A14WFK</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -2617,7 +2623,7 @@
           <t>Katana 18 HX A14WGK</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -2697,7 +2703,7 @@
           <t>Katana 18 HX A14WEOK</t>
         </is>
       </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2773,7 +2779,7 @@
           <t>Katana 18 HX A14WFOK</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2849,7 +2855,7 @@
           <t>Katana 18 HX A14WGOK</t>
         </is>
       </c>
-      <c r="D31" s="13" t="inlineStr">
+      <c r="D31" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2925,7 +2931,7 @@
           <t>Crosshair 18 Max HX B14WEO</t>
         </is>
       </c>
-      <c r="D32" s="13" t="inlineStr">
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3001,7 +3007,7 @@
           <t>Crosshair 18 Max HX B14WFO</t>
         </is>
       </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3077,7 +3083,7 @@
           <t>Crosshair 18 Max HX B14WGO</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D34" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3153,7 +3159,7 @@
           <t>Crosshair 18 Max HX B14WGXO</t>
         </is>
       </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="D35" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3229,7 +3235,7 @@
           <t>Crosshair 18 Max HX B14WE</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -3309,7 +3315,7 @@
           <t>Crosshair 18 Max HX B14WF</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
+      <c r="D37" s="13" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -3389,7 +3395,7 @@
           <t>Crosshair 18 Max HX B14WG</t>
         </is>
       </c>
-      <c r="D38" s="15" t="inlineStr">
+      <c r="D38" s="13" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -3469,7 +3475,7 @@
           <t>Crosshair 18 Max HX B14WGX</t>
         </is>
       </c>
-      <c r="D39" s="15" t="inlineStr">
+      <c r="D39" s="13" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -3549,7 +3555,7 @@
           <t>Crosshair 18 Max HX B2WE</t>
         </is>
       </c>
-      <c r="D40" s="16" t="inlineStr">
+      <c r="D40" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3621,7 +3627,7 @@
           <t>Crosshair 18 Max HX B2WEO</t>
         </is>
       </c>
-      <c r="D41" s="16" t="inlineStr">
+      <c r="D41" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3693,7 +3699,7 @@
           <t>Crosshair 18 Max HX B2WF</t>
         </is>
       </c>
-      <c r="D42" s="16" t="inlineStr">
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3765,7 +3771,7 @@
           <t>Crosshair 18 Max HX B2WFO</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3837,7 +3843,7 @@
           <t>Crosshair 18 Max HX B2WG</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
+      <c r="D44" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3909,7 +3915,7 @@
           <t>Crosshair 18 Max HX B2WGO</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
+      <c r="D45" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -3981,7 +3987,7 @@
           <t>Crosshair 18 Max HX B2WGX</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
+      <c r="D46" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4053,7 +4059,7 @@
           <t>Crosshair 18 Max HX B2WGXO</t>
         </is>
       </c>
-      <c r="D47" s="16" t="inlineStr">
+      <c r="D47" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4125,7 +4131,7 @@
           <t>Katana 18 HX A2WEK</t>
         </is>
       </c>
-      <c r="D48" s="16" t="inlineStr">
+      <c r="D48" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4197,7 +4203,7 @@
           <t>Katana 18 HX A2WEOK</t>
         </is>
       </c>
-      <c r="D49" s="16" t="inlineStr">
+      <c r="D49" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4273,7 +4279,7 @@
           <t>Katana 18 HX A2WFK</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
+      <c r="D50" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4345,7 +4351,7 @@
           <t>Katana 18 HX A2WFOK</t>
         </is>
       </c>
-      <c r="D51" s="16" t="inlineStr">
+      <c r="D51" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4421,7 +4427,7 @@
           <t>Katana 18 HX A2WGK</t>
         </is>
       </c>
-      <c r="D52" s="16" t="inlineStr">
+      <c r="D52" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4493,7 +4499,7 @@
           <t>Katana 18 HX A2WGOK</t>
         </is>
       </c>
-      <c r="D53" s="16" t="inlineStr">
+      <c r="D53" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4569,7 +4575,7 @@
           <t>Prestige 14 AI</t>
         </is>
       </c>
-      <c r="D54" s="12" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -4649,7 +4655,7 @@
           <t>Prestige 14 AI+ Flip</t>
         </is>
       </c>
-      <c r="D55" s="13" t="inlineStr">
+      <c r="D55" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -4729,7 +4735,7 @@
           <t>Prestige 16 AI+</t>
         </is>
       </c>
-      <c r="D56" s="12" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -4805,7 +4811,7 @@
           <t>Prestige 16 Flip AI+</t>
         </is>
       </c>
-      <c r="D57" s="13" t="inlineStr">
+      <c r="D57" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -4961,7 +4967,7 @@
           <t>Stealth 16 AI+ B4WI</t>
         </is>
       </c>
-      <c r="D59" s="12" t="inlineStr">
+      <c r="D59" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -5018,12 +5024,12 @@
       </c>
       <c r="O59" s="6" t="inlineStr">
         <is>
-          <t>DVT SMT@7/23, RD 開機中</t>
+          <t>RD debug中 (PCBA僅HDMI會顯示)</t>
         </is>
       </c>
       <c r="P59" s="6" t="inlineStr">
         <is>
-          <t>1)目前0M PCBA未開機,0N geberout@8/25;
+          <t>1)目前0M PCBA開機,但目前僅HDMI會顯示，0N geberout@8/25，請RD幫忙盡快debug;
 2) B07-669945C-T07，FW 燒錄不上，待治具更新軟體;
 3) Schedule:NV VBIOS @1/6, gating 8天,預計12/E 拿到WHQL，可能影響到最終TTM 時間</t>
         </is>
@@ -5043,7 +5049,7 @@
           <t>Stealth 16 AI+ B4WH</t>
         </is>
       </c>
-      <c r="D60" s="13" t="inlineStr">
+      <c r="D60" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -5100,7 +5106,7 @@
       </c>
       <c r="O60" s="11" t="inlineStr">
         <is>
-          <t>DVT SMT@7/23, RD 開機中</t>
+          <t>RD debug中 (PCBA僅HDMI會顯示)</t>
         </is>
       </c>
       <c r="P60" s="11" t="inlineStr">
@@ -5123,7 +5129,7 @@
           <t>Stealth 16 AI+ B4WJ</t>
         </is>
       </c>
-      <c r="D61" s="13" t="inlineStr">
+      <c r="D61" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -5180,7 +5186,7 @@
       </c>
       <c r="O61" s="11" t="inlineStr">
         <is>
-          <t>DVT SMT@7/23, RD 開機中</t>
+          <t>RD debug中 (PCBA僅HDMI會顯示)</t>
         </is>
       </c>
       <c r="P61" s="11" t="inlineStr">
@@ -5284,7 +5290,7 @@
           <t>Stealth 16 AI+ B4WF</t>
         </is>
       </c>
-      <c r="D63" s="16" t="inlineStr">
+      <c r="D63" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5365,7 +5371,7 @@
           <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
         </is>
       </c>
-      <c r="D64" s="16" t="inlineStr">
+      <c r="D64" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5446,7 +5452,7 @@
           <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
         </is>
       </c>
-      <c r="D65" s="16" t="inlineStr">
+      <c r="D65" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5607,7 +5613,7 @@
           <t>Raider 16 HX B14WI</t>
         </is>
       </c>
-      <c r="D67" s="16" t="inlineStr">
+      <c r="D67" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5687,7 +5693,7 @@
           <t>Raider 16 HX B14WJ</t>
         </is>
       </c>
-      <c r="D68" s="16" t="inlineStr">
+      <c r="D68" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -5767,7 +5773,7 @@
           <t>Raider 16 Max HX B4WH</t>
         </is>
       </c>
-      <c r="D69" s="12" t="inlineStr">
+      <c r="D69" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -5847,7 +5853,7 @@
           <t>Raider 16 Max HX B4WI</t>
         </is>
       </c>
-      <c r="D70" s="13" t="inlineStr">
+      <c r="D70" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -5927,7 +5933,7 @@
           <t>Raider 16 Max HX B4WJ</t>
         </is>
       </c>
-      <c r="D71" s="13" t="inlineStr">
+      <c r="D71" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -6007,7 +6013,7 @@
           <t>Raider 16 HX B4WE</t>
         </is>
       </c>
-      <c r="D72" s="12" t="inlineStr">
+      <c r="D72" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -6087,7 +6093,7 @@
           <t>Raider 16 HX B4WF</t>
         </is>
       </c>
-      <c r="D73" s="13" t="inlineStr">
+      <c r="D73" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -6167,7 +6173,7 @@
           <t>Raider 16 HX B4WG</t>
         </is>
       </c>
-      <c r="D74" s="13" t="inlineStr">
+      <c r="D74" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -6247,7 +6253,7 @@
           <t>Raider 16 HX B4WGX</t>
         </is>
       </c>
-      <c r="D75" s="13" t="inlineStr">
+      <c r="D75" s="14" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -6384,13 +6390,12 @@
       </c>
       <c r="O76" s="6" t="inlineStr">
         <is>
-          <t>LAN footprint線路修改,0M gerber out變更為8/3,暫不影響後續EVT schedule.</t>
+          <t>製程DFM修改需求,0M gerber out變更為8/4,暫不影響後續EVT schedule.</t>
         </is>
       </c>
       <c r="P76" s="6" t="inlineStr">
         <is>
-          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.
-2) Seamless Haptic TP待Liteon提供final線路圖/2D3D/Spec for Lockdown確認.</t>
+          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6413,7 @@
           <t>Titan 18 HX B4WI</t>
         </is>
       </c>
-      <c r="D77" s="16" t="inlineStr">
+      <c r="D77" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6465,13 +6470,12 @@
       </c>
       <c r="O77" s="11" t="inlineStr">
         <is>
-          <t>LAN footprint線路修改,0M gerber out變更為8/3,暫不影響後續EVT schedule.</t>
+          <t>製程DFM修改需求,0M gerber out變更為8/4,暫不影響後續EVT schedule.</t>
         </is>
       </c>
       <c r="P77" s="11" t="inlineStr">
         <is>
-          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.
-2) Seamless Haptic TP待Liteon提供final線路圖/2D3D/Spec for Lockdown確認.</t>
+          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.</t>
         </is>
       </c>
     </row>
@@ -6489,7 +6493,7 @@
           <t>Titan 18 HX B4WJ</t>
         </is>
       </c>
-      <c r="D78" s="16" t="inlineStr">
+      <c r="D78" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6546,13 +6550,12 @@
       </c>
       <c r="O78" s="11" t="inlineStr">
         <is>
-          <t>LAN footprint線路修改,0M gerber out變更為8/3,暫不影響後續EVT schedule.</t>
+          <t>製程DFM修改需求,0M gerber out變更為8/4,暫不影響後續EVT schedule.</t>
         </is>
       </c>
       <c r="P78" s="11" t="inlineStr">
         <is>
-          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.
-2) Seamless Haptic TP待Liteon提供final線路圖/2D3D/Spec for Lockdown確認.</t>
+          <t>1) SSE需要進行約4週的POC評估確認1851 aRGB介面Light Bar的技術可行性以及後續FW開發工作,已提供MCU demo board/Light bar for SSE POC study, SSE預計WW33提供評估結果.</t>
         </is>
       </c>
     </row>
@@ -6570,7 +6573,7 @@
           <t>Raider 18 Max HX B4WH</t>
         </is>
       </c>
-      <c r="D79" s="16" t="inlineStr">
+      <c r="D79" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6627,7 +6630,7 @@
       </c>
       <c r="O79" s="11" t="inlineStr">
         <is>
-          <t>LAN footprint線路修改,0M gerber out變更為8/3,暫不影響後續EVT schedule.</t>
+          <t>製程DFM修改需求,0M gerber out變更為8/4,暫不影響後續EVT schedule.</t>
         </is>
       </c>
       <c r="P79" s="11" t="inlineStr">
@@ -6650,7 +6653,7 @@
           <t>Raider 18 Max HX B4WI</t>
         </is>
       </c>
-      <c r="D80" s="16" t="inlineStr">
+      <c r="D80" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6707,7 +6710,7 @@
       </c>
       <c r="O80" s="11" t="inlineStr">
         <is>
-          <t>LAN footprint線路修改,0M gerber out變更為8/3,暫不影響後續EVT schedule.</t>
+          <t>製程DFM修改需求,0M gerber out變更為8/4,暫不影響後續EVT schedule.</t>
         </is>
       </c>
       <c r="P80" s="11" t="inlineStr">
@@ -6730,7 +6733,7 @@
           <t>Raider 18 Max HX B4WJ</t>
         </is>
       </c>
-      <c r="D81" s="16" t="inlineStr">
+      <c r="D81" s="15" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -6787,7 +6790,7 @@
       </c>
       <c r="O81" s="11" t="inlineStr">
         <is>
-          <t>LAN footprint線路修改,0M gerber out變更為8/3,暫不影響後續EVT schedule.</t>
+          <t>製程DFM修改需求,0M gerber out變更為8/4,暫不影響後續EVT schedule.</t>
         </is>
       </c>
       <c r="P81" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Update NPI Dashboard 2026-08-11 10:09
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -1127,7 +1127,7 @@
       </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
-          <t>DDR5 sku, MVT 測試中</t>
+          <t>DDR5 sku, MVT驗證中</t>
         </is>
       </c>
       <c r="P8" s="6" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="O9" s="11" t="inlineStr">
         <is>
-          <t>DDR5 sku, MVT 測試中</t>
+          <t>DDR5 sku, MVT驗證中</t>
         </is>
       </c>
       <c r="P9" s="11" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="O10" s="11" t="inlineStr">
         <is>
-          <t>DDR5 sku, MVT 測試中</t>
+          <t>DDR5 sku, MVT驗證中</t>
         </is>
       </c>
       <c r="P10" s="11" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="O11" s="11" t="inlineStr">
         <is>
-          <t>DDR4 sku, MVT 測試中,預計8/7 PCB risk buy</t>
+          <t>DDR4 sku, MVT驗證中</t>
         </is>
       </c>
       <c r="P11" s="11" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="O12" s="11" t="inlineStr">
         <is>
-          <t>DDR4 sku, MVT 測試中,預計8/7 PCB risk buy</t>
+          <t>DDR4 sku, MVT驗證中</t>
         </is>
       </c>
       <c r="P12" s="11" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="O13" s="11" t="inlineStr">
         <is>
-          <t>DDR4 sku, MVT 測試中,預計8/7 PCB risk buy</t>
+          <t>DDR4 sku, MVT驗證中</t>
         </is>
       </c>
       <c r="P13" s="11" t="inlineStr">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1PWF</t>
+          <t>Cyborg A15 Max C1PWE</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1911,15 +1911,16 @@
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
-          <t>HPT sku:預計8/7 MVT SMT,8/10試組,8/12組裝</t>
+          <t>HPT sku:預計8/10 MVT 試組,8/12組裝</t>
         </is>
       </c>
       <c r="P18" s="6" t="inlineStr">
         <is>
-          <t>"
-1).Schedule:AMD PI 1200i NDA release@7/28 USA time(original 6/19,delay 39天)與工廠將MVT排程延至8/7 (original 8/4,delay 3天),因要和量產工單一起生產,因應上述時程變更,MP預計延至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
-22),後續將依實際測試結果滾動式調整專案時程。
-2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響"</t>
+          <t>1).Schedule:AMD PI 1200I NDA Release delay(6/19→7/
+28)與MVT SMT 排程延後(8/4→8/
+7), 累計delay 42天, 取消 DVT排程改以 APU Rework 驗證追趕時程後, MP還是會delay 22天至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
+22),後續將依實際測試結果滾動式調整專案時程
+2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1935,7 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1PWG</t>
+          <t>Cyborg A15 Max C1PWF</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1949,7 +1950,7 @@
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
@@ -1990,15 +1991,16 @@
       </c>
       <c r="O19" s="11" t="inlineStr">
         <is>
-          <t>HPT sku:預計8/7 MVT SMT,8/10試組,8/12組裝</t>
+          <t>HPT sku:預計8/10 MVT 試組,8/12組裝</t>
         </is>
       </c>
       <c r="P19" s="11" t="inlineStr">
         <is>
-          <t>"
-1).Schedule:AMD PI 1200i NDA release@7/28 USA time(original 6/19,delay 39天)與工廠將MVT排程延至8/7 (original 8/4,delay 3天),因要和量產工單一起生產,因應上述時程變更,MP預計延至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
-22),後續將依實際測試結果滾動式調整專案時程。
-2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響"</t>
+          <t>1).Schedule:AMD PI 1200I NDA Release delay(6/19→7/
+28)與MVT SMT 排程延後(8/4→8/
+7), 累計delay 42天, 取消 DVT排程改以 APU Rework 驗證追趕時程後, MP還是會delay 22天至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
+22),後續將依實際測試結果滾動式調整專案時程
+2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2015,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Cyborg A15 Max C1PWE</t>
+          <t>Cyborg A15 Max C1PWG</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
@@ -2028,7 +2030,7 @@
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
@@ -2069,13 +2071,15 @@
       </c>
       <c r="O20" s="11" t="inlineStr">
         <is>
-          <t>HPT sku:預計8/7 MVT SMT,8/10試組,8/12組裝</t>
+          <t>HPT sku:預計8/10 MVT 試組,8/12組裝</t>
         </is>
       </c>
       <c r="P20" s="11" t="inlineStr">
         <is>
-          <t>1).Schedule:AMD PI 1200i NDA release@7/28 USA time(original 6/19,delay 39天)與工廠將MVT排程延至8/7 (original 8/4,delay 3天),因要和量產工單一起生產,因應上述時程變更,MP預計延至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
-22),後續將依實際測試結果滾動式調整專案時程。
+          <t>1).Schedule:AMD PI 1200I NDA Release delay(6/19→7/
+28)與MVT SMT 排程延後(8/4→8/
+7), 累計delay 42天, 取消 DVT排程改以 APU Rework 驗證追趕時程後, MP還是會delay 22天至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
+22),後續將依實際測試結果滾動式調整專案時程
 2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
         </is>
       </c>
@@ -2147,13 +2151,15 @@
       </c>
       <c r="O21" s="11" t="inlineStr">
         <is>
-          <t>HPT sku:預計8/7 MVT SMT,8/10試組,8/12組裝</t>
+          <t>HPT sku:預計8/10 MVT 試組,8/12組裝</t>
         </is>
       </c>
       <c r="P21" s="11" t="inlineStr">
         <is>
-          <t>1).Schedule:AMD PI 1200i NDA release@7/28 USA time(original 6/19,delay 39天)與工廠將MVT排程延至8/7 (original 8/4,delay 3天),因要和量產工單一起生產,因應上述時程變更,MP預計延至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
-22),後續將依實際測試結果滾動式調整專案時程。
+          <t>1).Schedule:AMD PI 1200I NDA Release delay(6/19→7/
+28)與MVT SMT 排程延後(8/4→8/
+7), 累計delay 42天, 取消 DVT排程改以 APU Rework 驗證追趕時程後, MP還是會delay 22天至9/22(先前已由 9 /17提前至 8/31, 現又延至9/
+22),後續將依實際測試結果滾動式調整專案時程
 2).Material:Thermal module依現有設計圖面take risk讓廠商去進行修模同時備料MVT &amp; ATS,若實測結果未達預期,物料需報廢,schedule也可能因此造成影響</t>
         </is>
       </c>
@@ -2236,7 +2242,7 @@
       <c r="P22" s="6" t="inlineStr">
         <is>
           <t>1) Schedule:  a. MVT拆分兩次SMT搭配PS software作驗證 b. 量產software更新時間至10/16, update ATS@11/9.
-2)備料：量產交料2.8k HQ23, 最新MP*1K交期回復在12/M（follow leading customer）交料, 與ATS start Gap 2個月, 採購協助push廠商交期中</t>
+2)備料：量產交料2.8k HQ23, 最新MP*1K交期, MSI &amp; Samsung co-work, target 10/M交料for ATS, tracking</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NPI Dashboard 2026-08-27 15:04
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPI Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NPI Dashboard'!$A$1:$P$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -134,6 +134,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -519,7 +522,7 @@
     <outlinePr summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -689,7 +692,7 @@
       </c>
       <c r="O2" s="6" t="inlineStr">
         <is>
-          <t>DDR5: RTX5050進行C/R組裝@8/20 26PN078888C*50</t>
+          <t>DDR5: RTX5050,8/28正式進入MP</t>
         </is>
       </c>
       <c r="P2" s="6" t="inlineStr">
@@ -765,7 +768,7 @@
       </c>
       <c r="O3" s="11" t="inlineStr">
         <is>
-          <t>DDR5: RTX5060預計C/R組裝@8/28 26PN077951C*50</t>
+          <t>DDR5: RTX5060預計C/R組裝@8/29 26PN077951C*50</t>
         </is>
       </c>
       <c r="P3" s="11" t="inlineStr">
@@ -841,7 +844,7 @@
       </c>
       <c r="O4" s="11" t="inlineStr">
         <is>
-          <t>DDR5: RTX5070進行ATS 組裝@8/20 26PN077002A*100</t>
+          <t>DDR5: RTX5070,8/28正式進入MP</t>
         </is>
       </c>
       <c r="P4" s="11" t="inlineStr">
@@ -917,7 +920,7 @@
       </c>
       <c r="O5" s="11" t="inlineStr">
         <is>
-          <t>DDR4: RTX5050進行C/R組裝@8/20 26PN078888C*50</t>
+          <t>DDR4: RTX5050,8/28正式進入MP</t>
         </is>
       </c>
       <c r="P5" s="11" t="inlineStr">
@@ -993,7 +996,7 @@
       </c>
       <c r="O6" s="11" t="inlineStr">
         <is>
-          <t>DDR4: RTX5060預計C/R組裝@8/28 26PN077951C*50</t>
+          <t>DDR4: RTX5060預計C/R組裝@8/29 26PN077951C*50</t>
         </is>
       </c>
       <c r="P6" s="11" t="inlineStr">
@@ -1069,7 +1072,7 @@
       </c>
       <c r="O7" s="11" t="inlineStr">
         <is>
-          <t>DDR4: RTX5070進行ATS 組裝@8/20 26PN077002A*100</t>
+          <t>DDR4: RTX5070,8/28正式進入MP</t>
         </is>
       </c>
       <c r="P7" s="11" t="inlineStr">
@@ -1305,7 +1308,7 @@
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
-          <t>1) ATS 組裝@ 8/20, 工單:26PN072477A / 26PN072950A 各50</t>
+          <t>1) 8/28正式進入MP</t>
         </is>
       </c>
       <c r="P10" s="6" t="inlineStr">
@@ -1381,17 +1384,14 @@
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
-          <t>MSI:  MVT DQA test中 微步：ATS ASSY@8/25--會再匯整料況明確組裝時間</t>
+          <t>微步：ATS ASSY@8/27早進行首件組裝, 客驗機器8/28 ready</t>
         </is>
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>1) Function issue： a.	HDI: 8/20提供MP HDI申請單, 8/21開始製作 b.	BIOS: 待8/20 微步提供BIOS 100 , 需驗證bug &amp; 測試完整BIOS Function c.	Long run reboot issue, 5台run 500 loops, 3台hang MSI logo, 微步team正在分析中 (
+          <t>1) Function issue：等8/27 BIOS 102作驗證 a.UCSI充电的OS信息, 驗證在60W的時候, 幾率性不跳OS彈窗 b.	User Password進入BSU, Storage Information &amp; System Information有灰階 c.	AC下无法透过1P15 Docking的LAN唤醒MODS d.	BSU下使用UEFI BIOS update方式有概率更新BIOS fail ME Issue:Drop &amp; Shock(non-OP)測試需使用ATS客驗機器複驗	 (
 2) ATS工單： 9S7-24V111-006*38 9S7-24V111-015*56 (
-3)8月&amp;9月業務訂單認證追蹤 a. DE 9S7-24V111-011* 56 CE認證, 取證時間target 8/E, 具體日期待微步確認中 b. NZ* 76 （9S7-24V111-005* 38+ 9S7-24V111-006 *
-38） RCM認證, CE+ 1 week提供RCM報告, 需進口商登記完成後出貨 c.UA* 112（9S7-24V111-017*56+ 9S7-24V111-015*
-56） Ukraine RF CoC+DoC認證, 由MSI負責申請, UA業務確認follow系統時間排單出貨 d.JP*56(9S7-24V111-009*50+ 9S7-24V111-016*
-6) VCCI認證, 8/E之前可 取證完成, 出貨時間需考量JP鍵盤備料ready日期, 9/E之前可出貨. (
+3)8月&amp;9月業務訂單認證追蹤 a. DE : CE草稿8/27 ready, Review OK後加一周取證 b. NZ: RCM認證, CE+ 1 week提供RCM報告, 需進口商登記完成後出貨 c.UA：Ukraine RF CoC+DoC認證, 由MSI負責申請, UA業務確認follow系統時間排單出貨 d.JP*56: VCCI認證8/26完成, 出貨時間需考量JP鍵盤備料ready日期, 9/E之前可出貨. (
 4) JP KB 開模9/10試模, 9/20交料, JP工單可出貨時間@9/24</t>
         </is>
       </c>
@@ -1468,9 +1468,10 @@
       </c>
       <c r="P12" s="6" t="inlineStr">
         <is>
-          <t>1) Function issue：同24V1, ME issue: a.Panel Mura: 使用COST panel, 微步回復需增加輔料，預抓8/21寄送機器增加Mura對策for MSI驗證 b.	Shock測試fail, B件攝像頭位置彈開&amp;電池定位柱斷裂：需要新的鍵芯支架 複驗, 同時參考26VL機種, 將力度改160G作複測, 樣品可提供時間待微步確認 c.	Panel Scuff測試屏幕碎晶：參考26VL機種, 使用加背包的方式進行模擬複測 d.	Shock測試屏幕破損: 參考26VL機種, 將力度改160G作測試 (
-2) ATS工單: 9S7-26V111-006*20 9S7-26V111-004*200 9S7-26V111-005*400 (
-2) 8月&amp;9月業務訂單認證追蹤 a.DE* 1650 CE認證, 取證時間target 8/E, 具體日期待微步確認中 b.IT 9S7-26V111-002*300 CE認證, 取證時間target 8/E, 具體日期待微步確認中 c.US 9S7-26V111-001*1020 FCC ID， Target 9/M取證(已經拿到FCC報告在內部確認中)  d.PL 9S7-26V111-003*56 CE認證, 取證時間target 8/E, 具體日期待微步確認中</t>
+          <t>1) Function issue：同24V1 (
+2) ATS工單:  9S7-26V111-005*400 (
+2) 8月&amp;9月業務訂單認證追蹤：a. DE&amp;IT&amp;PL : CE草稿8/27 ready, Review OK後加一周取證 b.US: FCC: 報告確認天線位置需修改   ETL認證: 待微步更新進度  ，9/B control number, ETL認證logo圖樣 9/M取證, (
+4) 新增: JP KB開模備料時間待確認, 日本業務期望11月份的訂單</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1486,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Cyborg A15 C1PWE</t>
+          <t>Cyborg A15 Max C1PWF</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -1500,7 +1501,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1541,12 +1542,12 @@
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
-          <t>HPT sku:MVT測試中</t>
+          <t>HPT:MVT測試中</t>
         </is>
       </c>
       <c r="P13" s="6" t="inlineStr">
         <is>
-          <t>1).業務下單要收斂到Cyborg A15 non Max, 因team member已取得Max HPT MVT機台測試中,只會完成MVT測試,Max不開BTO,不做ATS
+          <t>1).8/25 業務通知需專案開BTO,滿足業務已接訂單
 2).Schedule:AMD PI 1200I NDA Release delay(6/19→7/
 28)與生管延後MVT SMT 排程(8/4→8/
 7),累計delay 42天,取消 DVT排程改以 APU Rework 驗證追趕時程後,MP還是會delay 22天至9/22(先前已由 9 /17提前至 8/31,現又延至9/
@@ -1554,84 +1555,82 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+    <row r="14" hidden="1" outlineLevel="1">
+      <c r="A14" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>1T91</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Claw 8 EX AI+ CG3M</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>15TK</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Cyborg A15 C1PWE</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
         <is>
           <t>MVT</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>PTL-H 25W</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>楊淑賢</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>2025/11/06</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>2025/12/16</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>2026/01/31</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>2026/08/26</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>2026/08/18</t>
-        </is>
-      </c>
-      <c r="M14" s="4" t="inlineStr">
-        <is>
-          <t>2026/09/15</t>
-        </is>
-      </c>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>2026/09/30</t>
-        </is>
-      </c>
-      <c r="O14" s="6" t="inlineStr">
-        <is>
-          <t>1. function: 需補測G3+LPDDR5x-32GB的performance/BAT/thermal test, PCBA預抓8/26 SMT
-2)藍色機構件驗證: 8/21樣品到料, ME RD更換4台機器, 8/24 test start</t>
-        </is>
-      </c>
-      <c r="P14" s="6" t="inlineStr">
-        <is>
-          <t>新增藍色SKU G3+ LPDDR5x-32GB需求, 1st MOQ: 3K</t>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>HWK 45W</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5050</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>蔡東宏</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/28</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/26</t>
+        </is>
+      </c>
+      <c r="J14" s="9" t="inlineStr"/>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/07</t>
+        </is>
+      </c>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/21</t>
+        </is>
+      </c>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/12</t>
+        </is>
+      </c>
+      <c r="N14" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/22</t>
+        </is>
+      </c>
+      <c r="O14" s="11" t="inlineStr">
+        <is>
+          <t>HPT:MVT測試中</t>
+        </is>
+      </c>
+      <c r="P14" s="11" t="inlineStr">
+        <is>
+          <t>1).Schedule:AMD PI 1200I NDA Release delay(6/19→7/
+28)與生管延後MVT SMT 排程(8/4→8/
+7),累計delay 42天,取消 DVT排程改以 APU Rework 驗證追趕時程後,MP還是會delay 22天至9/22(先前已由 9 /17提前至 8/31,現又延至9/
+22),後續將依實際測試結果滾動式調整專案時程</t>
         </is>
       </c>
     </row>
@@ -1641,12 +1640,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>14T3</t>
+          <t>1T91</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Prestige N14 AI+ D1M</t>
+          <t>Claw 8 EX AI+ CG3M</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -1656,7 +1655,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>N1 35W</t>
+          <t>PTL-H 25W</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1666,53 +1665,52 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>倪嬌嬌</t>
+          <t>楊淑賢</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>2025/04/30</t>
+          <t>2025/11/06</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>2025/09/01</t>
+          <t>2025/12/16</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>2026/04/15</t>
+          <t>2026/01/31</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>2026/08/13</t>
+          <t>2026/08/26</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>2026/09/14</t>
+          <t>2026/08/18</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026/11/09</t>
+          <t>2026/09/21</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>2026/11/23</t>
+          <t>2026/09/30</t>
         </is>
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>MVT2 SMT depend on PS Software時間-- PS software release@8/21, 可排單日期預抓8/27, 需與MPM討論後確認</t>
+          <t>MVT DQA test中, 8/26-9/11</t>
         </is>
       </c>
       <c r="P15" s="6" t="inlineStr">
         <is>
-          <t>1) Schedule:  a. MVT2 SMT date考量PS software release時間 b. 2.8K panel*286 pcs 8/28 ETD, 廠內庫存不足, 計劃等9/4進料後再作MVT ASSY
-2)備料：量產交料2.8k HQ23, 最新MP*1K交期,  Samsung回復計劃10/E ETD, 可滿足ATS需求, 持續追蹤</t>
+          <t>1）備料: 藍色機構件9/18, update ATS start@9/21</t>
         </is>
       </c>
     </row>
@@ -1722,12 +1720,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2623</t>
+          <t>14T3</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Prestige N16 AI+ C1M</t>
+          <t>Prestige N14 AI+ D1M</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
@@ -1737,7 +1735,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>N1 45W</t>
+          <t>N1 35W</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1747,7 +1745,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>賴雪鳳</t>
+          <t>倪嬌嬌</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1787,12 +1785,12 @@
       </c>
       <c r="O16" s="6" t="inlineStr">
         <is>
-          <t>MVT1:8/13 SMT, 8/14 Pre -Assy  for 少數RD 測試, 待PS SW ready 再上線做MVT2 for 全部team member</t>
+          <t>MVT2 SMT@8/28, MVT ASSY@9/4-- depend on panel交期</t>
         </is>
       </c>
       <c r="P16" s="6" t="inlineStr">
         <is>
-          <t>備料: Samsung 2.8K panel 採購備料HR14*2K for N1 ATS 用, 另外要再驗證HR16 for後續出貨需求</t>
+          <t>1)備料：a. 2.8K panel: MP*1K交期, 計劃10/E ETD, 可滿足ATS需求, 但需持續追蹤DR set測試狀況 b. PCB原材: 1st MOQ1K,目前只先留300 pcs PCB原材for ATS use, 剩餘PCB原材料預估需11/E才能ready, PCB備料L/T 8weeks, PCB交料預估到一月份, 採購持續pull in中</t>
         </is>
       </c>
     </row>
@@ -1802,155 +1800,155 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
+          <t>2623</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Prestige N16 AI+ C1M</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>MVT</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>N1 45W</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>賴雪鳳</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>2025/04/30</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>2025/09/01</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>2026/04/15</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/13</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/14</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/09</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/23</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>MVT1:8/13 SMT, 8/14 Pre -Assy  for 少數RD 測試, 待PS SW ready 再上線做MVT2 for 全部team member</t>
+        </is>
+      </c>
+      <c r="P17" s="6" t="inlineStr">
+        <is>
+          <t>備料: Samsung 2.8K panel 採購備料HR14*2K for N1 ATS 用, 另外要再驗證HR16 for後續出貨需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
           <t>1861</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Katana 18 HX A14WEK</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>RPL-HX refresh 55W</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>RTX 5050</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>顧曉琴</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>2026/05/08</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>2026/06/15</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>2026/08/13</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>2026/10/12</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>2026/11/02</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="M18" s="4" t="inlineStr">
         <is>
           <t>2026/11/21</t>
         </is>
       </c>
-      <c r="N17" s="4" t="inlineStr">
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>2026/11/30</t>
         </is>
       </c>
-      <c r="O17" s="6" t="inlineStr">
-        <is>
-          <t>RPL-HX R + DDR5: EVT SMT1 PCBA預計8/20 到台北供RD測試; SMT2 @ 8/24, Pre-assy @ 8/25, ASSY @ 8/29</t>
-        </is>
-      </c>
-      <c r="P17" s="6" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" hidden="1" outlineLevel="1">
-      <c r="A18" s="7" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>1861</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Katana 18 HX A14WFK</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>EVT</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>RPL-HX refresh 55W</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5060</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>顧曉琴</t>
-        </is>
-      </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I18" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/15</t>
-        </is>
-      </c>
-      <c r="J18" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/13</t>
-        </is>
-      </c>
-      <c r="K18" s="9" t="inlineStr">
-        <is>
-          <t>2026/10/12</t>
-        </is>
-      </c>
-      <c r="L18" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/02</t>
-        </is>
-      </c>
-      <c r="M18" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/21</t>
-        </is>
-      </c>
-      <c r="N18" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/30</t>
-        </is>
-      </c>
-      <c r="O18" s="11" t="inlineStr">
-        <is>
-          <t>RPL-HX R + DDR5: EVT SMT1 PCBA預計8/20 到台北供RD測試; SMT2 @ 8/24, Pre-assy @ 8/25, ASSY @ 8/29</t>
-        </is>
-      </c>
-      <c r="P18" s="11" t="inlineStr">
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>RPL-HX R + DDR5: EVT Pre-assy @ 8/25, ASSY @ 8/29, 預抓9/2提供給DQA測試</t>
+        </is>
+      </c>
+      <c r="P18" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1967,10 +1965,10 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WGK</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
+          <t>Katana 18 HX A14WFK</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -1982,7 +1980,7 @@
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
@@ -2027,7 +2025,7 @@
       </c>
       <c r="O19" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: EVT SMT1 PCBA預計8/20 到台北供RD測試; SMT2 @ 8/24, Pre-assy @ 8/25, ASSY @ 8/29</t>
+          <t>RPL-HX R + DDR5: EVT Pre-assy @ 8/25, ASSY @ 8/29, 預抓9/2提供給DQA測試</t>
         </is>
       </c>
       <c r="P19" s="11" t="inlineStr">
@@ -2047,10 +2045,10 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WGXK</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
+          <t>Katana 18 HX A14WGK</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>EVT</t>
         </is>
@@ -2107,7 +2105,7 @@
       </c>
       <c r="O20" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR5: EVT SMT1 PCBA預計8/20 到台北供RD測試; SMT2 @ 8/24, Pre-assy @ 8/25, ASSY @ 8/29</t>
+          <t>RPL-HX R + DDR5: EVT Pre-assy @ 8/25, ASSY @ 8/29, 預抓9/2提供給DQA測試</t>
         </is>
       </c>
       <c r="P20" s="11" t="inlineStr">
@@ -2127,12 +2125,12 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WEOK</t>
+          <t>Katana 18 HX A14WGXK</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>DVT</t>
+          <t>EVT</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -2142,7 +2140,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
@@ -2152,18 +2150,22 @@
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
+          <t>2026/05/08</t>
         </is>
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
-      <c r="J21" s="9" t="inlineStr"/>
+          <t>2026/06/15</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/13</t>
+        </is>
+      </c>
       <c r="K21" s="9" t="inlineStr">
         <is>
-          <t>2026/10/20</t>
+          <t>2026/10/12</t>
         </is>
       </c>
       <c r="L21" s="9" t="inlineStr">
@@ -2173,22 +2175,22 @@
       </c>
       <c r="M21" s="9" t="inlineStr">
         <is>
-          <t>2026/11/23</t>
+          <t>2026/11/21</t>
         </is>
       </c>
       <c r="N21" s="9" t="inlineStr">
         <is>
-          <t>2026/12/02</t>
+          <t>2026/11/30</t>
         </is>
       </c>
       <c r="O21" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX R + DDR4: DVT test start @ 7/6, 待9/E進版3.1 go MVT</t>
+          <t>RPL-HX R + DDR5: EVT Pre-assy @ 8/25, ASSY @ 8/29, 預抓9/2提供給DQA測試</t>
         </is>
       </c>
       <c r="P21" s="11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -2203,10 +2205,10 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WFOK</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="inlineStr">
+          <t>Katana 18 HX A14WEOK</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2218,7 +2220,7 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
@@ -2279,10 +2281,10 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WGOK</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="inlineStr">
+          <t>Katana 18 HX A14WFOK</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2294,7 +2296,7 @@
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
@@ -2355,10 +2357,10 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A14WGXOK</t>
-        </is>
-      </c>
-      <c r="D24" s="15" t="inlineStr">
+          <t>Katana 18 HX A14WGOK</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -2431,22 +2433,22 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WEK</t>
+          <t>Katana 18 HX A14WGXOK</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>RPL-HX Next 55W</t>
+          <t>RPL-HX refresh 55W</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>RTX 5050</t>
+          <t>RTX 5070</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
@@ -2456,34 +2458,38 @@
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I25" s="9" t="inlineStr"/>
+          <t>2026/05/20</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/27</t>
+        </is>
+      </c>
       <c r="J25" s="9" t="inlineStr"/>
       <c r="K25" s="9" t="inlineStr">
         <is>
-          <t>2026/12/08</t>
+          <t>2026/10/20</t>
         </is>
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/11/02</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>2027/01/19</t>
+          <t>2026/11/23</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>2027/01/30</t>
+          <t>2026/12/02</t>
         </is>
       </c>
       <c r="O25" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX R + DDR4: DVT test start @ 7/6, 待9/E進版3.1 go MVT</t>
         </is>
       </c>
       <c r="P25" s="11" t="inlineStr">
@@ -2503,10 +2509,10 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WEOK</t>
-        </is>
-      </c>
-      <c r="D26" s="16" t="inlineStr">
+          <t>Katana 18 HX A2WEK</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -2528,14 +2534,10 @@
       </c>
       <c r="H26" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
-        </is>
-      </c>
-      <c r="I26" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
+          <t>2026/05/08</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr"/>
       <c r="J26" s="9" t="inlineStr"/>
       <c r="K26" s="9" t="inlineStr">
         <is>
@@ -2559,7 +2561,7 @@
       </c>
       <c r="O26" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P26" s="11" t="inlineStr">
@@ -2579,10 +2581,10 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WFK</t>
-        </is>
-      </c>
-      <c r="D27" s="16" t="inlineStr">
+          <t>Katana 18 HX A2WEOK</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -2594,7 +2596,7 @@
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>RTX 5060</t>
+          <t>RTX 5050</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
@@ -2604,10 +2606,14 @@
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I27" s="9" t="inlineStr"/>
+          <t>2026/05/20</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/27</t>
+        </is>
+      </c>
       <c r="J27" s="9" t="inlineStr"/>
       <c r="K27" s="9" t="inlineStr">
         <is>
@@ -2631,7 +2637,7 @@
       </c>
       <c r="O27" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P27" s="11" t="inlineStr">
@@ -2651,10 +2657,10 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WFOK</t>
-        </is>
-      </c>
-      <c r="D28" s="16" t="inlineStr">
+          <t>Katana 18 HX A2WFK</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -2676,14 +2682,10 @@
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
-        </is>
-      </c>
-      <c r="I28" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
+          <t>2026/05/08</t>
+        </is>
+      </c>
+      <c r="I28" s="9" t="inlineStr"/>
       <c r="J28" s="9" t="inlineStr"/>
       <c r="K28" s="9" t="inlineStr">
         <is>
@@ -2707,7 +2709,7 @@
       </c>
       <c r="O28" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P28" s="11" t="inlineStr">
@@ -2727,10 +2729,10 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WGK</t>
-        </is>
-      </c>
-      <c r="D29" s="16" t="inlineStr">
+          <t>Katana 18 HX A2WFOK</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -2742,7 +2744,7 @@
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
@@ -2752,10 +2754,14 @@
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I29" s="9" t="inlineStr"/>
+          <t>2026/05/20</t>
+        </is>
+      </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/27</t>
+        </is>
+      </c>
       <c r="J29" s="9" t="inlineStr"/>
       <c r="K29" s="9" t="inlineStr">
         <is>
@@ -2779,7 +2785,7 @@
       </c>
       <c r="O29" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P29" s="11" t="inlineStr">
@@ -2799,10 +2805,10 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WGOK</t>
-        </is>
-      </c>
-      <c r="D30" s="16" t="inlineStr">
+          <t>Katana 18 HX A2WGK</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -2824,14 +2830,10 @@
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
-        </is>
-      </c>
-      <c r="I30" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
+          <t>2026/05/08</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr"/>
       <c r="J30" s="9" t="inlineStr"/>
       <c r="K30" s="9" t="inlineStr">
         <is>
@@ -2855,7 +2857,7 @@
       </c>
       <c r="O30" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P30" s="11" t="inlineStr">
@@ -2875,10 +2877,10 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WGXK</t>
-        </is>
-      </c>
-      <c r="D31" s="16" t="inlineStr">
+          <t>Katana 18 HX A2WGOK</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -2900,10 +2902,14 @@
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>2026/05/08</t>
-        </is>
-      </c>
-      <c r="I31" s="9" t="inlineStr"/>
+          <t>2026/05/20</t>
+        </is>
+      </c>
+      <c r="I31" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/27</t>
+        </is>
+      </c>
       <c r="J31" s="9" t="inlineStr"/>
       <c r="K31" s="9" t="inlineStr">
         <is>
@@ -2927,7 +2933,7 @@
       </c>
       <c r="O31" s="11" t="inlineStr">
         <is>
-          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+          <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
       <c r="P31" s="11" t="inlineStr">
@@ -2947,10 +2953,10 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Katana 18 HX A2WGXOK</t>
-        </is>
-      </c>
-      <c r="D32" s="16" t="inlineStr">
+          <t>Katana 18 HX A2WGXK</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -2972,14 +2978,10 @@
       </c>
       <c r="H32" s="9" t="inlineStr">
         <is>
-          <t>2026/05/20</t>
-        </is>
-      </c>
-      <c r="I32" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/27</t>
-        </is>
-      </c>
+          <t>2026/05/08</t>
+        </is>
+      </c>
+      <c r="I32" s="9" t="inlineStr"/>
       <c r="J32" s="9" t="inlineStr"/>
       <c r="K32" s="9" t="inlineStr">
         <is>
@@ -3003,92 +3005,88 @@
       </c>
       <c r="O32" s="11" t="inlineStr">
         <is>
+          <t>RPL-HX Next + DDR5: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
+        </is>
+      </c>
+      <c r="P32" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" hidden="1" outlineLevel="1">
+      <c r="A33" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>1861</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Katana 18 HX A2WGXOK</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>RPL-HX Next 55W</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>顧曉琴</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/20</t>
+        </is>
+      </c>
+      <c r="I33" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/27</t>
+        </is>
+      </c>
+      <c r="J33" s="9" t="inlineStr"/>
+      <c r="K33" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/08</t>
+        </is>
+      </c>
+      <c r="L33" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/30</t>
+        </is>
+      </c>
+      <c r="M33" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/19</t>
+        </is>
+      </c>
+      <c r="N33" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/30</t>
+        </is>
+      </c>
+      <c r="O33" s="11" t="inlineStr">
+        <is>
           <t>RPL-HX Next+ DDR4: follow RPL HX Refresh, 待RPL HX Next QS sample WW49到料後安排MVT</t>
         </is>
       </c>
-      <c r="P32" s="11" t="inlineStr">
+      <c r="P33" s="11" t="inlineStr">
         <is>
           <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>13Q5</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Prestige 13 AI+ A4M</t>
-        </is>
-      </c>
-      <c r="D33" s="17" t="inlineStr">
-        <is>
-          <t>DVT</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>NVL-H 28W</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Intel® Arc™ Graphics</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>顏春梅</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>2026/06/29</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>2026/08/18</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>2026/10/08</t>
-        </is>
-      </c>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/21</t>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/22</t>
-        </is>
-      </c>
-      <c r="M33" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/22</t>
-        </is>
-      </c>
-      <c r="N33" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/31</t>
-        </is>
-      </c>
-      <c r="O33" s="6" t="inlineStr">
-        <is>
-          <t>DVT PCBA 調撥回台@8/21</t>
-        </is>
-      </c>
-      <c r="P33" s="6" t="inlineStr">
-        <is>
-          <t>NA</t>
         </is>
       </c>
     </row>
@@ -3098,469 +3096,469 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
+          <t>13Q5</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Prestige 13 AI+ A4M</t>
+        </is>
+      </c>
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>NVL-H 28W</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Intel® Arc™ Graphics</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>顏春梅</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>2026/06/29</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/18</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>2026/10/08</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/21</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/22</t>
+        </is>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/22</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/31</t>
+        </is>
+      </c>
+      <c r="O34" s="6" t="inlineStr">
+        <is>
+          <t>DVT RD 測試中</t>
+        </is>
+      </c>
+      <c r="P34" s="6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
           <t>14T4</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Prestige 14 AI+ D4MG</t>
         </is>
       </c>
-      <c r="D34" s="17" t="inlineStr">
+      <c r="D35" s="18" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>NVL-H 30W</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>Intel® Arc™ Graphics</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>朱芳芳</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>2026/05/14</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I35" s="4" t="inlineStr">
         <is>
           <t>2026/07/27</t>
         </is>
       </c>
-      <c r="J34" s="4" t="inlineStr">
+      <c r="J35" s="4" t="inlineStr">
         <is>
           <t>2026/09/22</t>
         </is>
       </c>
-      <c r="K34" s="4" t="inlineStr">
+      <c r="K35" s="4" t="inlineStr">
         <is>
           <t>2026/11/12</t>
         </is>
       </c>
-      <c r="L34" s="4" t="inlineStr">
+      <c r="L35" s="4" t="inlineStr">
         <is>
           <t>2026/11/20</t>
         </is>
       </c>
-      <c r="M34" s="4" t="inlineStr">
+      <c r="M35" s="4" t="inlineStr">
         <is>
           <t>2026/12/21</t>
         </is>
       </c>
-      <c r="N34" s="4" t="inlineStr">
+      <c r="N35" s="4" t="inlineStr">
         <is>
           <t>2026/12/31</t>
         </is>
       </c>
-      <c r="O34" s="6" t="inlineStr">
-        <is>
-          <t>DVT RD test中 :8/4~9/7</t>
-        </is>
-      </c>
-      <c r="P34" s="6" t="inlineStr">
+      <c r="O35" s="6" t="inlineStr">
+        <is>
+          <t>DVT RD test中 :8/4~9/7，9/7 0B gerberout</t>
+        </is>
+      </c>
+      <c r="P35" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="35" hidden="1" outlineLevel="1">
-      <c r="A35" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
+    <row r="36" hidden="1" outlineLevel="1">
+      <c r="A36" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>14T4</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>Prestige 14 Flip AI+ D4MTG</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
+      <c r="D36" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E36" s="9" t="inlineStr">
         <is>
           <t>NVL-H 30W</t>
         </is>
       </c>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="F36" s="9" t="inlineStr">
         <is>
           <t>Intel® Arc™ Graphics</t>
         </is>
       </c>
-      <c r="G35" s="9" t="inlineStr">
+      <c r="G36" s="9" t="inlineStr">
         <is>
           <t>朱芳芳</t>
         </is>
       </c>
-      <c r="H35" s="9" t="inlineStr">
+      <c r="H36" s="9" t="inlineStr">
         <is>
           <t>2026/05/14</t>
         </is>
       </c>
-      <c r="I35" s="9" t="inlineStr">
+      <c r="I36" s="9" t="inlineStr">
         <is>
           <t>2026/07/27</t>
         </is>
       </c>
-      <c r="J35" s="9" t="inlineStr">
+      <c r="J36" s="9" t="inlineStr">
         <is>
           <t>2026/09/22</t>
         </is>
       </c>
-      <c r="K35" s="9" t="inlineStr">
+      <c r="K36" s="9" t="inlineStr">
         <is>
           <t>2026/11/12</t>
         </is>
       </c>
-      <c r="L35" s="9" t="inlineStr">
+      <c r="L36" s="9" t="inlineStr">
         <is>
           <t>2026/11/20</t>
         </is>
       </c>
-      <c r="M35" s="9" t="inlineStr">
+      <c r="M36" s="9" t="inlineStr">
         <is>
           <t>2026/12/21</t>
         </is>
       </c>
-      <c r="N35" s="9" t="inlineStr">
+      <c r="N36" s="9" t="inlineStr">
         <is>
           <t>2026/12/31</t>
         </is>
       </c>
-      <c r="O35" s="11" t="inlineStr">
-        <is>
-          <t>DVT RD test中 :8/4~9/7</t>
-        </is>
-      </c>
-      <c r="P35" s="11" t="inlineStr">
+      <c r="O36" s="11" t="inlineStr">
+        <is>
+          <t>DVT RD test中 :8/4~9/7，9/7 0B gerberout</t>
+        </is>
+      </c>
+      <c r="P36" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>2624</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>Prestige 16 AI+</t>
         </is>
       </c>
-      <c r="D36" s="17" t="inlineStr">
+      <c r="D37" s="18" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>NVL-H 30W</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>Intel® Arc™ Graphics</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G37" s="4" t="inlineStr">
         <is>
           <t>朱芳芳</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="H37" s="4" t="inlineStr">
         <is>
           <t>2026/05/14</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr"/>
-      <c r="J36" s="4" t="inlineStr">
+      <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="4" t="inlineStr">
         <is>
           <t>2026/09/22</t>
         </is>
       </c>
-      <c r="K36" s="4" t="inlineStr">
+      <c r="K37" s="4" t="inlineStr">
         <is>
           <t>2026/11/12</t>
         </is>
       </c>
-      <c r="L36" s="4" t="inlineStr">
+      <c r="L37" s="4" t="inlineStr">
         <is>
           <t>2026/11/20</t>
         </is>
       </c>
-      <c r="M36" s="4" t="inlineStr">
+      <c r="M37" s="4" t="inlineStr">
         <is>
           <t>2026/12/21</t>
         </is>
       </c>
-      <c r="N36" s="4" t="inlineStr">
+      <c r="N37" s="4" t="inlineStr">
         <is>
           <t>2026/12/31</t>
         </is>
       </c>
-      <c r="O36" s="6" t="inlineStr">
-        <is>
-          <t>DVT RD test中 :8/4~9/7</t>
-        </is>
-      </c>
-      <c r="P36" s="6" t="inlineStr">
+      <c r="O37" s="6" t="inlineStr">
+        <is>
+          <t>DVT RD test中 :8/4~9/7，9/7 0B gerberout</t>
+        </is>
+      </c>
+      <c r="P37" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="37" hidden="1" outlineLevel="1">
-      <c r="A37" s="7" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="8" t="inlineStr">
+    <row r="38" hidden="1" outlineLevel="1">
+      <c r="A38" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>2624</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>Prestige 16 Flip AI+</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
+      <c r="D38" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>NVL-H 30W</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="F38" s="9" t="inlineStr">
         <is>
           <t>Intel® Arc™ Graphics</t>
         </is>
       </c>
-      <c r="G37" s="9" t="inlineStr">
+      <c r="G38" s="9" t="inlineStr">
         <is>
           <t>朱芳芳</t>
         </is>
       </c>
-      <c r="H37" s="9" t="inlineStr">
+      <c r="H38" s="9" t="inlineStr">
         <is>
           <t>2026/05/14</t>
         </is>
       </c>
-      <c r="I37" s="9" t="inlineStr"/>
-      <c r="J37" s="9" t="inlineStr">
+      <c r="I38" s="9" t="inlineStr"/>
+      <c r="J38" s="9" t="inlineStr">
         <is>
           <t>2026/09/22</t>
         </is>
       </c>
-      <c r="K37" s="9" t="inlineStr">
+      <c r="K38" s="9" t="inlineStr">
         <is>
           <t>2026/11/12</t>
         </is>
       </c>
-      <c r="L37" s="9" t="inlineStr">
+      <c r="L38" s="9" t="inlineStr">
         <is>
           <t>2026/11/20</t>
         </is>
       </c>
-      <c r="M37" s="9" t="inlineStr">
+      <c r="M38" s="9" t="inlineStr">
         <is>
           <t>2026/12/21</t>
         </is>
       </c>
-      <c r="N37" s="9" t="inlineStr">
+      <c r="N38" s="9" t="inlineStr">
         <is>
           <t>2026/12/31</t>
         </is>
       </c>
-      <c r="O37" s="11" t="inlineStr">
-        <is>
-          <t>DVT RD test中 :8/4~9/7</t>
-        </is>
-      </c>
-      <c r="P37" s="11" t="inlineStr">
+      <c r="O38" s="11" t="inlineStr">
+        <is>
+          <t>DVT RD test中 :8/4~9/7，9/7 0B gerberout</t>
+        </is>
+      </c>
+      <c r="P38" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>2633</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Stealth 16 AI+ B4WI</t>
         </is>
       </c>
-      <c r="D38" s="17" t="inlineStr">
+      <c r="D39" s="18" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F39" s="4" t="inlineStr">
         <is>
           <t>RTX 5080</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>朱欣怡</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="H39" s="4" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I38" s="4" t="inlineStr">
+      <c r="I39" s="4" t="inlineStr">
         <is>
           <t>2026/07/23</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr">
+      <c r="J39" s="4" t="inlineStr">
         <is>
           <t>2026/09/16</t>
         </is>
       </c>
-      <c r="K38" s="4" t="inlineStr">
+      <c r="K39" s="4" t="inlineStr">
         <is>
           <t>2026/11/11</t>
         </is>
       </c>
-      <c r="L38" s="4" t="inlineStr">
+      <c r="L39" s="4" t="inlineStr">
         <is>
           <t>2026/11/30</t>
         </is>
       </c>
-      <c r="M38" s="4" t="inlineStr">
+      <c r="M39" s="4" t="inlineStr">
         <is>
           <t>2026/12/29</t>
         </is>
       </c>
-      <c r="N38" s="4" t="inlineStr">
+      <c r="N39" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="O38" s="6" t="inlineStr">
+      <c r="O39" s="6" t="inlineStr">
         <is>
           <t>RD 測試中, 0N gerberout @8/25</t>
         </is>
       </c>
-      <c r="P38" s="6" t="inlineStr">
+      <c r="P39" s="6" t="inlineStr">
         <is>
           <t>1) Schedule:NV VBIOS @1/6, gating 8天,預計12/E 拿到WHQL，可能影響到最終TTM 時間</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" hidden="1" outlineLevel="1">
-      <c r="A39" s="7" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>2633</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WH</t>
-        </is>
-      </c>
-      <c r="D39" s="15" t="inlineStr">
-        <is>
-          <t>DVT</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 45W</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5070Ti</t>
-        </is>
-      </c>
-      <c r="G39" s="9" t="inlineStr">
-        <is>
-          <t>朱欣怡</t>
-        </is>
-      </c>
-      <c r="H39" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/22</t>
-        </is>
-      </c>
-      <c r="I39" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/23</t>
-        </is>
-      </c>
-      <c r="J39" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/16</t>
-        </is>
-      </c>
-      <c r="K39" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/11</t>
-        </is>
-      </c>
-      <c r="L39" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/30</t>
-        </is>
-      </c>
-      <c r="M39" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/29</t>
-        </is>
-      </c>
-      <c r="N39" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="O39" s="11" t="inlineStr">
-        <is>
-          <t>RD 測試中, 0N gerberout @8/25</t>
-        </is>
-      </c>
-      <c r="P39" s="11" t="inlineStr">
-        <is>
-          <t>NA</t>
         </is>
       </c>
     </row>
@@ -3575,231 +3573,230 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
+          <t>Stealth 16 AI+ B4WH</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>NVL-H 45W</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070Ti</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>朱欣怡</t>
+        </is>
+      </c>
+      <c r="H40" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="I40" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/23</t>
+        </is>
+      </c>
+      <c r="J40" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/16</t>
+        </is>
+      </c>
+      <c r="K40" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/11</t>
+        </is>
+      </c>
+      <c r="L40" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/30</t>
+        </is>
+      </c>
+      <c r="M40" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/29</t>
+        </is>
+      </c>
+      <c r="N40" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="O40" s="11" t="inlineStr">
+        <is>
+          <t>RD 測試中, 0N gerberout @8/25</t>
+        </is>
+      </c>
+      <c r="P40" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" hidden="1" outlineLevel="1">
+      <c r="A41" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>2633</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
           <t>Stealth 16 AI+ B4WJ</t>
         </is>
       </c>
-      <c r="D40" s="15" t="inlineStr">
+      <c r="D41" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E40" s="9" t="inlineStr">
+      <c r="E41" s="9" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F40" s="9" t="inlineStr">
+      <c r="F41" s="9" t="inlineStr">
         <is>
           <t>RTX 5090</t>
         </is>
       </c>
-      <c r="G40" s="9" t="inlineStr">
+      <c r="G41" s="9" t="inlineStr">
         <is>
           <t>朱欣怡</t>
         </is>
       </c>
-      <c r="H40" s="9" t="inlineStr">
+      <c r="H41" s="9" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I40" s="9" t="inlineStr">
+      <c r="I41" s="9" t="inlineStr">
         <is>
           <t>2026/07/23</t>
         </is>
       </c>
-      <c r="J40" s="9" t="inlineStr">
+      <c r="J41" s="9" t="inlineStr">
         <is>
           <t>2026/09/16</t>
         </is>
       </c>
-      <c r="K40" s="9" t="inlineStr">
+      <c r="K41" s="9" t="inlineStr">
         <is>
           <t>2026/11/11</t>
         </is>
       </c>
-      <c r="L40" s="9" t="inlineStr">
+      <c r="L41" s="9" t="inlineStr">
         <is>
           <t>2026/11/30</t>
         </is>
       </c>
-      <c r="M40" s="9" t="inlineStr">
+      <c r="M41" s="9" t="inlineStr">
         <is>
           <t>2026/12/29</t>
         </is>
       </c>
-      <c r="N40" s="9" t="inlineStr">
+      <c r="N41" s="9" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="O40" s="11" t="inlineStr">
+      <c r="O41" s="11" t="inlineStr">
         <is>
           <t>RD 測試中, 0N gerberout @8/25</t>
         </is>
       </c>
-      <c r="P40" s="11" t="inlineStr">
+      <c r="P41" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>2634</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Stealth 16 AI+ B4WE</t>
         </is>
       </c>
-      <c r="D41" s="17" t="inlineStr">
+      <c r="D42" s="18" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>NVL-H 45W</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>RTX 5050</t>
         </is>
       </c>
-      <c r="G41" s="4" t="inlineStr">
+      <c r="G42" s="4" t="inlineStr">
         <is>
           <t>賴雪鳳</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="H42" s="4" t="inlineStr">
         <is>
           <t>2026/05/22</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="I42" s="4" t="inlineStr">
         <is>
           <t>2026/07/31</t>
         </is>
       </c>
-      <c r="J41" s="4" t="inlineStr">
+      <c r="J42" s="4" t="inlineStr">
         <is>
           <t>2026/09/16</t>
         </is>
       </c>
-      <c r="K41" s="4" t="inlineStr">
+      <c r="K42" s="4" t="inlineStr">
         <is>
           <t>2026/11/11</t>
         </is>
       </c>
-      <c r="L41" s="4" t="inlineStr">
+      <c r="L42" s="4" t="inlineStr">
         <is>
           <t>2026/11/27</t>
         </is>
       </c>
-      <c r="M41" s="4" t="inlineStr">
+      <c r="M42" s="4" t="inlineStr">
         <is>
           <t>2026/12/29</t>
         </is>
       </c>
-      <c r="N41" s="4" t="inlineStr">
+      <c r="N42" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="O41" s="6" t="inlineStr">
+      <c r="O42" s="6" t="inlineStr">
         <is>
           <t>0A PCBA DVT 驗證中,預計9/2 0B 出圖</t>
         </is>
       </c>
-      <c r="P41" s="6" t="inlineStr">
-        <is>
-          <t>1)NV VBIOS 驗證時間6周
-2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" hidden="1" outlineLevel="1">
-      <c r="A42" s="7" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>2634</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="inlineStr">
-        <is>
-          <t>Stealth 16 AI+ B4WF</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>DVT</t>
-        </is>
-      </c>
-      <c r="E42" s="9" t="inlineStr">
-        <is>
-          <t>NVL-H 45W</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5060</t>
-        </is>
-      </c>
-      <c r="G42" s="9" t="inlineStr">
-        <is>
-          <t>賴雪鳳</t>
-        </is>
-      </c>
-      <c r="H42" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/22</t>
-        </is>
-      </c>
-      <c r="I42" s="9" t="inlineStr">
-        <is>
-          <t>2026/07/31</t>
-        </is>
-      </c>
-      <c r="J42" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/16</t>
-        </is>
-      </c>
-      <c r="K42" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/11</t>
-        </is>
-      </c>
-      <c r="L42" s="9" t="inlineStr">
-        <is>
-          <t>2026/11/27</t>
-        </is>
-      </c>
-      <c r="M42" s="9" t="inlineStr">
-        <is>
-          <t>2026/12/29</t>
-        </is>
-      </c>
-      <c r="N42" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="O42" s="11" t="inlineStr">
-        <is>
-          <t>0A PCBA DVT 驗證中,預計9/2 0B 出圖</t>
-        </is>
-      </c>
-      <c r="P42" s="11" t="inlineStr">
+      <c r="P42" s="6" t="inlineStr">
         <is>
           <t>1)NV VBIOS 驗證時間6周
 2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
@@ -3817,10 +3814,10 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
-        </is>
-      </c>
-      <c r="D43" s="15" t="inlineStr">
+          <t>Stealth 16 AI+ B4WF</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3832,7 +3829,7 @@
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
@@ -3898,10 +3895,10 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
-        </is>
-      </c>
-      <c r="D44" s="15" t="inlineStr">
+          <t>Stealth 16 AI+ B4WG/GD7 8GB</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -3968,83 +3965,84 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="2" t="n">
+    <row r="45" hidden="1" outlineLevel="1">
+      <c r="A45" s="7" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>14W1</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Modern 14S H3M</t>
-        </is>
-      </c>
-      <c r="D45" s="18" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>WCL 25W</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Intel® graphics</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>許婕</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>2026/08/11</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>2026/09/28</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>2026/11/10</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/10</t>
-        </is>
-      </c>
-      <c r="L45" s="4" t="inlineStr">
-        <is>
-          <t>2026/12/15</t>
-        </is>
-      </c>
-      <c r="M45" s="4" t="inlineStr">
-        <is>
-          <t>2027/01/12</t>
-        </is>
-      </c>
-      <c r="N45" s="4" t="inlineStr">
-        <is>
-          <t>2027/01/22</t>
-        </is>
-      </c>
-      <c r="O45" s="6" t="inlineStr">
-        <is>
-          <t>8/11 已kick off，预计9/14 0A gerberout</t>
-        </is>
-      </c>
-      <c r="P45" s="6" t="inlineStr">
-        <is>
-          <t>BOE FHD 120Hz panel MP料交期16w-20w，RD回復需等EVT 測試結束視結果備MP料，MP料最快到料時間3/E，機種MP 4/M，與target gap 2.5M</t>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>2634</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Stealth 16 AI+ B4WGX/GD7 12GB</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>NVL-H 45W</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>賴雪鳳</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="I45" s="9" t="inlineStr">
+        <is>
+          <t>2026/07/31</t>
+        </is>
+      </c>
+      <c r="J45" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/16</t>
+        </is>
+      </c>
+      <c r="K45" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/11</t>
+        </is>
+      </c>
+      <c r="L45" s="9" t="inlineStr">
+        <is>
+          <t>2026/11/27</t>
+        </is>
+      </c>
+      <c r="M45" s="9" t="inlineStr">
+        <is>
+          <t>2026/12/29</t>
+        </is>
+      </c>
+      <c r="N45" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="O45" s="11" t="inlineStr">
+        <is>
+          <t>0A PCBA DVT 驗證中,預計9/2 0B 出圖</t>
+        </is>
+      </c>
+      <c r="P45" s="11" t="inlineStr">
+        <is>
+          <t>1)NV VBIOS 驗證時間6周
+2)Intel WHQL :12/E 拿到 可能影響到最終TTM 時間</t>
         </is>
       </c>
     </row>
@@ -4054,15 +4052,15 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>2661</t>
+          <t>14W1</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Modern 16S H3M</t>
-        </is>
-      </c>
-      <c r="D46" s="18" t="inlineStr">
+          <t>Modern 14S H3M</t>
+        </is>
+      </c>
+      <c r="D46" s="19" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
@@ -4119,12 +4117,12 @@
       </c>
       <c r="O46" s="6" t="inlineStr">
         <is>
-          <t>leverage Modern 14S H3M</t>
+          <t>8/11 已kick off，预计9/14 0A gerberout</t>
         </is>
       </c>
       <c r="P46" s="6" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>BOE FHD 120Hz panel MP料交期16w-20w，RD回復需等EVT 測試結束視結果備MP料，MP料最快到料時間3/E，機種MP 4/M，與target gap 2.5M</t>
         </is>
       </c>
     </row>
@@ -4134,155 +4132,155 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
+          <t>2661</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Modern 16S H3M</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>WCL 25W</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Intel® graphics</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>許婕</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>2026/08/11</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>2026/09/28</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>2026/11/10</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/10</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>2026/12/15</t>
+        </is>
+      </c>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/12</t>
+        </is>
+      </c>
+      <c r="N47" s="4" t="inlineStr">
+        <is>
+          <t>2027/01/22</t>
+        </is>
+      </c>
+      <c r="O47" s="6" t="inlineStr">
+        <is>
+          <t>leverage Modern 14S H3M</t>
+        </is>
+      </c>
+      <c r="P47" s="6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
           <t>2654</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Raider 16 Max HX B4WH</t>
         </is>
       </c>
-      <c r="D47" s="17" t="inlineStr">
+      <c r="D48" s="18" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>RTX 5070Ti</t>
         </is>
       </c>
-      <c r="G47" s="4" t="inlineStr">
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>吳美芳</t>
         </is>
       </c>
-      <c r="H47" s="4" t="inlineStr">
+      <c r="H48" s="4" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I47" s="4" t="inlineStr">
+      <c r="I48" s="4" t="inlineStr">
         <is>
           <t>2026/08/05</t>
         </is>
       </c>
-      <c r="J47" s="4" t="inlineStr">
+      <c r="J48" s="4" t="inlineStr">
         <is>
           <t>2026/09/29</t>
         </is>
       </c>
-      <c r="K47" s="4" t="inlineStr">
+      <c r="K48" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L47" s="4" t="inlineStr">
+      <c r="L48" s="4" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M47" s="4" t="inlineStr">
+      <c r="M48" s="4" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N47" s="4" t="inlineStr">
+      <c r="N48" s="4" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O47" s="6" t="inlineStr">
+      <c r="O48" s="6" t="inlineStr">
         <is>
           <t>DVT RD測試中8/14~9/11，預計9/11 0N出圖</t>
         </is>
       </c>
-      <c r="P47" s="6" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" hidden="1" outlineLevel="1">
-      <c r="A48" s="7" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>2654</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>Raider 16 Max HX B4WI</t>
-        </is>
-      </c>
-      <c r="D48" s="15" t="inlineStr">
-        <is>
-          <t>DVT</t>
-        </is>
-      </c>
-      <c r="E48" s="9" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5080</t>
-        </is>
-      </c>
-      <c r="G48" s="9" t="inlineStr">
-        <is>
-          <t>吳美芳</t>
-        </is>
-      </c>
-      <c r="H48" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/19</t>
-        </is>
-      </c>
-      <c r="I48" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/05</t>
-        </is>
-      </c>
-      <c r="J48" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/29</t>
-        </is>
-      </c>
-      <c r="K48" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="L48" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/02</t>
-        </is>
-      </c>
-      <c r="M48" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/08</t>
-        </is>
-      </c>
-      <c r="N48" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/18</t>
-        </is>
-      </c>
-      <c r="O48" s="11" t="inlineStr">
-        <is>
-          <t>DVT RD測試中8/14~9/11，預計9/11 0N出圖</t>
-        </is>
-      </c>
-      <c r="P48" s="11" t="inlineStr">
+      <c r="P48" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -4299,230 +4297,230 @@
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
+          <t>Raider 16 Max HX B4WI</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5080</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>吳美芳</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/19</t>
+        </is>
+      </c>
+      <c r="I49" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/05</t>
+        </is>
+      </c>
+      <c r="J49" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/29</t>
+        </is>
+      </c>
+      <c r="K49" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="L49" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/02</t>
+        </is>
+      </c>
+      <c r="M49" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N49" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O49" s="11" t="inlineStr">
+        <is>
+          <t>DVT RD測試中8/14~9/11，預計9/11 0N出圖</t>
+        </is>
+      </c>
+      <c r="P49" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" hidden="1" outlineLevel="1">
+      <c r="A50" s="7" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>2654</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
           <t>Raider 16 Max HX B4WJ</t>
         </is>
       </c>
-      <c r="D49" s="15" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E49" s="9" t="inlineStr">
+      <c r="E50" s="9" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F49" s="9" t="inlineStr">
+      <c r="F50" s="9" t="inlineStr">
         <is>
           <t>RTX 5090</t>
         </is>
       </c>
-      <c r="G49" s="9" t="inlineStr">
+      <c r="G50" s="9" t="inlineStr">
         <is>
           <t>吳美芳</t>
         </is>
       </c>
-      <c r="H49" s="9" t="inlineStr">
+      <c r="H50" s="9" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I49" s="9" t="inlineStr">
+      <c r="I50" s="9" t="inlineStr">
         <is>
           <t>2026/08/05</t>
         </is>
       </c>
-      <c r="J49" s="9" t="inlineStr">
+      <c r="J50" s="9" t="inlineStr">
         <is>
           <t>2026/09/29</t>
         </is>
       </c>
-      <c r="K49" s="9" t="inlineStr">
+      <c r="K50" s="9" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L49" s="9" t="inlineStr">
+      <c r="L50" s="9" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M49" s="9" t="inlineStr">
+      <c r="M50" s="9" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N49" s="9" t="inlineStr">
+      <c r="N50" s="9" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O49" s="11" t="inlineStr">
+      <c r="O50" s="11" t="inlineStr">
         <is>
           <t>DVT RD測試中8/14~9/11，預計9/11 0N出圖</t>
         </is>
       </c>
-      <c r="P49" s="11" t="inlineStr">
+      <c r="P50" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>1851</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Titan 18 HX B4WH</t>
         </is>
       </c>
-      <c r="D50" s="18" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="D51" s="18" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="F51" s="4" t="inlineStr">
         <is>
           <t>RTX 5070Ti</t>
         </is>
       </c>
-      <c r="G50" s="4" t="inlineStr">
+      <c r="G51" s="4" t="inlineStr">
         <is>
           <t>高宇奇</t>
         </is>
       </c>
-      <c r="H50" s="4" t="inlineStr">
+      <c r="H51" s="4" t="inlineStr">
         <is>
           <t>2026/06/29</t>
         </is>
       </c>
-      <c r="I50" s="4" t="inlineStr">
+      <c r="I51" s="4" t="inlineStr">
         <is>
           <t>2026/08/19</t>
         </is>
       </c>
-      <c r="J50" s="4" t="inlineStr">
+      <c r="J51" s="4" t="inlineStr">
         <is>
           <t>2026/10/23</t>
         </is>
       </c>
-      <c r="K50" s="4" t="inlineStr">
+      <c r="K51" s="4" t="inlineStr">
         <is>
           <t>2027/01/08</t>
         </is>
       </c>
-      <c r="L50" s="4" t="inlineStr">
+      <c r="L51" s="4" t="inlineStr">
         <is>
           <t>2027/02/01</t>
         </is>
       </c>
-      <c r="M50" s="4" t="inlineStr">
+      <c r="M51" s="4" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N50" s="4" t="inlineStr">
+      <c r="N51" s="4" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O50" s="6" t="inlineStr">
-        <is>
-          <t>1) 根據料況及排程,已安排8/19 DVT上線SMT,打板後不測試立即入庫調撥,Target 8/24 for台北RD測試開機.</t>
-        </is>
-      </c>
-      <c r="P50" s="6" t="inlineStr">
-        <is>
-          <t>1) 根據SSE POC會議討論共識,1851最後採用2顆MCU架構for所有的發光device,並且根據SSE提出的建議,第1顆MCU控制Per key KB,另1顆MCU控制其餘所有發光device,預計9月初提供1台1851 mockup系統for SSE FW implement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" hidden="1" outlineLevel="1">
-      <c r="A51" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>1851</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>Titan 18 HX B4WI</t>
-        </is>
-      </c>
-      <c r="D51" s="16" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E51" s="9" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5080</t>
-        </is>
-      </c>
-      <c r="G51" s="9" t="inlineStr">
-        <is>
-          <t>高宇奇</t>
-        </is>
-      </c>
-      <c r="H51" s="9" t="inlineStr">
-        <is>
-          <t>2026/06/29</t>
-        </is>
-      </c>
-      <c r="I51" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/19</t>
-        </is>
-      </c>
-      <c r="J51" s="9" t="inlineStr">
-        <is>
-          <t>2026/10/23</t>
-        </is>
-      </c>
-      <c r="K51" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/08</t>
-        </is>
-      </c>
-      <c r="L51" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/01</t>
-        </is>
-      </c>
-      <c r="M51" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/08</t>
-        </is>
-      </c>
-      <c r="N51" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/18</t>
-        </is>
-      </c>
-      <c r="O51" s="11" t="inlineStr">
-        <is>
-          <t>1) 根據料況及排程,已安排8/19 DVT上線SMT,打板後不測試立即入庫調撥,Target 8/24 for台北RD測試開機.</t>
-        </is>
-      </c>
-      <c r="P51" s="11" t="inlineStr">
+      <c r="O51" s="6" t="inlineStr">
+        <is>
+          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
+        </is>
+      </c>
+      <c r="P51" s="6" t="inlineStr">
         <is>
           <t>1) 根據SSE POC會議討論共識,1851最後採用2顆MCU架構for所有的發光device,並且根據SSE提出的建議,第1顆MCU控制Per key KB,另1顆MCU控制其餘所有發光device,預計9月初提供1台1851 mockup系統for SSE FW implement.</t>
         </is>
@@ -4539,12 +4537,12 @@
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>Titan 18 HX B4WJ</t>
+          <t>Titan 18 HX B4WI</t>
         </is>
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
@@ -4554,7 +4552,7 @@
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>RTX 5090</t>
+          <t>RTX 5080</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
@@ -4599,7 +4597,7 @@
       </c>
       <c r="O52" s="11" t="inlineStr">
         <is>
-          <t>1) 根據料況及排程,已安排8/19 DVT上線SMT,打板後不測試立即入庫調撥,Target 8/24 for台北RD測試開機.</t>
+          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
         </is>
       </c>
       <c r="P52" s="11" t="inlineStr">
@@ -4619,22 +4617,22 @@
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>Raider 18 Max HX B4WH</t>
+          <t>Titan 18 HX B4WJ</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>NVL-HX 65W</t>
+          <t>NVL-HX 55W</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070Ti</t>
+          <t>RTX 5090</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
@@ -4679,7 +4677,7 @@
       </c>
       <c r="O53" s="11" t="inlineStr">
         <is>
-          <t>1) 根據料況及排程,已安排8/19 DVT上線SMT,打板後不測試立即入庫調撥,Target 8/24 for台北RD測試開機.</t>
+          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
         </is>
       </c>
       <c r="P53" s="11" t="inlineStr">
@@ -4699,12 +4697,12 @@
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Raider 18 Max HX B4WI</t>
+          <t>Raider 18 Max HX B4WH</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>DVT</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
@@ -4714,7 +4712,7 @@
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>RTX 5080</t>
+          <t>RTX 5070Ti</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
@@ -4759,7 +4757,7 @@
       </c>
       <c r="O54" s="11" t="inlineStr">
         <is>
-          <t>1) 根據料況及排程,已安排8/19 DVT上線SMT,打板後不測試立即入庫調撥,Target 8/24 for台北RD測試開機.</t>
+          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
         </is>
       </c>
       <c r="P54" s="11" t="inlineStr">
@@ -4779,230 +4777,230 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
+          <t>Raider 18 Max HX B4WI</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 65W</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5080</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>高宇奇</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>2026/06/29</t>
+        </is>
+      </c>
+      <c r="I55" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/19</t>
+        </is>
+      </c>
+      <c r="J55" s="9" t="inlineStr">
+        <is>
+          <t>2026/10/23</t>
+        </is>
+      </c>
+      <c r="K55" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/08</t>
+        </is>
+      </c>
+      <c r="L55" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/01</t>
+        </is>
+      </c>
+      <c r="M55" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N55" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O55" s="11" t="inlineStr">
+        <is>
+          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
+        </is>
+      </c>
+      <c r="P55" s="11" t="inlineStr">
+        <is>
+          <t>1) 根據SSE POC會議討論共識,1851最後採用2顆MCU架構for所有的發光device,並且根據SSE提出的建議,第1顆MCU控制Per key KB,另1顆MCU控制其餘所有發光device,預計9月初提供1台1851 mockup系統for SSE FW implement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" hidden="1" outlineLevel="1">
+      <c r="A56" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>1851</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
           <t>Raider 18 Max HX B4WJ</t>
         </is>
       </c>
-      <c r="D55" s="16" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E55" s="9" t="inlineStr">
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
         <is>
           <t>NVL-HX 65W</t>
         </is>
       </c>
-      <c r="F55" s="9" t="inlineStr">
+      <c r="F56" s="9" t="inlineStr">
         <is>
           <t>RTX 5090</t>
         </is>
       </c>
-      <c r="G55" s="9" t="inlineStr">
+      <c r="G56" s="9" t="inlineStr">
         <is>
           <t>高宇奇</t>
         </is>
       </c>
-      <c r="H55" s="9" t="inlineStr">
+      <c r="H56" s="9" t="inlineStr">
         <is>
           <t>2026/06/29</t>
         </is>
       </c>
-      <c r="I55" s="9" t="inlineStr">
+      <c r="I56" s="9" t="inlineStr">
         <is>
           <t>2026/08/19</t>
         </is>
       </c>
-      <c r="J55" s="9" t="inlineStr">
+      <c r="J56" s="9" t="inlineStr">
         <is>
           <t>2026/10/23</t>
         </is>
       </c>
-      <c r="K55" s="9" t="inlineStr">
+      <c r="K56" s="9" t="inlineStr">
         <is>
           <t>2027/01/08</t>
         </is>
       </c>
-      <c r="L55" s="9" t="inlineStr">
+      <c r="L56" s="9" t="inlineStr">
         <is>
           <t>2027/02/01</t>
         </is>
       </c>
-      <c r="M55" s="9" t="inlineStr">
+      <c r="M56" s="9" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N55" s="9" t="inlineStr">
+      <c r="N56" s="9" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O55" s="11" t="inlineStr">
-        <is>
-          <t>1) 根據料況及排程,已安排8/19 DVT上線SMT,打板後不測試立即入庫調撥,Target 8/24 for台北RD測試開機.</t>
-        </is>
-      </c>
-      <c r="P55" s="11" t="inlineStr">
+      <c r="O56" s="11" t="inlineStr">
+        <is>
+          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
+        </is>
+      </c>
+      <c r="P56" s="11" t="inlineStr">
         <is>
           <t>1) 根據SSE POC會議討論共識,1851最後採用2顆MCU架構for所有的發光device,並且根據SSE提出的建議,第1顆MCU控制Per key KB,另1顆MCU控制其餘所有發光device,預計9月初提供1台1851 mockup系統for SSE FW implement.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>2655</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>Crosshair 16 Max HX E4WEK</t>
         </is>
       </c>
-      <c r="D56" s="17" t="inlineStr">
+      <c r="D57" s="18" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="E57" s="4" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>RTX 5050</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>鮑佩佩</t>
         </is>
       </c>
-      <c r="H56" s="4" t="inlineStr">
+      <c r="H57" s="4" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I56" s="4" t="inlineStr">
+      <c r="I57" s="4" t="inlineStr">
         <is>
           <t>2026/08/06</t>
         </is>
       </c>
-      <c r="J56" s="4" t="inlineStr">
+      <c r="J57" s="4" t="inlineStr">
         <is>
           <t>2026/09/29</t>
         </is>
       </c>
-      <c r="K56" s="4" t="inlineStr">
+      <c r="K57" s="4" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L56" s="4" t="inlineStr">
+      <c r="L57" s="4" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M56" s="4" t="inlineStr">
+      <c r="M57" s="4" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N56" s="4" t="inlineStr">
+      <c r="N57" s="4" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O56" s="6" t="inlineStr">
+      <c r="O57" s="6" t="inlineStr">
         <is>
           <t>DVT 測試中</t>
         </is>
       </c>
-      <c r="P56" s="6" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" hidden="1" outlineLevel="1">
-      <c r="A57" s="7" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>2655</t>
-        </is>
-      </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>Crosshair 16 Max HX E4WFK</t>
-        </is>
-      </c>
-      <c r="D57" s="15" t="inlineStr">
-        <is>
-          <t>DVT</t>
-        </is>
-      </c>
-      <c r="E57" s="9" t="inlineStr">
-        <is>
-          <t>NVL-HX 55W</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="inlineStr">
-        <is>
-          <t>RTX 5060</t>
-        </is>
-      </c>
-      <c r="G57" s="9" t="inlineStr">
-        <is>
-          <t>鮑佩佩</t>
-        </is>
-      </c>
-      <c r="H57" s="9" t="inlineStr">
-        <is>
-          <t>2026/05/19</t>
-        </is>
-      </c>
-      <c r="I57" s="9" t="inlineStr">
-        <is>
-          <t>2026/08/06</t>
-        </is>
-      </c>
-      <c r="J57" s="9" t="inlineStr">
-        <is>
-          <t>2026/09/29</t>
-        </is>
-      </c>
-      <c r="K57" s="9" t="inlineStr">
-        <is>
-          <t>2027/01/11</t>
-        </is>
-      </c>
-      <c r="L57" s="9" t="inlineStr">
-        <is>
-          <t>2027/02/02</t>
-        </is>
-      </c>
-      <c r="M57" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/08</t>
-        </is>
-      </c>
-      <c r="N57" s="9" t="inlineStr">
-        <is>
-          <t>2027/03/18</t>
-        </is>
-      </c>
-      <c r="O57" s="11" t="inlineStr">
-        <is>
-          <t>DVT 測試中</t>
-        </is>
-      </c>
-      <c r="P57" s="11" t="inlineStr">
+      <c r="P57" s="6" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -5019,10 +5017,10 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Crosshair 16 Max HX E4WGK</t>
-        </is>
-      </c>
-      <c r="D58" s="15" t="inlineStr">
+          <t>Crosshair 16 Max HX E4WFK</t>
+        </is>
+      </c>
+      <c r="D58" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
@@ -5034,7 +5032,7 @@
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>RTX 5070</t>
+          <t>RTX 5060</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
@@ -5099,77 +5097,157 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
+          <t>Crosshair 16 Max HX E4WGK</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>DVT</t>
+        </is>
+      </c>
+      <c r="E59" s="9" t="inlineStr">
+        <is>
+          <t>NVL-HX 55W</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="inlineStr">
+        <is>
+          <t>RTX 5070</t>
+        </is>
+      </c>
+      <c r="G59" s="9" t="inlineStr">
+        <is>
+          <t>鮑佩佩</t>
+        </is>
+      </c>
+      <c r="H59" s="9" t="inlineStr">
+        <is>
+          <t>2026/05/19</t>
+        </is>
+      </c>
+      <c r="I59" s="9" t="inlineStr">
+        <is>
+          <t>2026/08/06</t>
+        </is>
+      </c>
+      <c r="J59" s="9" t="inlineStr">
+        <is>
+          <t>2026/09/29</t>
+        </is>
+      </c>
+      <c r="K59" s="9" t="inlineStr">
+        <is>
+          <t>2027/01/11</t>
+        </is>
+      </c>
+      <c r="L59" s="9" t="inlineStr">
+        <is>
+          <t>2027/02/02</t>
+        </is>
+      </c>
+      <c r="M59" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/08</t>
+        </is>
+      </c>
+      <c r="N59" s="9" t="inlineStr">
+        <is>
+          <t>2027/03/18</t>
+        </is>
+      </c>
+      <c r="O59" s="11" t="inlineStr">
+        <is>
+          <t>DVT 測試中</t>
+        </is>
+      </c>
+      <c r="P59" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" hidden="1" outlineLevel="1">
+      <c r="A60" s="7" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>2655</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
           <t>Crosshair 16 Max HX E4WGXK</t>
         </is>
       </c>
-      <c r="D59" s="15" t="inlineStr">
+      <c r="D60" s="16" t="inlineStr">
         <is>
           <t>DVT</t>
         </is>
       </c>
-      <c r="E59" s="9" t="inlineStr">
+      <c r="E60" s="9" t="inlineStr">
         <is>
           <t>NVL-HX 55W</t>
         </is>
       </c>
-      <c r="F59" s="9" t="inlineStr">
+      <c r="F60" s="9" t="inlineStr">
         <is>
           <t>RTX 5070</t>
         </is>
       </c>
-      <c r="G59" s="9" t="inlineStr">
+      <c r="G60" s="9" t="inlineStr">
         <is>
           <t>鮑佩佩</t>
         </is>
       </c>
-      <c r="H59" s="9" t="inlineStr">
+      <c r="H60" s="9" t="inlineStr">
         <is>
           <t>2026/05/19</t>
         </is>
       </c>
-      <c r="I59" s="9" t="inlineStr">
+      <c r="I60" s="9" t="inlineStr">
         <is>
           <t>2026/08/06</t>
         </is>
       </c>
-      <c r="J59" s="9" t="inlineStr">
+      <c r="J60" s="9" t="inlineStr">
         <is>
           <t>2026/09/29</t>
         </is>
       </c>
-      <c r="K59" s="9" t="inlineStr">
+      <c r="K60" s="9" t="inlineStr">
         <is>
           <t>2027/01/11</t>
         </is>
       </c>
-      <c r="L59" s="9" t="inlineStr">
+      <c r="L60" s="9" t="inlineStr">
         <is>
           <t>2027/02/02</t>
         </is>
       </c>
-      <c r="M59" s="9" t="inlineStr">
+      <c r="M60" s="9" t="inlineStr">
         <is>
           <t>2027/03/08</t>
         </is>
       </c>
-      <c r="N59" s="9" t="inlineStr">
+      <c r="N60" s="9" t="inlineStr">
         <is>
           <t>2027/03/18</t>
         </is>
       </c>
-      <c r="O59" s="11" t="inlineStr">
+      <c r="O60" s="11" t="inlineStr">
         <is>
           <t>DVT 測試中</t>
         </is>
       </c>
-      <c r="P59" s="11" t="inlineStr">
+      <c r="P60" s="11" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P59"/>
+  <autoFilter ref="A1:P60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update NPI Dashboard 2026-09-04 16:21
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -847,16 +847,16 @@
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
-          <t>HPT:MVT進行中, APU R7 155 ETD@9/21, 暫定9/24進行C/R@26PN081119C*50</t>
+          <t>HPT:MVT進行中, 預計9/11 ATS@26PN083486A*100</t>
         </is>
       </c>
       <c r="P4" s="6" t="inlineStr">
         <is>
-          <t>1).8/31 業務通知決定收斂到Max, non Max 還有最後2.9K 套料, 接完就收斂.現在開始的新報價往Max
+          <t>1).9/3 業務通知:R7 155 報價單會改回在non-Max sku,優先消化non-Max thermal庫存
 2).Schedule:AMD PI 1200I NDA Release delay(6/19→7/
-28)與生管延後MVT SMT 排程(8/4→8/
-7),累計delay 42天,取消 DVT排程改以 APU Rework 驗證追趕時程後,MP還是會delay 22天至9/22(先前已由 9 /17提前至 8/31,現又延至9/
-22),後續將依實際測試結果滾動式調整專案時程</t>
+28)與生管延後MVT SMT (8/4→8/
+7),累計delay 42天,取消 DVT排程改以 APU Rework 驗證追趕進度後,MP還是會delay 22天至9/22(先前已由 9 /17提前至 8/31,現又延至9/
+22)</t>
         </is>
       </c>
     </row>
@@ -927,16 +927,16 @@
       </c>
       <c r="O5" s="12" t="inlineStr">
         <is>
-          <t>HPT:MVT進行中, 預計9/11 ATS@26PN083486A*100</t>
+          <t>HPT:MVT進行中, APU R7 155 ETD@9/21, 暫定9/24進行C/R@26PN081119C*50</t>
         </is>
       </c>
       <c r="P5" s="12" t="inlineStr">
         <is>
-          <t>1).8/31 業務通知決定收斂到Max, non Max 還有最後2.9K 套料, 接完就收斂.現在開始的新報價往Max
+          <t>1).9/3 業務通知:R7 155 報價單會改回在non-Max sku,優先消化non-Max thermal庫存
 2).Schedule:AMD PI 1200I NDA Release delay(6/19→7/
-28)與生管延後MVT SMT 排程(8/4→8/
-7),累計delay 42天,取消 DVT排程改以 APU Rework 驗證追趕時程後,MP還是會delay 22天至9/22(先前已由 9 /17提前至 8/31,現又延至9/
-22),後續將依實際測試結果滾動式調整專案時程</t>
+28)與生管延後MVT SMT (8/4→8/
+7),累計delay 42天,取消 DVT排程改以 APU Rework 驗證追趕進度後,MP還是會delay 22天至9/22(先前已由 9 /17提前至 8/31,現又延至9/
+22)</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1)備料: 業務尚未提供1st lot需求, 塑膠顆粒先按MOQ備料</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1)備料: 業務尚未提供1st lot需求, 塑膠顆粒先按MOQ備料</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1)備料: 業務尚未提供1st lot需求, 塑膠顆粒先按MOQ備料</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="P12" s="12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1)備料: 業務尚未提供1st lot需求, 塑膠顆粒先按MOQ備料</t>
         </is>
       </c>
     </row>
@@ -3828,12 +3828,12 @@
       </c>
       <c r="O42" s="6" t="inlineStr">
         <is>
-          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
+          <t>DVT板子測試中</t>
         </is>
       </c>
       <c r="P42" s="6" t="inlineStr">
         <is>
-          <t>1) 根據SSE POC會議討論共識,1851最後採用2顆MCU架構for所有的發光device,並且根據SSE提出的建議,第1顆MCU控制Per key KB,另1顆MCU控制其餘所有發光device,預計9月初提供1台1851 mockup系統for SSE FW implement.</t>
+          <t>1851目前上4支memory才能開機,RD正在跟Intel debug/study此問題.</t>
         </is>
       </c>
     </row>
@@ -3908,12 +3908,12 @@
       </c>
       <c r="O43" s="12" t="inlineStr">
         <is>
-          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
+          <t>DVT板子測試中</t>
         </is>
       </c>
       <c r="P43" s="12" t="inlineStr">
         <is>
-          <t>1) 根據SSE POC會議討論共識,1851最後採用2顆MCU架構for所有的發光device,並且根據SSE提出的建議,第1顆MCU控制Per key KB,另1顆MCU控制其餘所有發光device,預計9月初提供1台1851 mockup系統for SSE FW implement.</t>
+          <t>1851目前上4支memory才能開機,RD正在跟Intel debug/study此問題.</t>
         </is>
       </c>
     </row>
@@ -3988,12 +3988,12 @@
       </c>
       <c r="O44" s="12" t="inlineStr">
         <is>
-          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
+          <t>DVT板子測試中</t>
         </is>
       </c>
       <c r="P44" s="12" t="inlineStr">
         <is>
-          <t>1) 根據SSE POC會議討論共識,1851最後採用2顆MCU架構for所有的發光device,並且根據SSE提出的建議,第1顆MCU控制Per key KB,另1顆MCU控制其餘所有發光device,預計9月初提供1台1851 mockup系統for SSE FW implement.</t>
+          <t>1851目前上4支memory才能開機,RD正在跟Intel debug/study此問題.</t>
         </is>
       </c>
     </row>
@@ -4068,12 +4068,12 @@
       </c>
       <c r="O45" s="12" t="inlineStr">
         <is>
-          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
+          <t>DVT板子測試中</t>
         </is>
       </c>
       <c r="P45" s="12" t="inlineStr">
         <is>
-          <t>1) 根據SSE POC會議討論共識,1851最後採用2顆MCU架構for所有的發光device,並且根據SSE提出的建議,第1顆MCU控制Per key KB,另1顆MCU控制其餘所有發光device,預計9月初提供1台1851 mockup系統for SSE FW implement.</t>
+          <t>1851目前上4支memory才能開機,RD正在跟Intel debug/study此問題.</t>
         </is>
       </c>
     </row>
@@ -4148,12 +4148,12 @@
       </c>
       <c r="O46" s="12" t="inlineStr">
         <is>
-          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
+          <t>DVT板子測試中</t>
         </is>
       </c>
       <c r="P46" s="12" t="inlineStr">
         <is>
-          <t>1) 根據SSE POC會議討論共識,1851最後採用2顆MCU架構for所有的發光device,並且根據SSE提出的建議,第1顆MCU控制Per key KB,另1顆MCU控制其餘所有發光device,預計9月初提供1台1851 mockup系統for SSE FW implement.</t>
+          <t>1851目前上4支memory才能開機,RD正在跟Intel debug/study此問題.</t>
         </is>
       </c>
     </row>
@@ -4228,12 +4228,12 @@
       </c>
       <c r="O47" s="12" t="inlineStr">
         <is>
-          <t>1) DVT板子已於8/24到台北,目前板子已開機並分發給各team member開始進行測試.</t>
+          <t>DVT板子測試中</t>
         </is>
       </c>
       <c r="P47" s="12" t="inlineStr">
         <is>
-          <t>1) 根據SSE POC會議討論共識,1851最後採用2顆MCU架構for所有的發光device,並且根據SSE提出的建議,第1顆MCU控制Per key KB,另1顆MCU控制其餘所有發光device,預計9月初提供1台1851 mockup系統for SSE FW implement.</t>
+          <t>1851目前上4支memory才能開機,RD正在跟Intel debug/study此問題.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NPI Dashboard 2026-09-07 14:30
</commit_message>
<xml_diff>
--- a/npi_dashboard.xlsx
+++ b/npi_dashboard.xlsx
@@ -847,7 +847,7 @@
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
-          <t>HPT:MVT進行中, 預計9/11 ATS@26PN083486A*100</t>
+          <t>HPT: 預計9/11 ATS@26PN083486A*100</t>
         </is>
       </c>
       <c r="P4" s="6" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="O5" s="12" t="inlineStr">
         <is>
-          <t>HPT:MVT進行中, APU R7 155 ETD@9/21, 暫定9/24進行C/R@26PN081119C*50</t>
+          <t>HPT: APU R7 155 ETD@9/21, 暫定9/24進行C/R@26PN081119C*50</t>
         </is>
       </c>
       <c r="P5" s="12" t="inlineStr">

</xml_diff>